<commit_message>
add dc lines, transformers, and parallel processing
</commit_message>
<xml_diff>
--- a/test/inputs/case118/case118.xlsx
+++ b/test/inputs/case118/case118.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nomyk\Desktop\Network Reduction Model\NetworkReduction.jl\test\inputs\case118\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{529FD465-F4B0-4217-AB4C-5A3279106415}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D02B6407-E370-4E89-9E9F-B95C3D4D8089}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1015" uniqueCount="337">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1015" uniqueCount="338">
   <si>
     <t>Line_name</t>
   </si>
@@ -1050,6 +1050,9 @@
   </si>
   <si>
     <t>IsRepresentative</t>
+  </si>
+  <si>
+    <t>Z4</t>
   </si>
 </sst>
 </file>
@@ -1059,7 +1062,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1094,11 +1097,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
-      <name val="Segoe UI"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -1107,6 +1105,27 @@
     <font>
       <sz val="11"/>
       <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1194,12 +1213,13 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1"/>
@@ -1220,14 +1240,24 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="7" fillId="2" borderId="0" xfId="2" applyNumberFormat="1"/>
-    <xf numFmtId="2" fontId="7" fillId="2" borderId="4" xfId="2" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="6" fillId="2" borderId="0" xfId="2" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="6" fillId="2" borderId="4" xfId="2" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="3"/>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="4">
     <cellStyle name="Good" xfId="2" builtinId="26"/>
+    <cellStyle name="Hyperlink" xfId="3" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Standard 2" xfId="1" xr:uid="{4781E190-0CBC-4ACB-9E92-DBE0057C370D}"/>
   </cellStyles>
@@ -1567,7 +1597,7 @@
       <c r="D2" s="12" t="s">
         <v>276</v>
       </c>
-      <c r="E2" s="17">
+      <c r="E2" s="16">
         <v>138</v>
       </c>
       <c r="F2" s="10">
@@ -1599,7 +1629,7 @@
       <c r="D3" s="10" t="s">
         <v>277</v>
       </c>
-      <c r="E3" s="18">
+      <c r="E3" s="17">
         <v>138</v>
       </c>
       <c r="F3" s="10">
@@ -1631,7 +1661,7 @@
       <c r="D4" s="10" t="s">
         <v>279</v>
       </c>
-      <c r="E4" s="18">
+      <c r="E4" s="17">
         <v>138</v>
       </c>
       <c r="F4" s="10">
@@ -1663,7 +1693,7 @@
       <c r="D5" s="10" t="s">
         <v>279</v>
       </c>
-      <c r="E5" s="18">
+      <c r="E5" s="17">
         <v>138</v>
       </c>
       <c r="F5" s="10">
@@ -1695,7 +1725,7 @@
       <c r="D6" s="10" t="s">
         <v>280</v>
       </c>
-      <c r="E6" s="18">
+      <c r="E6" s="17">
         <v>138</v>
       </c>
       <c r="F6" s="10">
@@ -1727,7 +1757,7 @@
       <c r="D7" s="10" t="s">
         <v>281</v>
       </c>
-      <c r="E7" s="18">
+      <c r="E7" s="17">
         <v>138</v>
       </c>
       <c r="F7" s="10">
@@ -1759,7 +1789,7 @@
       <c r="D8" s="10" t="s">
         <v>283</v>
       </c>
-      <c r="E8" s="18">
+      <c r="E8" s="17">
         <v>345</v>
       </c>
       <c r="F8" s="10">
@@ -1791,19 +1821,19 @@
       <c r="D9" s="10" t="s">
         <v>279</v>
       </c>
-      <c r="E9" s="18">
+      <c r="E9" s="17">
         <v>345</v>
       </c>
       <c r="F9" s="10">
         <v>1506.1311370164149</v>
       </c>
-      <c r="G9" s="19">
+      <c r="G9" s="18">
         <v>0</v>
       </c>
       <c r="H9" s="13">
         <v>31.779675000000001</v>
       </c>
-      <c r="I9" s="20">
+      <c r="I9" s="19">
         <v>0</v>
       </c>
       <c r="J9" s="13">
@@ -1823,7 +1853,7 @@
       <c r="D10" s="10" t="s">
         <v>284</v>
       </c>
-      <c r="E10" s="18">
+      <c r="E10" s="17">
         <v>345</v>
       </c>
       <c r="F10" s="10">
@@ -1855,7 +1885,7 @@
       <c r="D11" s="10" t="s">
         <v>285</v>
       </c>
-      <c r="E11" s="18">
+      <c r="E11" s="17">
         <v>138</v>
       </c>
       <c r="F11" s="10">
@@ -1887,7 +1917,7 @@
       <c r="D12" s="10" t="s">
         <v>285</v>
       </c>
-      <c r="E12" s="18">
+      <c r="E12" s="17">
         <v>138</v>
       </c>
       <c r="F12" s="10">
@@ -1919,7 +1949,7 @@
       <c r="D13" s="10" t="s">
         <v>272</v>
       </c>
-      <c r="E13" s="18">
+      <c r="E13" s="17">
         <v>138</v>
       </c>
       <c r="F13" s="10">
@@ -1951,7 +1981,7 @@
       <c r="D14" s="10" t="s">
         <v>272</v>
       </c>
-      <c r="E14" s="18">
+      <c r="E14" s="17">
         <v>138</v>
       </c>
       <c r="F14" s="10">
@@ -1983,7 +2013,7 @@
       <c r="D15" s="10" t="s">
         <v>272</v>
       </c>
-      <c r="E15" s="18">
+      <c r="E15" s="17">
         <v>138</v>
       </c>
       <c r="F15" s="10">
@@ -2015,7 +2045,7 @@
       <c r="D16" s="10" t="s">
         <v>272</v>
       </c>
-      <c r="E16" s="18">
+      <c r="E16" s="17">
         <v>138</v>
       </c>
       <c r="F16" s="10">
@@ -2047,7 +2077,7 @@
       <c r="D17" s="10" t="s">
         <v>286</v>
       </c>
-      <c r="E17" s="18">
+      <c r="E17" s="17">
         <v>138</v>
       </c>
       <c r="F17" s="10">
@@ -2079,7 +2109,7 @@
       <c r="D18" s="10" t="s">
         <v>287</v>
       </c>
-      <c r="E18" s="18">
+      <c r="E18" s="17">
         <v>138</v>
       </c>
       <c r="F18" s="10">
@@ -2111,7 +2141,7 @@
       <c r="D19" s="10" t="s">
         <v>288</v>
       </c>
-      <c r="E19" s="18">
+      <c r="E19" s="17">
         <v>138</v>
       </c>
       <c r="F19" s="10">
@@ -2143,7 +2173,7 @@
       <c r="D20" s="10" t="s">
         <v>288</v>
       </c>
-      <c r="E20" s="18">
+      <c r="E20" s="17">
         <v>138</v>
       </c>
       <c r="F20" s="10">
@@ -2175,7 +2205,7 @@
       <c r="D21" s="10" t="s">
         <v>289</v>
       </c>
-      <c r="E21" s="18">
+      <c r="E21" s="17">
         <v>138</v>
       </c>
       <c r="F21" s="10">
@@ -2207,7 +2237,7 @@
       <c r="D22" s="10" t="s">
         <v>265</v>
       </c>
-      <c r="E22" s="18">
+      <c r="E22" s="17">
         <v>138</v>
       </c>
       <c r="F22" s="10">
@@ -2239,7 +2269,7 @@
       <c r="D23" s="10" t="s">
         <v>265</v>
       </c>
-      <c r="E23" s="18">
+      <c r="E23" s="17">
         <v>138</v>
       </c>
       <c r="F23" s="10">
@@ -2271,7 +2301,7 @@
       <c r="D24" s="10" t="s">
         <v>290</v>
       </c>
-      <c r="E24" s="18">
+      <c r="E24" s="17">
         <v>138</v>
       </c>
       <c r="F24" s="10">
@@ -2303,7 +2333,7 @@
       <c r="D25" s="10" t="s">
         <v>291</v>
       </c>
-      <c r="E25" s="18">
+      <c r="E25" s="17">
         <v>138</v>
       </c>
       <c r="F25" s="10">
@@ -2335,7 +2365,7 @@
       <c r="D26" s="10" t="s">
         <v>292</v>
       </c>
-      <c r="E26" s="18">
+      <c r="E26" s="17">
         <v>138</v>
       </c>
       <c r="F26" s="10">
@@ -2367,7 +2397,7 @@
       <c r="D27" s="10" t="s">
         <v>291</v>
       </c>
-      <c r="E27" s="18">
+      <c r="E27" s="17">
         <v>138</v>
       </c>
       <c r="F27" s="10">
@@ -2399,7 +2429,7 @@
       <c r="D28" s="10" t="s">
         <v>293</v>
       </c>
-      <c r="E28" s="18">
+      <c r="E28" s="17">
         <v>138</v>
       </c>
       <c r="F28" s="10">
@@ -2431,7 +2461,7 @@
       <c r="D29" s="10" t="s">
         <v>294</v>
       </c>
-      <c r="E29" s="18">
+      <c r="E29" s="17">
         <v>138</v>
       </c>
       <c r="F29" s="10">
@@ -2463,7 +2493,7 @@
       <c r="D30" s="10" t="s">
         <v>295</v>
       </c>
-      <c r="E30" s="18">
+      <c r="E30" s="17">
         <v>138</v>
       </c>
       <c r="F30" s="10">
@@ -2495,7 +2525,7 @@
       <c r="D31" s="10" t="s">
         <v>222</v>
       </c>
-      <c r="E31" s="18">
+      <c r="E31" s="17">
         <v>138</v>
       </c>
       <c r="F31" s="10">
@@ -2527,7 +2557,7 @@
       <c r="D32" s="10" t="s">
         <v>296</v>
       </c>
-      <c r="E32" s="18">
+      <c r="E32" s="17">
         <v>138</v>
       </c>
       <c r="F32" s="10">
@@ -2559,19 +2589,19 @@
       <c r="D33" s="10" t="s">
         <v>296</v>
       </c>
-      <c r="E33" s="18">
+      <c r="E33" s="17">
         <v>345</v>
       </c>
       <c r="F33" s="10">
         <v>920.41347262114243</v>
       </c>
-      <c r="G33" s="19">
+      <c r="G33" s="18">
         <v>0</v>
       </c>
       <c r="H33" s="13">
         <v>45.467550000000003</v>
       </c>
-      <c r="I33" s="20">
+      <c r="I33" s="19">
         <v>0</v>
       </c>
       <c r="J33" s="13">
@@ -2591,7 +2621,7 @@
       <c r="D34" s="10" t="s">
         <v>269</v>
       </c>
-      <c r="E34" s="18">
+      <c r="E34" s="17">
         <v>138</v>
       </c>
       <c r="F34" s="10">
@@ -2623,7 +2653,7 @@
       <c r="D35" s="10" t="s">
         <v>298</v>
       </c>
-      <c r="E35" s="18">
+      <c r="E35" s="17">
         <v>138</v>
       </c>
       <c r="F35" s="10">
@@ -2655,7 +2685,7 @@
       <c r="D36" s="10" t="s">
         <v>299</v>
       </c>
-      <c r="E36" s="18">
+      <c r="E36" s="17">
         <v>138</v>
       </c>
       <c r="F36" s="10">
@@ -2687,19 +2717,19 @@
       <c r="D37" s="10" t="s">
         <v>265</v>
       </c>
-      <c r="E37" s="18">
+      <c r="E37" s="17">
         <v>345</v>
       </c>
       <c r="F37" s="10">
         <v>920.41347262114243</v>
       </c>
-      <c r="G37" s="19">
+      <c r="G37" s="18">
         <v>0</v>
       </c>
       <c r="H37" s="13">
         <v>46.181699999999999</v>
       </c>
-      <c r="I37" s="20">
+      <c r="I37" s="19">
         <v>0</v>
       </c>
       <c r="J37" s="13">
@@ -2719,7 +2749,7 @@
       <c r="D38" s="10" t="s">
         <v>300</v>
       </c>
-      <c r="E38" s="18">
+      <c r="E38" s="17">
         <v>345</v>
       </c>
       <c r="F38" s="10">
@@ -2751,7 +2781,7 @@
       <c r="D39" s="10" t="s">
         <v>300</v>
       </c>
-      <c r="E39" s="18">
+      <c r="E39" s="17">
         <v>345</v>
       </c>
       <c r="F39" s="10">
@@ -2783,7 +2813,7 @@
       <c r="D40" s="10" t="s">
         <v>301</v>
       </c>
-      <c r="E40" s="18">
+      <c r="E40" s="17">
         <v>138</v>
       </c>
       <c r="F40" s="10">
@@ -2815,7 +2845,7 @@
       <c r="D41" s="10" t="s">
         <v>301</v>
       </c>
-      <c r="E41" s="18">
+      <c r="E41" s="17">
         <v>138</v>
       </c>
       <c r="F41" s="10">
@@ -2847,7 +2877,7 @@
       <c r="D42" s="10" t="s">
         <v>267</v>
       </c>
-      <c r="E42" s="18">
+      <c r="E42" s="17">
         <v>138</v>
       </c>
       <c r="F42" s="10">
@@ -2879,7 +2909,7 @@
       <c r="D43" s="10" t="s">
         <v>267</v>
       </c>
-      <c r="E43" s="18">
+      <c r="E43" s="17">
         <v>138</v>
       </c>
       <c r="F43" s="10">
@@ -2911,7 +2941,7 @@
       <c r="D44" s="10" t="s">
         <v>267</v>
       </c>
-      <c r="E44" s="18">
+      <c r="E44" s="17">
         <v>138</v>
       </c>
       <c r="F44" s="10">
@@ -2943,7 +2973,7 @@
       <c r="D45" s="10" t="s">
         <v>302</v>
       </c>
-      <c r="E45" s="18">
+      <c r="E45" s="17">
         <v>138</v>
       </c>
       <c r="F45" s="10">
@@ -2975,7 +3005,7 @@
       <c r="D46" s="10" t="s">
         <v>303</v>
       </c>
-      <c r="E46" s="18">
+      <c r="E46" s="17">
         <v>138</v>
       </c>
       <c r="F46" s="10">
@@ -3007,7 +3037,7 @@
       <c r="D47" s="10" t="s">
         <v>305</v>
       </c>
-      <c r="E47" s="18">
+      <c r="E47" s="17">
         <v>138</v>
       </c>
       <c r="F47" s="10">
@@ -3039,7 +3069,7 @@
       <c r="D48" s="10" t="s">
         <v>306</v>
       </c>
-      <c r="E48" s="18">
+      <c r="E48" s="17">
         <v>138</v>
       </c>
       <c r="F48" s="10">
@@ -3071,7 +3101,7 @@
       <c r="D49" s="10" t="s">
         <v>306</v>
       </c>
-      <c r="E49" s="18">
+      <c r="E49" s="17">
         <v>138</v>
       </c>
       <c r="F49" s="10">
@@ -3103,7 +3133,7 @@
       <c r="D50" s="10" t="s">
         <v>305</v>
       </c>
-      <c r="E50" s="18">
+      <c r="E50" s="17">
         <v>138</v>
       </c>
       <c r="F50" s="10">
@@ -3135,7 +3165,7 @@
       <c r="D51" s="10" t="s">
         <v>306</v>
       </c>
-      <c r="E51" s="18">
+      <c r="E51" s="17">
         <v>138</v>
       </c>
       <c r="F51" s="10">
@@ -3167,19 +3197,19 @@
       <c r="D52" s="10" t="s">
         <v>306</v>
       </c>
-      <c r="E52" s="18">
+      <c r="E52" s="17">
         <v>345</v>
       </c>
       <c r="F52" s="10">
         <v>920.41347262114243</v>
       </c>
-      <c r="G52" s="19">
+      <c r="G52" s="18">
         <v>0</v>
       </c>
       <c r="H52" s="13">
         <v>44.634374999999999</v>
       </c>
-      <c r="I52" s="20">
+      <c r="I52" s="19">
         <v>0</v>
       </c>
       <c r="J52" s="13">
@@ -3199,7 +3229,7 @@
       <c r="D53" s="10" t="s">
         <v>308</v>
       </c>
-      <c r="E53" s="18">
+      <c r="E53" s="17">
         <v>138</v>
       </c>
       <c r="F53" s="10">
@@ -3231,7 +3261,7 @@
       <c r="D54" s="10" t="s">
         <v>309</v>
       </c>
-      <c r="E54" s="18">
+      <c r="E54" s="17">
         <v>138</v>
       </c>
       <c r="F54" s="10">
@@ -3263,7 +3293,7 @@
       <c r="D55" s="10" t="s">
         <v>307</v>
       </c>
-      <c r="E55" s="18">
+      <c r="E55" s="17">
         <v>345</v>
       </c>
       <c r="F55" s="10">
@@ -3295,7 +3325,7 @@
       <c r="D56" s="10" t="s">
         <v>309</v>
       </c>
-      <c r="E56" s="18">
+      <c r="E56" s="17">
         <v>138</v>
       </c>
       <c r="F56" s="10">
@@ -3327,7 +3357,7 @@
       <c r="D57" s="10" t="s">
         <v>310</v>
       </c>
-      <c r="E57" s="18">
+      <c r="E57" s="17">
         <v>138</v>
       </c>
       <c r="F57" s="10">
@@ -3359,7 +3389,7 @@
       <c r="D58" s="10" t="s">
         <v>311</v>
       </c>
-      <c r="E58" s="18">
+      <c r="E58" s="17">
         <v>138</v>
       </c>
       <c r="F58" s="10">
@@ -3391,7 +3421,7 @@
       <c r="D59" s="10" t="s">
         <v>311</v>
       </c>
-      <c r="E59" s="18">
+      <c r="E59" s="17">
         <v>138</v>
       </c>
       <c r="F59" s="10">
@@ -3423,7 +3453,7 @@
       <c r="D60" s="10" t="s">
         <v>313</v>
       </c>
-      <c r="E60" s="18">
+      <c r="E60" s="17">
         <v>138</v>
       </c>
       <c r="F60" s="10">
@@ -3455,7 +3485,7 @@
       <c r="D61" s="10" t="s">
         <v>312</v>
       </c>
-      <c r="E61" s="18">
+      <c r="E61" s="17">
         <v>138</v>
       </c>
       <c r="F61" s="10">
@@ -3487,7 +3517,7 @@
       <c r="D62" s="10" t="s">
         <v>314</v>
       </c>
-      <c r="E62" s="18">
+      <c r="E62" s="17">
         <v>138</v>
       </c>
       <c r="F62" s="10">
@@ -3519,7 +3549,7 @@
       <c r="D63" s="10" t="s">
         <v>315</v>
       </c>
-      <c r="E63" s="18">
+      <c r="E63" s="17">
         <v>138</v>
       </c>
       <c r="F63" s="10">
@@ -3551,7 +3581,7 @@
       <c r="D64" s="10" t="s">
         <v>218</v>
       </c>
-      <c r="E64" s="18">
+      <c r="E64" s="17">
         <v>138</v>
       </c>
       <c r="F64" s="10">
@@ -3583,7 +3613,7 @@
       <c r="D65" s="10" t="s">
         <v>316</v>
       </c>
-      <c r="E65" s="18">
+      <c r="E65" s="17">
         <v>138</v>
       </c>
       <c r="F65" s="10">
@@ -3615,7 +3645,7 @@
       <c r="D66" s="10" t="s">
         <v>220</v>
       </c>
-      <c r="E66" s="18">
+      <c r="E66" s="17">
         <v>138</v>
       </c>
       <c r="F66" s="10">
@@ -3647,7 +3677,7 @@
       <c r="D67" s="10" t="s">
         <v>220</v>
       </c>
-      <c r="E67" s="18">
+      <c r="E67" s="17">
         <v>138</v>
       </c>
       <c r="F67" s="10">
@@ -3679,7 +3709,7 @@
       <c r="D68" s="10" t="s">
         <v>220</v>
       </c>
-      <c r="E68" s="18">
+      <c r="E68" s="17">
         <v>138</v>
       </c>
       <c r="F68" s="10">
@@ -3711,7 +3741,7 @@
       <c r="D69" s="10" t="s">
         <v>220</v>
       </c>
-      <c r="E69" s="18">
+      <c r="E69" s="17">
         <v>138</v>
       </c>
       <c r="F69" s="10">
@@ -3743,7 +3773,7 @@
       <c r="D70" s="10" t="s">
         <v>220</v>
       </c>
-      <c r="E70" s="18">
+      <c r="E70" s="17">
         <v>138</v>
       </c>
       <c r="F70" s="10">
@@ -3775,7 +3805,7 @@
       <c r="D71" s="10" t="s">
         <v>317</v>
       </c>
-      <c r="E71" s="18">
+      <c r="E71" s="17">
         <v>138</v>
       </c>
       <c r="F71" s="10">
@@ -3807,7 +3837,7 @@
       <c r="D72" s="10" t="s">
         <v>318</v>
       </c>
-      <c r="E72" s="18">
+      <c r="E72" s="17">
         <v>138</v>
       </c>
       <c r="F72" s="10">
@@ -3839,7 +3869,7 @@
       <c r="D73" s="10" t="s">
         <v>319</v>
       </c>
-      <c r="E73" s="18">
+      <c r="E73" s="17">
         <v>138</v>
       </c>
       <c r="F73" s="10">
@@ -3871,7 +3901,7 @@
       <c r="D74" s="10" t="s">
         <v>320</v>
       </c>
-      <c r="E74" s="18">
+      <c r="E74" s="17">
         <v>138</v>
       </c>
       <c r="F74" s="10">
@@ -3903,7 +3933,7 @@
       <c r="D75" s="10" t="s">
         <v>321</v>
       </c>
-      <c r="E75" s="18">
+      <c r="E75" s="17">
         <v>138</v>
       </c>
       <c r="F75" s="10">
@@ -3935,7 +3965,7 @@
       <c r="D76" s="10" t="s">
         <v>321</v>
       </c>
-      <c r="E76" s="18">
+      <c r="E76" s="17">
         <v>138</v>
       </c>
       <c r="F76" s="10">
@@ -3967,7 +3997,7 @@
       <c r="D77" s="10" t="s">
         <v>321</v>
       </c>
-      <c r="E77" s="18">
+      <c r="E77" s="17">
         <v>138</v>
       </c>
       <c r="F77" s="10">
@@ -3999,7 +4029,7 @@
       <c r="D78" s="10" t="s">
         <v>322</v>
       </c>
-      <c r="E78" s="18">
+      <c r="E78" s="17">
         <v>138</v>
       </c>
       <c r="F78" s="10">
@@ -4031,7 +4061,7 @@
       <c r="D79" s="10" t="s">
         <v>323</v>
       </c>
-      <c r="E79" s="18">
+      <c r="E79" s="17">
         <v>138</v>
       </c>
       <c r="F79" s="10">
@@ -4063,7 +4093,7 @@
       <c r="D80" s="10" t="s">
         <v>323</v>
       </c>
-      <c r="E80" s="18">
+      <c r="E80" s="17">
         <v>138</v>
       </c>
       <c r="F80" s="10">
@@ -4095,7 +4125,7 @@
       <c r="D81" s="10" t="s">
         <v>324</v>
       </c>
-      <c r="E81" s="18">
+      <c r="E81" s="17">
         <v>138</v>
       </c>
       <c r="F81" s="10">
@@ -4127,7 +4157,7 @@
       <c r="D82" s="10" t="s">
         <v>324</v>
       </c>
-      <c r="E82" s="18">
+      <c r="E82" s="17">
         <v>138</v>
       </c>
       <c r="F82" s="10">
@@ -4159,7 +4189,7 @@
       <c r="D83" s="10" t="s">
         <v>325</v>
       </c>
-      <c r="E83" s="18">
+      <c r="E83" s="17">
         <v>138</v>
       </c>
       <c r="F83" s="10">
@@ -4191,7 +4221,7 @@
       <c r="D84" s="10" t="s">
         <v>325</v>
       </c>
-      <c r="E84" s="18">
+      <c r="E84" s="17">
         <v>138</v>
       </c>
       <c r="F84" s="10">
@@ -4223,7 +4253,7 @@
       <c r="D85" s="10" t="s">
         <v>326</v>
       </c>
-      <c r="E85" s="18">
+      <c r="E85" s="17">
         <v>138</v>
       </c>
       <c r="F85" s="10">
@@ -4255,7 +4285,7 @@
       <c r="D86" s="10" t="s">
         <v>326</v>
       </c>
-      <c r="E86" s="18">
+      <c r="E86" s="17">
         <v>138</v>
       </c>
       <c r="F86" s="10">
@@ -4287,7 +4317,7 @@
       <c r="D87" s="10" t="s">
         <v>326</v>
       </c>
-      <c r="E87" s="18">
+      <c r="E87" s="17">
         <v>138</v>
       </c>
       <c r="F87" s="10">
@@ -4319,7 +4349,7 @@
       <c r="D88" s="10" t="s">
         <v>326</v>
       </c>
-      <c r="E88" s="18">
+      <c r="E88" s="17">
         <v>138</v>
       </c>
       <c r="F88" s="10">
@@ -4351,7 +4381,7 @@
       <c r="D89" s="10" t="s">
         <v>327</v>
       </c>
-      <c r="E89" s="18">
+      <c r="E89" s="17">
         <v>138</v>
       </c>
       <c r="F89" s="10">
@@ -4383,7 +4413,7 @@
       <c r="D90" s="10" t="s">
         <v>328</v>
       </c>
-      <c r="E90" s="18">
+      <c r="E90" s="17">
         <v>138</v>
       </c>
       <c r="F90" s="10">
@@ -4415,7 +4445,7 @@
       <c r="D91" s="10" t="s">
         <v>328</v>
       </c>
-      <c r="E91" s="18">
+      <c r="E91" s="17">
         <v>138</v>
       </c>
       <c r="F91" s="10">
@@ -4447,7 +4477,7 @@
       <c r="D92" s="10" t="s">
         <v>213</v>
       </c>
-      <c r="E92" s="18">
+      <c r="E92" s="17">
         <v>138</v>
       </c>
       <c r="F92" s="10">
@@ -4479,7 +4509,7 @@
       <c r="D93" s="10" t="s">
         <v>213</v>
       </c>
-      <c r="E93" s="18">
+      <c r="E93" s="17">
         <v>138</v>
       </c>
       <c r="F93" s="10">
@@ -4511,19 +4541,19 @@
       <c r="D94" s="10" t="s">
         <v>326</v>
       </c>
-      <c r="E94" s="18">
+      <c r="E94" s="17">
         <v>345</v>
       </c>
       <c r="F94" s="10">
         <v>920.41347262114243</v>
       </c>
-      <c r="G94" s="19">
+      <c r="G94" s="18">
         <v>0</v>
       </c>
       <c r="H94" s="13">
         <v>45.943650000000005</v>
       </c>
-      <c r="I94" s="20">
+      <c r="I94" s="19">
         <v>0</v>
       </c>
       <c r="J94" s="13">
@@ -4543,7 +4573,7 @@
       <c r="D95" s="10" t="s">
         <v>330</v>
       </c>
-      <c r="E95" s="18">
+      <c r="E95" s="17">
         <v>345</v>
       </c>
       <c r="F95" s="10">
@@ -4575,19 +4605,19 @@
       <c r="D96" s="10" t="s">
         <v>328</v>
       </c>
-      <c r="E96" s="18">
+      <c r="E96" s="17">
         <v>345</v>
       </c>
       <c r="F96" s="10">
         <v>920.41347262114243</v>
       </c>
-      <c r="G96" s="19">
+      <c r="G96" s="18">
         <v>0</v>
       </c>
       <c r="H96" s="13">
         <v>31.898699999999998</v>
       </c>
-      <c r="I96" s="20">
+      <c r="I96" s="19">
         <v>0</v>
       </c>
       <c r="J96" s="13">
@@ -4607,7 +4637,7 @@
       <c r="D97" s="10" t="s">
         <v>216</v>
       </c>
-      <c r="E97" s="18">
+      <c r="E97" s="17">
         <v>345</v>
       </c>
       <c r="F97" s="10">
@@ -4639,7 +4669,7 @@
       <c r="D98" s="10" t="s">
         <v>216</v>
       </c>
-      <c r="E98" s="18">
+      <c r="E98" s="17">
         <v>345</v>
       </c>
       <c r="F98" s="10">
@@ -4671,7 +4701,7 @@
       <c r="D99" s="10" t="s">
         <v>214</v>
       </c>
-      <c r="E99" s="18">
+      <c r="E99" s="17">
         <v>138</v>
       </c>
       <c r="F99" s="10">
@@ -4703,7 +4733,7 @@
       <c r="D100" s="10" t="s">
         <v>214</v>
       </c>
-      <c r="E100" s="18">
+      <c r="E100" s="17">
         <v>138</v>
       </c>
       <c r="F100" s="10">
@@ -4735,7 +4765,7 @@
       <c r="D101" s="10" t="s">
         <v>214</v>
       </c>
-      <c r="E101" s="18">
+      <c r="E101" s="17">
         <v>138</v>
       </c>
       <c r="F101" s="10">
@@ -4767,7 +4797,7 @@
       <c r="D102" s="10" t="s">
         <v>215</v>
       </c>
-      <c r="E102" s="18">
+      <c r="E102" s="17">
         <v>138</v>
       </c>
       <c r="F102" s="10">
@@ -4799,19 +4829,19 @@
       <c r="D103" s="10" t="s">
         <v>214</v>
       </c>
-      <c r="E103" s="18">
+      <c r="E103" s="17">
         <v>345</v>
       </c>
       <c r="F103" s="10">
         <v>1506.1311370164149</v>
       </c>
-      <c r="G103" s="19">
+      <c r="G103" s="18">
         <v>0</v>
       </c>
       <c r="H103" s="13">
         <v>44.039250000000003</v>
       </c>
-      <c r="I103" s="20">
+      <c r="I103" s="19">
         <v>0</v>
       </c>
       <c r="J103" s="13">
@@ -4831,7 +4861,7 @@
       <c r="D104" s="10" t="s">
         <v>215</v>
       </c>
-      <c r="E104" s="18">
+      <c r="E104" s="17">
         <v>138</v>
       </c>
       <c r="F104" s="10">
@@ -4863,7 +4893,7 @@
       <c r="D105" s="10" t="s">
         <v>217</v>
       </c>
-      <c r="E105" s="18">
+      <c r="E105" s="17">
         <v>345</v>
       </c>
       <c r="F105" s="10">
@@ -4895,7 +4925,7 @@
       <c r="D106" s="10" t="s">
         <v>219</v>
       </c>
-      <c r="E106" s="18">
+      <c r="E106" s="17">
         <v>138</v>
       </c>
       <c r="F106" s="10">
@@ -4927,7 +4957,7 @@
       <c r="D107" s="10" t="s">
         <v>219</v>
       </c>
-      <c r="E107" s="18">
+      <c r="E107" s="17">
         <v>138</v>
       </c>
       <c r="F107" s="10">
@@ -4959,19 +4989,19 @@
       <c r="D108" s="10" t="s">
         <v>219</v>
       </c>
-      <c r="E108" s="18">
+      <c r="E108" s="17">
         <v>345</v>
       </c>
       <c r="F108" s="10">
         <v>1506.1311370164149</v>
       </c>
-      <c r="G108" s="19">
+      <c r="G108" s="18">
         <v>0</v>
       </c>
       <c r="H108" s="13">
         <v>44.039250000000003</v>
       </c>
-      <c r="I108" s="20">
+      <c r="I108" s="19">
         <v>0</v>
       </c>
       <c r="J108" s="13">
@@ -4991,7 +5021,7 @@
       <c r="D109" s="10" t="s">
         <v>221</v>
       </c>
-      <c r="E109" s="18">
+      <c r="E109" s="17">
         <v>138</v>
       </c>
       <c r="F109" s="10">
@@ -5023,7 +5053,7 @@
       <c r="D110" s="10" t="s">
         <v>221</v>
       </c>
-      <c r="E110" s="18">
+      <c r="E110" s="17">
         <v>138</v>
       </c>
       <c r="F110" s="10">
@@ -5055,7 +5085,7 @@
       <c r="D111" s="10" t="s">
         <v>223</v>
       </c>
-      <c r="E111" s="18">
+      <c r="E111" s="17">
         <v>138</v>
       </c>
       <c r="F111" s="10">
@@ -5087,7 +5117,7 @@
       <c r="D112" s="10" t="s">
         <v>224</v>
       </c>
-      <c r="E112" s="18">
+      <c r="E112" s="17">
         <v>138</v>
       </c>
       <c r="F112" s="10">
@@ -5119,7 +5149,7 @@
       <c r="D113" s="10" t="s">
         <v>224</v>
       </c>
-      <c r="E113" s="18">
+      <c r="E113" s="17">
         <v>138</v>
       </c>
       <c r="F113" s="10">
@@ -5151,7 +5181,7 @@
       <c r="D114" s="10" t="s">
         <v>225</v>
       </c>
-      <c r="E114" s="18">
+      <c r="E114" s="17">
         <v>138</v>
       </c>
       <c r="F114" s="10">
@@ -5183,7 +5213,7 @@
       <c r="D115" s="10" t="s">
         <v>226</v>
       </c>
-      <c r="E115" s="18">
+      <c r="E115" s="17">
         <v>138</v>
       </c>
       <c r="F115" s="10">
@@ -5215,7 +5245,7 @@
       <c r="D116" s="10" t="s">
         <v>227</v>
       </c>
-      <c r="E116" s="18">
+      <c r="E116" s="17">
         <v>138</v>
       </c>
       <c r="F116" s="10">
@@ -5247,7 +5277,7 @@
       <c r="D117" s="10" t="s">
         <v>227</v>
       </c>
-      <c r="E117" s="18">
+      <c r="E117" s="17">
         <v>138</v>
       </c>
       <c r="F117" s="10">
@@ -5279,7 +5309,7 @@
       <c r="D118" s="10" t="s">
         <v>227</v>
       </c>
-      <c r="E118" s="18">
+      <c r="E118" s="17">
         <v>138</v>
       </c>
       <c r="F118" s="10">
@@ -5311,7 +5341,7 @@
       <c r="D119" s="10" t="s">
         <v>229</v>
       </c>
-      <c r="E119" s="18">
+      <c r="E119" s="17">
         <v>138</v>
       </c>
       <c r="F119" s="10">
@@ -5343,7 +5373,7 @@
       <c r="D120" s="10" t="s">
         <v>229</v>
       </c>
-      <c r="E120" s="18">
+      <c r="E120" s="17">
         <v>138</v>
       </c>
       <c r="F120" s="10">
@@ -5375,7 +5405,7 @@
       <c r="D121" s="10" t="s">
         <v>229</v>
       </c>
-      <c r="E121" s="18">
+      <c r="E121" s="17">
         <v>138</v>
       </c>
       <c r="F121" s="10">
@@ -5407,7 +5437,7 @@
       <c r="D122" s="10" t="s">
         <v>230</v>
       </c>
-      <c r="E122" s="18">
+      <c r="E122" s="17">
         <v>138</v>
       </c>
       <c r="F122" s="10">
@@ -5439,7 +5469,7 @@
       <c r="D123" s="10" t="s">
         <v>231</v>
       </c>
-      <c r="E123" s="18">
+      <c r="E123" s="17">
         <v>138</v>
       </c>
       <c r="F123" s="10">
@@ -5471,7 +5501,7 @@
       <c r="D124" s="10" t="s">
         <v>232</v>
       </c>
-      <c r="E124" s="18">
+      <c r="E124" s="17">
         <v>138</v>
       </c>
       <c r="F124" s="10">
@@ -5503,7 +5533,7 @@
       <c r="D125" s="10" t="s">
         <v>232</v>
       </c>
-      <c r="E125" s="18">
+      <c r="E125" s="17">
         <v>138</v>
       </c>
       <c r="F125" s="10">
@@ -5535,7 +5565,7 @@
       <c r="D126" s="10" t="s">
         <v>232</v>
       </c>
-      <c r="E126" s="18">
+      <c r="E126" s="17">
         <v>138</v>
       </c>
       <c r="F126" s="10">
@@ -5567,7 +5597,7 @@
       <c r="D127" s="10" t="s">
         <v>233</v>
       </c>
-      <c r="E127" s="18">
+      <c r="E127" s="17">
         <v>345</v>
       </c>
       <c r="F127" s="10">
@@ -5599,19 +5629,19 @@
       <c r="D128" s="10" t="s">
         <v>232</v>
       </c>
-      <c r="E128" s="18">
+      <c r="E128" s="17">
         <v>345</v>
       </c>
       <c r="F128" s="10">
         <v>1506.1311370164149</v>
       </c>
-      <c r="G128" s="19">
+      <c r="G128" s="18">
         <v>0</v>
       </c>
       <c r="H128" s="13">
         <v>44.039250000000003</v>
       </c>
-      <c r="I128" s="20">
+      <c r="I128" s="19">
         <v>0</v>
       </c>
       <c r="J128" s="13">
@@ -5631,7 +5661,7 @@
       <c r="D129" s="10" t="s">
         <v>234</v>
       </c>
-      <c r="E129" s="18">
+      <c r="E129" s="17">
         <v>138</v>
       </c>
       <c r="F129" s="10">
@@ -5663,7 +5693,7 @@
       <c r="D130" s="10" t="s">
         <v>235</v>
       </c>
-      <c r="E130" s="18">
+      <c r="E130" s="17">
         <v>138</v>
       </c>
       <c r="F130" s="10">
@@ -5695,7 +5725,7 @@
       <c r="D131" s="10" t="s">
         <v>236</v>
       </c>
-      <c r="E131" s="18">
+      <c r="E131" s="17">
         <v>138</v>
       </c>
       <c r="F131" s="10">
@@ -5727,7 +5757,7 @@
       <c r="D132" s="10" t="s">
         <v>237</v>
       </c>
-      <c r="E132" s="18">
+      <c r="E132" s="17">
         <v>138</v>
       </c>
       <c r="F132" s="10">
@@ -5759,7 +5789,7 @@
       <c r="D133" s="10" t="s">
         <v>237</v>
       </c>
-      <c r="E133" s="18">
+      <c r="E133" s="17">
         <v>138</v>
       </c>
       <c r="F133" s="10">
@@ -5791,7 +5821,7 @@
       <c r="D134" s="10" t="s">
         <v>238</v>
       </c>
-      <c r="E134" s="18">
+      <c r="E134" s="17">
         <v>138</v>
       </c>
       <c r="F134" s="10">
@@ -5823,7 +5853,7 @@
       <c r="D135" s="10" t="s">
         <v>239</v>
       </c>
-      <c r="E135" s="18">
+      <c r="E135" s="17">
         <v>138</v>
       </c>
       <c r="F135" s="10">
@@ -5855,7 +5885,7 @@
       <c r="D136" s="10" t="s">
         <v>240</v>
       </c>
-      <c r="E136" s="18">
+      <c r="E136" s="17">
         <v>138</v>
       </c>
       <c r="F136" s="10">
@@ -5887,7 +5917,7 @@
       <c r="D137" s="10" t="s">
         <v>241</v>
       </c>
-      <c r="E137" s="18">
+      <c r="E137" s="17">
         <v>138</v>
       </c>
       <c r="F137" s="10">
@@ -5919,7 +5949,7 @@
       <c r="D138" s="10" t="s">
         <v>241</v>
       </c>
-      <c r="E138" s="18">
+      <c r="E138" s="17">
         <v>138</v>
       </c>
       <c r="F138" s="10">
@@ -5951,7 +5981,7 @@
       <c r="D139" s="10" t="s">
         <v>242</v>
       </c>
-      <c r="E139" s="18">
+      <c r="E139" s="17">
         <v>138</v>
       </c>
       <c r="F139" s="10">
@@ -5983,7 +6013,7 @@
       <c r="D140" s="10" t="s">
         <v>242</v>
       </c>
-      <c r="E140" s="18">
+      <c r="E140" s="17">
         <v>138</v>
       </c>
       <c r="F140" s="10">
@@ -6015,7 +6045,7 @@
       <c r="D141" s="10" t="s">
         <v>243</v>
       </c>
-      <c r="E141" s="18">
+      <c r="E141" s="17">
         <v>138</v>
       </c>
       <c r="F141" s="10">
@@ -6047,7 +6077,7 @@
       <c r="D142" s="10" t="s">
         <v>244</v>
       </c>
-      <c r="E142" s="18">
+      <c r="E142" s="17">
         <v>138</v>
       </c>
       <c r="F142" s="10">
@@ -6079,7 +6109,7 @@
       <c r="D143" s="10" t="s">
         <v>244</v>
       </c>
-      <c r="E143" s="18">
+      <c r="E143" s="17">
         <v>138</v>
       </c>
       <c r="F143" s="10">
@@ -6111,7 +6141,7 @@
       <c r="D144" s="10" t="s">
         <v>244</v>
       </c>
-      <c r="E144" s="18">
+      <c r="E144" s="17">
         <v>138</v>
       </c>
       <c r="F144" s="10">
@@ -6143,7 +6173,7 @@
       <c r="D145" s="10" t="s">
         <v>245</v>
       </c>
-      <c r="E145" s="18">
+      <c r="E145" s="17">
         <v>138</v>
       </c>
       <c r="F145" s="10">
@@ -6175,7 +6205,7 @@
       <c r="D146" s="10" t="s">
         <v>246</v>
       </c>
-      <c r="E146" s="18">
+      <c r="E146" s="17">
         <v>138</v>
       </c>
       <c r="F146" s="10">
@@ -6207,7 +6237,7 @@
       <c r="D147" s="10" t="s">
         <v>246</v>
       </c>
-      <c r="E147" s="18">
+      <c r="E147" s="17">
         <v>138</v>
       </c>
       <c r="F147" s="10">
@@ -6239,7 +6269,7 @@
       <c r="D148" s="10" t="s">
         <v>247</v>
       </c>
-      <c r="E148" s="18">
+      <c r="E148" s="17">
         <v>138</v>
       </c>
       <c r="F148" s="10">
@@ -6271,7 +6301,7 @@
       <c r="D149" s="10" t="s">
         <v>248</v>
       </c>
-      <c r="E149" s="18">
+      <c r="E149" s="17">
         <v>138</v>
       </c>
       <c r="F149" s="10">
@@ -6303,7 +6333,7 @@
       <c r="D150" s="10" t="s">
         <v>248</v>
       </c>
-      <c r="E150" s="18">
+      <c r="E150" s="17">
         <v>138</v>
       </c>
       <c r="F150" s="10">
@@ -6335,7 +6365,7 @@
       <c r="D151" s="10" t="s">
         <v>248</v>
       </c>
-      <c r="E151" s="18">
+      <c r="E151" s="17">
         <v>138</v>
       </c>
       <c r="F151" s="10">
@@ -6367,7 +6397,7 @@
       <c r="D152" s="10" t="s">
         <v>249</v>
       </c>
-      <c r="E152" s="18">
+      <c r="E152" s="17">
         <v>138</v>
       </c>
       <c r="F152" s="10">
@@ -6399,7 +6429,7 @@
       <c r="D153" s="10" t="s">
         <v>250</v>
       </c>
-      <c r="E153" s="18">
+      <c r="E153" s="17">
         <v>138</v>
       </c>
       <c r="F153" s="10">
@@ -6431,7 +6461,7 @@
       <c r="D154" s="10" t="s">
         <v>251</v>
       </c>
-      <c r="E154" s="18">
+      <c r="E154" s="17">
         <v>138</v>
       </c>
       <c r="F154" s="10">
@@ -6463,7 +6493,7 @@
       <c r="D155" s="10" t="s">
         <v>252</v>
       </c>
-      <c r="E155" s="18">
+      <c r="E155" s="17">
         <v>138</v>
       </c>
       <c r="F155" s="10">
@@ -6495,7 +6525,7 @@
       <c r="D156" s="10" t="s">
         <v>252</v>
       </c>
-      <c r="E156" s="18">
+      <c r="E156" s="17">
         <v>138</v>
       </c>
       <c r="F156" s="10">
@@ -6527,7 +6557,7 @@
       <c r="D157" s="10" t="s">
         <v>248</v>
       </c>
-      <c r="E157" s="18">
+      <c r="E157" s="17">
         <v>138</v>
       </c>
       <c r="F157" s="10">
@@ -6559,7 +6589,7 @@
       <c r="D158" s="10" t="s">
         <v>249</v>
       </c>
-      <c r="E158" s="18">
+      <c r="E158" s="17">
         <v>138</v>
       </c>
       <c r="F158" s="10">
@@ -6591,7 +6621,7 @@
       <c r="D159" s="10" t="s">
         <v>252</v>
       </c>
-      <c r="E159" s="18">
+      <c r="E159" s="17">
         <v>138</v>
       </c>
       <c r="F159" s="10">
@@ -6623,7 +6653,7 @@
       <c r="D160" s="10" t="s">
         <v>252</v>
       </c>
-      <c r="E160" s="18">
+      <c r="E160" s="17">
         <v>138</v>
       </c>
       <c r="F160" s="10">
@@ -6655,7 +6685,7 @@
       <c r="D161" s="10" t="s">
         <v>253</v>
       </c>
-      <c r="E161" s="18">
+      <c r="E161" s="17">
         <v>138</v>
       </c>
       <c r="F161" s="10">
@@ -6687,7 +6717,7 @@
       <c r="D162" s="10" t="s">
         <v>254</v>
       </c>
-      <c r="E162" s="18">
+      <c r="E162" s="17">
         <v>138</v>
       </c>
       <c r="F162" s="10">
@@ -6719,7 +6749,7 @@
       <c r="D163" s="10" t="s">
         <v>254</v>
       </c>
-      <c r="E163" s="18">
+      <c r="E163" s="17">
         <v>138</v>
       </c>
       <c r="F163" s="10">
@@ -6751,7 +6781,7 @@
       <c r="D164" s="10" t="s">
         <v>255</v>
       </c>
-      <c r="E164" s="18">
+      <c r="E164" s="17">
         <v>138</v>
       </c>
       <c r="F164" s="10">
@@ -6783,7 +6813,7 @@
       <c r="D165" s="10" t="s">
         <v>256</v>
       </c>
-      <c r="E165" s="18">
+      <c r="E165" s="17">
         <v>138</v>
       </c>
       <c r="F165" s="10">
@@ -6815,7 +6845,7 @@
       <c r="D166" s="10" t="s">
         <v>256</v>
       </c>
-      <c r="E166" s="18">
+      <c r="E166" s="17">
         <v>138</v>
       </c>
       <c r="F166" s="10">
@@ -6847,7 +6877,7 @@
       <c r="D167" s="10" t="s">
         <v>257</v>
       </c>
-      <c r="E167" s="18">
+      <c r="E167" s="17">
         <v>138</v>
       </c>
       <c r="F167" s="10">
@@ -6879,7 +6909,7 @@
       <c r="D168" s="10" t="s">
         <v>258</v>
       </c>
-      <c r="E168" s="18">
+      <c r="E168" s="17">
         <v>138</v>
       </c>
       <c r="F168" s="10">
@@ -6911,7 +6941,7 @@
       <c r="D169" s="10" t="s">
         <v>257</v>
       </c>
-      <c r="E169" s="18">
+      <c r="E169" s="17">
         <v>138</v>
       </c>
       <c r="F169" s="10">
@@ -6943,7 +6973,7 @@
       <c r="D170" s="10" t="s">
         <v>258</v>
       </c>
-      <c r="E170" s="18">
+      <c r="E170" s="17">
         <v>138</v>
       </c>
       <c r="F170" s="10">
@@ -6975,7 +7005,7 @@
       <c r="D171" s="10" t="s">
         <v>259</v>
       </c>
-      <c r="E171" s="18">
+      <c r="E171" s="17">
         <v>138</v>
       </c>
       <c r="F171" s="10">
@@ -7007,7 +7037,7 @@
       <c r="D172" s="10" t="s">
         <v>260</v>
       </c>
-      <c r="E172" s="18">
+      <c r="E172" s="17">
         <v>138</v>
       </c>
       <c r="F172" s="10">
@@ -7039,7 +7069,7 @@
       <c r="D173" s="10" t="s">
         <v>259</v>
       </c>
-      <c r="E173" s="18">
+      <c r="E173" s="17">
         <v>138</v>
       </c>
       <c r="F173" s="10">
@@ -7071,7 +7101,7 @@
       <c r="D174" s="10" t="s">
         <v>261</v>
       </c>
-      <c r="E174" s="18">
+      <c r="E174" s="17">
         <v>138</v>
       </c>
       <c r="F174" s="10">
@@ -7103,7 +7133,7 @@
       <c r="D175" s="10" t="s">
         <v>262</v>
       </c>
-      <c r="E175" s="18">
+      <c r="E175" s="17">
         <v>138</v>
       </c>
       <c r="F175" s="10">
@@ -7135,7 +7165,7 @@
       <c r="D176" s="10" t="s">
         <v>262</v>
       </c>
-      <c r="E176" s="18">
+      <c r="E176" s="17">
         <v>138</v>
       </c>
       <c r="F176" s="10">
@@ -7167,7 +7197,7 @@
       <c r="D177" s="10" t="s">
         <v>263</v>
       </c>
-      <c r="E177" s="18">
+      <c r="E177" s="17">
         <v>138</v>
       </c>
       <c r="F177" s="10">
@@ -7199,7 +7229,7 @@
       <c r="D178" s="10" t="s">
         <v>264</v>
       </c>
-      <c r="E178" s="18">
+      <c r="E178" s="17">
         <v>138</v>
       </c>
       <c r="F178" s="10">
@@ -7231,7 +7261,7 @@
       <c r="D179" s="10" t="s">
         <v>266</v>
       </c>
-      <c r="E179" s="18">
+      <c r="E179" s="17">
         <v>138</v>
       </c>
       <c r="F179" s="10">
@@ -7263,7 +7293,7 @@
       <c r="D180" s="10" t="s">
         <v>266</v>
       </c>
-      <c r="E180" s="18">
+      <c r="E180" s="17">
         <v>138</v>
       </c>
       <c r="F180" s="10">
@@ -7295,7 +7325,7 @@
       <c r="D181" s="10" t="s">
         <v>268</v>
       </c>
-      <c r="E181" s="18">
+      <c r="E181" s="17">
         <v>138</v>
       </c>
       <c r="F181" s="10">
@@ -7327,7 +7357,7 @@
       <c r="D182" s="10" t="s">
         <v>270</v>
       </c>
-      <c r="E182" s="18">
+      <c r="E182" s="17">
         <v>138</v>
       </c>
       <c r="F182" s="10">
@@ -7359,7 +7389,7 @@
       <c r="D183" s="10" t="s">
         <v>270</v>
       </c>
-      <c r="E183" s="18">
+      <c r="E183" s="17">
         <v>138</v>
       </c>
       <c r="F183" s="10">
@@ -7391,7 +7421,7 @@
       <c r="D184" s="10" t="s">
         <v>271</v>
       </c>
-      <c r="E184" s="18">
+      <c r="E184" s="17">
         <v>345</v>
       </c>
       <c r="F184" s="10">
@@ -7423,7 +7453,7 @@
       <c r="D185" s="10" t="s">
         <v>273</v>
       </c>
-      <c r="E185" s="18">
+      <c r="E185" s="17">
         <v>138</v>
       </c>
       <c r="F185" s="10">
@@ -7455,7 +7485,7 @@
       <c r="D186" s="10" t="s">
         <v>274</v>
       </c>
-      <c r="E186" s="18">
+      <c r="E186" s="17">
         <v>138</v>
       </c>
       <c r="F186" s="10">
@@ -7571,14 +7601,15 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABBA67B1-483C-4642-AA56-A1B87583E7BE}">
-  <dimension ref="A1:P119"/>
+  <dimension ref="A1:Q152"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.5703125" customWidth="1"/>
     <col min="2" max="2" width="16.42578125" customWidth="1"/>
+    <col min="17" max="17" width="71.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16">
+    <row r="1" spans="1:17">
       <c r="A1" t="s">
         <v>11</v>
       </c>
@@ -7627,8 +7658,9 @@
       <c r="P1" s="9" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="2" spans="1:16">
+      <c r="Q1" s="20"/>
+    </row>
+    <row r="2" spans="1:17">
       <c r="A2" s="15" t="s">
         <v>275</v>
       </c>
@@ -7660,7 +7692,7 @@
       <c r="K2" s="15">
         <v>138</v>
       </c>
-      <c r="L2" t="s">
+      <c r="L2" s="15" t="s">
         <v>332</v>
       </c>
       <c r="M2" s="15">
@@ -7669,10 +7701,9 @@
       <c r="N2" s="15">
         <v>0.94</v>
       </c>
-      <c r="O2" s="15"/>
-      <c r="P2" s="15"/>
-    </row>
-    <row r="3" spans="1:16" ht="17.25">
+      <c r="Q2" s="20"/>
+    </row>
+    <row r="3" spans="1:17">
       <c r="A3" s="15" t="s">
         <v>276</v>
       </c>
@@ -7704,7 +7735,7 @@
       <c r="K3" s="15">
         <v>138</v>
       </c>
-      <c r="L3" t="s">
+      <c r="L3" s="15" t="s">
         <v>332</v>
       </c>
       <c r="M3" s="15">
@@ -7713,10 +7744,9 @@
       <c r="N3" s="15">
         <v>0.94</v>
       </c>
-      <c r="O3" s="16"/>
-      <c r="P3" s="15"/>
-    </row>
-    <row r="4" spans="1:16">
+      <c r="Q3" s="20"/>
+    </row>
+    <row r="4" spans="1:17">
       <c r="A4" s="15" t="s">
         <v>277</v>
       </c>
@@ -7748,7 +7778,7 @@
       <c r="K4" s="15">
         <v>138</v>
       </c>
-      <c r="L4" t="s">
+      <c r="L4" s="15" t="s">
         <v>332</v>
       </c>
       <c r="M4" s="15">
@@ -7757,10 +7787,9 @@
       <c r="N4" s="15">
         <v>0.94</v>
       </c>
-      <c r="O4" s="15"/>
-      <c r="P4" s="15"/>
-    </row>
-    <row r="5" spans="1:16">
+      <c r="Q4" s="20"/>
+    </row>
+    <row r="5" spans="1:17">
       <c r="A5" s="15" t="s">
         <v>278</v>
       </c>
@@ -7792,7 +7821,7 @@
       <c r="K5" s="15">
         <v>138</v>
       </c>
-      <c r="L5" t="s">
+      <c r="L5" s="15" t="s">
         <v>332</v>
       </c>
       <c r="M5" s="15">
@@ -7801,10 +7830,9 @@
       <c r="N5" s="15">
         <v>0.94</v>
       </c>
-      <c r="O5" s="15"/>
-      <c r="P5" s="15"/>
-    </row>
-    <row r="6" spans="1:16">
+      <c r="Q5" s="20"/>
+    </row>
+    <row r="6" spans="1:17">
       <c r="A6" s="15" t="s">
         <v>279</v>
       </c>
@@ -7836,7 +7864,7 @@
       <c r="K6" s="15">
         <v>138</v>
       </c>
-      <c r="L6" t="s">
+      <c r="L6" s="15" t="s">
         <v>332</v>
       </c>
       <c r="M6" s="15">
@@ -7845,10 +7873,9 @@
       <c r="N6" s="15">
         <v>0.94</v>
       </c>
-      <c r="O6" s="15"/>
-      <c r="P6" s="15"/>
-    </row>
-    <row r="7" spans="1:16">
+      <c r="Q6" s="20"/>
+    </row>
+    <row r="7" spans="1:17">
       <c r="A7" s="15" t="s">
         <v>280</v>
       </c>
@@ -7880,7 +7907,7 @@
       <c r="K7" s="15">
         <v>138</v>
       </c>
-      <c r="L7" t="s">
+      <c r="L7" s="15" t="s">
         <v>332</v>
       </c>
       <c r="M7" s="15">
@@ -7889,10 +7916,9 @@
       <c r="N7" s="15">
         <v>0.94</v>
       </c>
-      <c r="O7" s="15"/>
-      <c r="P7" s="15"/>
-    </row>
-    <row r="8" spans="1:16">
+      <c r="Q7" s="20"/>
+    </row>
+    <row r="8" spans="1:17">
       <c r="A8" s="15" t="s">
         <v>281</v>
       </c>
@@ -7924,7 +7950,7 @@
       <c r="K8" s="15">
         <v>138</v>
       </c>
-      <c r="L8" t="s">
+      <c r="L8" s="15" t="s">
         <v>332</v>
       </c>
       <c r="M8" s="15">
@@ -7933,10 +7959,9 @@
       <c r="N8" s="15">
         <v>0.94</v>
       </c>
-      <c r="O8" s="15"/>
-      <c r="P8" s="15"/>
-    </row>
-    <row r="9" spans="1:16">
+      <c r="Q8" s="20"/>
+    </row>
+    <row r="9" spans="1:17">
       <c r="A9" s="15" t="s">
         <v>282</v>
       </c>
@@ -7968,7 +7993,7 @@
       <c r="K9" s="15">
         <v>345</v>
       </c>
-      <c r="L9" t="s">
+      <c r="L9" s="15" t="s">
         <v>332</v>
       </c>
       <c r="M9" s="15">
@@ -7977,10 +8002,9 @@
       <c r="N9" s="15">
         <v>0.94</v>
       </c>
-      <c r="O9" s="15"/>
-      <c r="P9" s="15"/>
-    </row>
-    <row r="10" spans="1:16">
+      <c r="Q9" s="20"/>
+    </row>
+    <row r="10" spans="1:17">
       <c r="A10" s="15" t="s">
         <v>283</v>
       </c>
@@ -8012,7 +8036,7 @@
       <c r="K10" s="15">
         <v>345</v>
       </c>
-      <c r="L10" t="s">
+      <c r="L10" s="15" t="s">
         <v>332</v>
       </c>
       <c r="M10" s="15">
@@ -8021,10 +8045,9 @@
       <c r="N10" s="15">
         <v>0.94</v>
       </c>
-      <c r="O10" s="15"/>
-      <c r="P10" s="15"/>
-    </row>
-    <row r="11" spans="1:16">
+      <c r="Q10" s="20"/>
+    </row>
+    <row r="11" spans="1:17">
       <c r="A11" s="15" t="s">
         <v>284</v>
       </c>
@@ -8056,7 +8079,7 @@
       <c r="K11" s="15">
         <v>345</v>
       </c>
-      <c r="L11" t="s">
+      <c r="L11" s="15" t="s">
         <v>332</v>
       </c>
       <c r="M11" s="15">
@@ -8065,10 +8088,9 @@
       <c r="N11" s="15">
         <v>0.94</v>
       </c>
-      <c r="O11" s="15"/>
-      <c r="P11" s="15"/>
-    </row>
-    <row r="12" spans="1:16">
+      <c r="Q11" s="20"/>
+    </row>
+    <row r="12" spans="1:17">
       <c r="A12" s="15" t="s">
         <v>285</v>
       </c>
@@ -8100,7 +8122,7 @@
       <c r="K12" s="15">
         <v>138</v>
       </c>
-      <c r="L12" t="s">
+      <c r="L12" s="15" t="s">
         <v>332</v>
       </c>
       <c r="M12" s="15">
@@ -8109,10 +8131,9 @@
       <c r="N12" s="15">
         <v>0.94</v>
       </c>
-      <c r="O12" s="15"/>
-      <c r="P12" s="15"/>
-    </row>
-    <row r="13" spans="1:16">
+      <c r="Q12" s="20"/>
+    </row>
+    <row r="13" spans="1:17">
       <c r="A13" s="15" t="s">
         <v>272</v>
       </c>
@@ -8144,7 +8165,7 @@
       <c r="K13" s="15">
         <v>138</v>
       </c>
-      <c r="L13" t="s">
+      <c r="L13" s="15" t="s">
         <v>332</v>
       </c>
       <c r="M13" s="15">
@@ -8153,10 +8174,9 @@
       <c r="N13" s="15">
         <v>0.94</v>
       </c>
-      <c r="O13" s="15"/>
-      <c r="P13" s="15"/>
-    </row>
-    <row r="14" spans="1:16">
+      <c r="Q13" s="20"/>
+    </row>
+    <row r="14" spans="1:17">
       <c r="A14" s="15" t="s">
         <v>286</v>
       </c>
@@ -8188,7 +8208,7 @@
       <c r="K14" s="15">
         <v>138</v>
       </c>
-      <c r="L14" t="s">
+      <c r="L14" s="15" t="s">
         <v>332</v>
       </c>
       <c r="M14" s="15">
@@ -8197,10 +8217,9 @@
       <c r="N14" s="15">
         <v>0.94</v>
       </c>
-      <c r="O14" s="15"/>
-      <c r="P14" s="15"/>
-    </row>
-    <row r="15" spans="1:16">
+      <c r="Q14" s="20"/>
+    </row>
+    <row r="15" spans="1:17">
       <c r="A15" s="15" t="s">
         <v>287</v>
       </c>
@@ -8232,7 +8251,7 @@
       <c r="K15" s="15">
         <v>138</v>
       </c>
-      <c r="L15" t="s">
+      <c r="L15" s="15" t="s">
         <v>332</v>
       </c>
       <c r="M15" s="15">
@@ -8241,10 +8260,9 @@
       <c r="N15" s="15">
         <v>0.94</v>
       </c>
-      <c r="O15" s="15"/>
-      <c r="P15" s="15"/>
-    </row>
-    <row r="16" spans="1:16">
+      <c r="Q15" s="20"/>
+    </row>
+    <row r="16" spans="1:17">
       <c r="A16" s="15" t="s">
         <v>288</v>
       </c>
@@ -8276,7 +8294,7 @@
       <c r="K16" s="15">
         <v>138</v>
       </c>
-      <c r="L16" t="s">
+      <c r="L16" s="15" t="s">
         <v>332</v>
       </c>
       <c r="M16" s="15">
@@ -8285,10 +8303,9 @@
       <c r="N16" s="15">
         <v>0.94</v>
       </c>
-      <c r="O16" s="15"/>
-      <c r="P16" s="15"/>
-    </row>
-    <row r="17" spans="1:16">
+      <c r="Q16" s="20"/>
+    </row>
+    <row r="17" spans="1:17">
       <c r="A17" s="15" t="s">
         <v>289</v>
       </c>
@@ -8320,7 +8337,7 @@
       <c r="K17" s="15">
         <v>138</v>
       </c>
-      <c r="L17" t="s">
+      <c r="L17" s="15" t="s">
         <v>332</v>
       </c>
       <c r="M17" s="15">
@@ -8329,10 +8346,9 @@
       <c r="N17" s="15">
         <v>0.94</v>
       </c>
-      <c r="O17" s="15"/>
-      <c r="P17" s="15"/>
-    </row>
-    <row r="18" spans="1:16">
+      <c r="Q17" s="20"/>
+    </row>
+    <row r="18" spans="1:17">
       <c r="A18" s="15" t="s">
         <v>265</v>
       </c>
@@ -8364,8 +8380,8 @@
       <c r="K18" s="15">
         <v>138</v>
       </c>
-      <c r="L18" t="s">
-        <v>332</v>
+      <c r="L18" s="15" t="s">
+        <v>333</v>
       </c>
       <c r="M18" s="15">
         <v>1.06</v>
@@ -8373,10 +8389,9 @@
       <c r="N18" s="15">
         <v>0.94</v>
       </c>
-      <c r="O18" s="15"/>
-      <c r="P18" s="15"/>
-    </row>
-    <row r="19" spans="1:16">
+      <c r="Q18" s="20"/>
+    </row>
+    <row r="19" spans="1:17">
       <c r="A19" s="15" t="s">
         <v>290</v>
       </c>
@@ -8408,8 +8423,8 @@
       <c r="K19" s="15">
         <v>138</v>
       </c>
-      <c r="L19" t="s">
-        <v>332</v>
+      <c r="L19" s="15" t="s">
+        <v>333</v>
       </c>
       <c r="M19" s="15">
         <v>1.06</v>
@@ -8417,10 +8432,9 @@
       <c r="N19" s="15">
         <v>0.94</v>
       </c>
-      <c r="O19" s="15"/>
-      <c r="P19" s="15"/>
-    </row>
-    <row r="20" spans="1:16">
+      <c r="Q19" s="20"/>
+    </row>
+    <row r="20" spans="1:17">
       <c r="A20" s="15" t="s">
         <v>291</v>
       </c>
@@ -8452,8 +8466,8 @@
       <c r="K20" s="15">
         <v>138</v>
       </c>
-      <c r="L20" t="s">
-        <v>332</v>
+      <c r="L20" s="15" t="s">
+        <v>333</v>
       </c>
       <c r="M20" s="15">
         <v>1.06</v>
@@ -8461,10 +8475,9 @@
       <c r="N20" s="15">
         <v>0.94</v>
       </c>
-      <c r="O20" s="15"/>
-      <c r="P20" s="15"/>
-    </row>
-    <row r="21" spans="1:16">
+      <c r="Q20" s="20"/>
+    </row>
+    <row r="21" spans="1:17">
       <c r="A21" s="15" t="s">
         <v>292</v>
       </c>
@@ -8496,8 +8509,8 @@
       <c r="K21" s="15">
         <v>138</v>
       </c>
-      <c r="L21" t="s">
-        <v>332</v>
+      <c r="L21" s="15" t="s">
+        <v>333</v>
       </c>
       <c r="M21" s="15">
         <v>1.06</v>
@@ -8505,10 +8518,9 @@
       <c r="N21" s="15">
         <v>0.94</v>
       </c>
-      <c r="O21" s="15"/>
-      <c r="P21" s="15"/>
-    </row>
-    <row r="22" spans="1:16">
+      <c r="Q21" s="20"/>
+    </row>
+    <row r="22" spans="1:17">
       <c r="A22" s="15" t="s">
         <v>293</v>
       </c>
@@ -8540,8 +8552,8 @@
       <c r="K22" s="15">
         <v>138</v>
       </c>
-      <c r="L22" t="s">
-        <v>332</v>
+      <c r="L22" s="15" t="s">
+        <v>333</v>
       </c>
       <c r="M22" s="15">
         <v>1.06</v>
@@ -8549,10 +8561,9 @@
       <c r="N22" s="15">
         <v>0.94</v>
       </c>
-      <c r="O22" s="15"/>
-      <c r="P22" s="15"/>
-    </row>
-    <row r="23" spans="1:16">
+      <c r="Q22" s="20"/>
+    </row>
+    <row r="23" spans="1:17">
       <c r="A23" s="15" t="s">
         <v>294</v>
       </c>
@@ -8584,8 +8595,8 @@
       <c r="K23" s="15">
         <v>138</v>
       </c>
-      <c r="L23" t="s">
-        <v>332</v>
+      <c r="L23" s="15" t="s">
+        <v>333</v>
       </c>
       <c r="M23" s="15">
         <v>1.06</v>
@@ -8593,10 +8604,9 @@
       <c r="N23" s="15">
         <v>0.94</v>
       </c>
-      <c r="O23" s="15"/>
-      <c r="P23" s="15"/>
-    </row>
-    <row r="24" spans="1:16">
+      <c r="Q23" s="20"/>
+    </row>
+    <row r="24" spans="1:17">
       <c r="A24" s="15" t="s">
         <v>295</v>
       </c>
@@ -8628,8 +8638,8 @@
       <c r="K24" s="15">
         <v>138</v>
       </c>
-      <c r="L24" t="s">
-        <v>332</v>
+      <c r="L24" s="15" t="s">
+        <v>333</v>
       </c>
       <c r="M24" s="15">
         <v>1.06</v>
@@ -8637,10 +8647,9 @@
       <c r="N24" s="15">
         <v>0.94</v>
       </c>
-      <c r="O24" s="15"/>
-      <c r="P24" s="15"/>
-    </row>
-    <row r="25" spans="1:16">
+      <c r="Q24" s="20"/>
+    </row>
+    <row r="25" spans="1:17">
       <c r="A25" s="15" t="s">
         <v>222</v>
       </c>
@@ -8672,8 +8681,8 @@
       <c r="K25" s="15">
         <v>138</v>
       </c>
-      <c r="L25" t="s">
-        <v>332</v>
+      <c r="L25" s="15" t="s">
+        <v>333</v>
       </c>
       <c r="M25" s="15">
         <v>1.06</v>
@@ -8681,10 +8690,9 @@
       <c r="N25" s="15">
         <v>0.94</v>
       </c>
-      <c r="O25" s="15"/>
-      <c r="P25" s="15"/>
-    </row>
-    <row r="26" spans="1:16">
+      <c r="Q25" s="20"/>
+    </row>
+    <row r="26" spans="1:17">
       <c r="A26" s="15" t="s">
         <v>296</v>
       </c>
@@ -8716,8 +8724,8 @@
       <c r="K26" s="15">
         <v>138</v>
       </c>
-      <c r="L26" t="s">
-        <v>332</v>
+      <c r="L26" s="15" t="s">
+        <v>333</v>
       </c>
       <c r="M26" s="15">
         <v>1.06</v>
@@ -8725,10 +8733,9 @@
       <c r="N26" s="15">
         <v>0.94</v>
       </c>
-      <c r="O26" s="15"/>
-      <c r="P26" s="15"/>
-    </row>
-    <row r="27" spans="1:16">
+      <c r="Q26" s="20"/>
+    </row>
+    <row r="27" spans="1:17">
       <c r="A27" s="15" t="s">
         <v>297</v>
       </c>
@@ -8760,8 +8767,8 @@
       <c r="K27" s="15">
         <v>345</v>
       </c>
-      <c r="L27" t="s">
-        <v>332</v>
+      <c r="L27" s="15" t="s">
+        <v>333</v>
       </c>
       <c r="M27" s="15">
         <v>1.06</v>
@@ -8769,10 +8776,9 @@
       <c r="N27" s="15">
         <v>0.94</v>
       </c>
-      <c r="O27" s="15"/>
-      <c r="P27" s="15"/>
-    </row>
-    <row r="28" spans="1:16">
+      <c r="Q27" s="20"/>
+    </row>
+    <row r="28" spans="1:17">
       <c r="A28" s="15" t="s">
         <v>269</v>
       </c>
@@ -8804,8 +8810,8 @@
       <c r="K28" s="15">
         <v>138</v>
       </c>
-      <c r="L28" t="s">
-        <v>332</v>
+      <c r="L28" s="15" t="s">
+        <v>333</v>
       </c>
       <c r="M28" s="15">
         <v>1.06</v>
@@ -8813,10 +8819,9 @@
       <c r="N28" s="15">
         <v>0.94</v>
       </c>
-      <c r="O28" s="15"/>
-      <c r="P28" s="15"/>
-    </row>
-    <row r="29" spans="1:16">
+      <c r="Q28" s="20"/>
+    </row>
+    <row r="29" spans="1:17">
       <c r="A29" s="15" t="s">
         <v>298</v>
       </c>
@@ -8848,8 +8853,8 @@
       <c r="K29" s="15">
         <v>138</v>
       </c>
-      <c r="L29" t="s">
-        <v>332</v>
+      <c r="L29" s="15" t="s">
+        <v>333</v>
       </c>
       <c r="M29" s="15">
         <v>1.06</v>
@@ -8857,10 +8862,9 @@
       <c r="N29" s="15">
         <v>0.94</v>
       </c>
-      <c r="O29" s="15"/>
-      <c r="P29" s="15"/>
-    </row>
-    <row r="30" spans="1:16">
+      <c r="Q29" s="20"/>
+    </row>
+    <row r="30" spans="1:17">
       <c r="A30" s="15" t="s">
         <v>299</v>
       </c>
@@ -8892,8 +8896,8 @@
       <c r="K30" s="15">
         <v>138</v>
       </c>
-      <c r="L30" t="s">
-        <v>332</v>
+      <c r="L30" s="15" t="s">
+        <v>333</v>
       </c>
       <c r="M30" s="15">
         <v>1.06</v>
@@ -8901,10 +8905,9 @@
       <c r="N30" s="15">
         <v>0.94</v>
       </c>
-      <c r="O30" s="15"/>
-      <c r="P30" s="15"/>
-    </row>
-    <row r="31" spans="1:16">
+      <c r="Q30" s="20"/>
+    </row>
+    <row r="31" spans="1:17">
       <c r="A31" s="15" t="s">
         <v>300</v>
       </c>
@@ -8936,8 +8939,8 @@
       <c r="K31" s="15">
         <v>345</v>
       </c>
-      <c r="L31" t="s">
-        <v>332</v>
+      <c r="L31" s="15" t="s">
+        <v>333</v>
       </c>
       <c r="M31" s="15">
         <v>1.06</v>
@@ -8945,10 +8948,9 @@
       <c r="N31" s="15">
         <v>0.94</v>
       </c>
-      <c r="O31" s="15"/>
-      <c r="P31" s="15"/>
-    </row>
-    <row r="32" spans="1:16">
+      <c r="Q31" s="20"/>
+    </row>
+    <row r="32" spans="1:17">
       <c r="A32" s="15" t="s">
         <v>301</v>
       </c>
@@ -8980,8 +8982,8 @@
       <c r="K32" s="15">
         <v>138</v>
       </c>
-      <c r="L32" t="s">
-        <v>332</v>
+      <c r="L32" s="15" t="s">
+        <v>333</v>
       </c>
       <c r="M32" s="15">
         <v>1.06</v>
@@ -8989,10 +8991,9 @@
       <c r="N32" s="15">
         <v>0.94</v>
       </c>
-      <c r="O32" s="15"/>
-      <c r="P32" s="15"/>
-    </row>
-    <row r="33" spans="1:16">
+      <c r="Q32" s="20"/>
+    </row>
+    <row r="33" spans="1:17">
       <c r="A33" s="15" t="s">
         <v>267</v>
       </c>
@@ -9024,8 +9025,8 @@
       <c r="K33" s="15">
         <v>138</v>
       </c>
-      <c r="L33" t="s">
-        <v>332</v>
+      <c r="L33" s="15" t="s">
+        <v>333</v>
       </c>
       <c r="M33" s="15">
         <v>1.06</v>
@@ -9033,10 +9034,9 @@
       <c r="N33" s="15">
         <v>0.94</v>
       </c>
-      <c r="O33" s="15"/>
-      <c r="P33" s="15"/>
-    </row>
-    <row r="34" spans="1:16">
+      <c r="Q33" s="20"/>
+    </row>
+    <row r="34" spans="1:17">
       <c r="A34" s="15" t="s">
         <v>302</v>
       </c>
@@ -9068,8 +9068,8 @@
       <c r="K34" s="15">
         <v>138</v>
       </c>
-      <c r="L34" t="s">
-        <v>332</v>
+      <c r="L34" s="15" t="s">
+        <v>333</v>
       </c>
       <c r="M34" s="15">
         <v>1.06</v>
@@ -9077,10 +9077,9 @@
       <c r="N34" s="15">
         <v>0.94</v>
       </c>
-      <c r="O34" s="15"/>
-      <c r="P34" s="15"/>
-    </row>
-    <row r="35" spans="1:16">
+      <c r="Q34" s="20"/>
+    </row>
+    <row r="35" spans="1:17">
       <c r="A35" s="15" t="s">
         <v>303</v>
       </c>
@@ -9112,7 +9111,7 @@
       <c r="K35" s="15">
         <v>138</v>
       </c>
-      <c r="L35" t="s">
+      <c r="L35" s="15" t="s">
         <v>333</v>
       </c>
       <c r="M35" s="15">
@@ -9121,10 +9120,9 @@
       <c r="N35" s="15">
         <v>0.94</v>
       </c>
-      <c r="O35" s="15"/>
-      <c r="P35" s="15"/>
-    </row>
-    <row r="36" spans="1:16">
+      <c r="Q35" s="20"/>
+    </row>
+    <row r="36" spans="1:17">
       <c r="A36" s="15" t="s">
         <v>304</v>
       </c>
@@ -9156,7 +9154,7 @@
       <c r="K36" s="15">
         <v>138</v>
       </c>
-      <c r="L36" t="s">
+      <c r="L36" s="15" t="s">
         <v>333</v>
       </c>
       <c r="M36" s="15">
@@ -9165,10 +9163,9 @@
       <c r="N36" s="15">
         <v>0.94</v>
       </c>
-      <c r="O36" s="15"/>
-      <c r="P36" s="15"/>
-    </row>
-    <row r="37" spans="1:16">
+      <c r="Q36" s="20"/>
+    </row>
+    <row r="37" spans="1:17">
       <c r="A37" s="15" t="s">
         <v>305</v>
       </c>
@@ -9200,7 +9197,7 @@
       <c r="K37" s="15">
         <v>138</v>
       </c>
-      <c r="L37" t="s">
+      <c r="L37" s="15" t="s">
         <v>333</v>
       </c>
       <c r="M37" s="15">
@@ -9209,10 +9206,9 @@
       <c r="N37" s="15">
         <v>0.94</v>
       </c>
-      <c r="O37" s="15"/>
-      <c r="P37" s="15"/>
-    </row>
-    <row r="38" spans="1:16">
+      <c r="Q37" s="20"/>
+    </row>
+    <row r="38" spans="1:17">
       <c r="A38" s="15" t="s">
         <v>306</v>
       </c>
@@ -9244,7 +9240,7 @@
       <c r="K38" s="15">
         <v>138</v>
       </c>
-      <c r="L38" t="s">
+      <c r="L38" s="15" t="s">
         <v>333</v>
       </c>
       <c r="M38" s="15">
@@ -9253,10 +9249,9 @@
       <c r="N38" s="15">
         <v>0.94</v>
       </c>
-      <c r="O38" s="15"/>
-      <c r="P38" s="15"/>
-    </row>
-    <row r="39" spans="1:16">
+      <c r="Q38" s="20"/>
+    </row>
+    <row r="39" spans="1:17">
       <c r="A39" s="15" t="s">
         <v>307</v>
       </c>
@@ -9288,7 +9283,7 @@
       <c r="K39" s="15">
         <v>345</v>
       </c>
-      <c r="L39" t="s">
+      <c r="L39" s="15" t="s">
         <v>333</v>
       </c>
       <c r="M39" s="15">
@@ -9297,10 +9292,9 @@
       <c r="N39" s="15">
         <v>0.94</v>
       </c>
-      <c r="O39" s="15"/>
-      <c r="P39" s="15"/>
-    </row>
-    <row r="40" spans="1:16">
+      <c r="Q39" s="20"/>
+    </row>
+    <row r="40" spans="1:17">
       <c r="A40" s="15" t="s">
         <v>308</v>
       </c>
@@ -9332,7 +9326,7 @@
       <c r="K40" s="15">
         <v>138</v>
       </c>
-      <c r="L40" t="s">
+      <c r="L40" s="15" t="s">
         <v>333</v>
       </c>
       <c r="M40" s="15">
@@ -9341,10 +9335,9 @@
       <c r="N40" s="15">
         <v>0.94</v>
       </c>
-      <c r="O40" s="15"/>
-      <c r="P40" s="15"/>
-    </row>
-    <row r="41" spans="1:16">
+      <c r="Q40" s="20"/>
+    </row>
+    <row r="41" spans="1:17">
       <c r="A41" s="15" t="s">
         <v>309</v>
       </c>
@@ -9376,7 +9369,7 @@
       <c r="K41" s="15">
         <v>138</v>
       </c>
-      <c r="L41" t="s">
+      <c r="L41" s="15" t="s">
         <v>333</v>
       </c>
       <c r="M41" s="15">
@@ -9385,10 +9378,9 @@
       <c r="N41" s="15">
         <v>0.94</v>
       </c>
-      <c r="O41" s="15"/>
-      <c r="P41" s="15"/>
-    </row>
-    <row r="42" spans="1:16">
+      <c r="Q41" s="20"/>
+    </row>
+    <row r="42" spans="1:17">
       <c r="A42" s="15" t="s">
         <v>310</v>
       </c>
@@ -9420,8 +9412,8 @@
       <c r="K42" s="15">
         <v>138</v>
       </c>
-      <c r="L42" t="s">
-        <v>333</v>
+      <c r="L42" s="15" t="s">
+        <v>334</v>
       </c>
       <c r="M42" s="15">
         <v>1.06</v>
@@ -9429,10 +9421,9 @@
       <c r="N42" s="15">
         <v>0.94</v>
       </c>
-      <c r="O42" s="15"/>
-      <c r="P42" s="15"/>
-    </row>
-    <row r="43" spans="1:16">
+      <c r="Q42" s="20"/>
+    </row>
+    <row r="43" spans="1:17">
       <c r="A43" s="15" t="s">
         <v>311</v>
       </c>
@@ -9464,8 +9455,8 @@
       <c r="K43" s="15">
         <v>138</v>
       </c>
-      <c r="L43" t="s">
-        <v>333</v>
+      <c r="L43" s="15" t="s">
+        <v>334</v>
       </c>
       <c r="M43" s="15">
         <v>1.06</v>
@@ -9473,10 +9464,9 @@
       <c r="N43" s="15">
         <v>0.94</v>
       </c>
-      <c r="O43" s="15"/>
-      <c r="P43" s="15"/>
-    </row>
-    <row r="44" spans="1:16">
+      <c r="Q43" s="20"/>
+    </row>
+    <row r="44" spans="1:17">
       <c r="A44" s="15" t="s">
         <v>312</v>
       </c>
@@ -9508,8 +9498,8 @@
       <c r="K44" s="15">
         <v>138</v>
       </c>
-      <c r="L44" t="s">
-        <v>333</v>
+      <c r="L44" s="15" t="s">
+        <v>334</v>
       </c>
       <c r="M44" s="15">
         <v>1.06</v>
@@ -9517,10 +9507,9 @@
       <c r="N44" s="15">
         <v>0.94</v>
       </c>
-      <c r="O44" s="15"/>
-      <c r="P44" s="15"/>
-    </row>
-    <row r="45" spans="1:16">
+      <c r="Q44" s="20"/>
+    </row>
+    <row r="45" spans="1:17">
       <c r="A45" s="15" t="s">
         <v>313</v>
       </c>
@@ -9552,7 +9541,7 @@
       <c r="K45" s="15">
         <v>138</v>
       </c>
-      <c r="L45" t="s">
+      <c r="L45" s="15" t="s">
         <v>334</v>
       </c>
       <c r="M45" s="15">
@@ -9561,10 +9550,9 @@
       <c r="N45" s="15">
         <v>0.94</v>
       </c>
-      <c r="O45" s="15"/>
-      <c r="P45" s="15"/>
-    </row>
-    <row r="46" spans="1:16">
+      <c r="Q45" s="20"/>
+    </row>
+    <row r="46" spans="1:17">
       <c r="A46" s="15" t="s">
         <v>314</v>
       </c>
@@ -9596,7 +9584,7 @@
       <c r="K46" s="15">
         <v>138</v>
       </c>
-      <c r="L46" t="s">
+      <c r="L46" s="15" t="s">
         <v>334</v>
       </c>
       <c r="M46" s="15">
@@ -9605,10 +9593,9 @@
       <c r="N46" s="15">
         <v>0.94</v>
       </c>
-      <c r="O46" s="15"/>
-      <c r="P46" s="15"/>
-    </row>
-    <row r="47" spans="1:16">
+      <c r="Q46" s="20"/>
+    </row>
+    <row r="47" spans="1:17">
       <c r="A47" s="15" t="s">
         <v>315</v>
       </c>
@@ -9640,7 +9627,7 @@
       <c r="K47" s="15">
         <v>138</v>
       </c>
-      <c r="L47" t="s">
+      <c r="L47" s="15" t="s">
         <v>334</v>
       </c>
       <c r="M47" s="15">
@@ -9649,10 +9636,9 @@
       <c r="N47" s="15">
         <v>0.94</v>
       </c>
-      <c r="O47" s="15"/>
-      <c r="P47" s="15"/>
-    </row>
-    <row r="48" spans="1:16">
+      <c r="Q47" s="20"/>
+    </row>
+    <row r="48" spans="1:17">
       <c r="A48" s="15" t="s">
         <v>218</v>
       </c>
@@ -9684,7 +9670,7 @@
       <c r="K48" s="15">
         <v>138</v>
       </c>
-      <c r="L48" t="s">
+      <c r="L48" s="15" t="s">
         <v>334</v>
       </c>
       <c r="M48" s="15">
@@ -9693,10 +9679,9 @@
       <c r="N48" s="15">
         <v>0.94</v>
       </c>
-      <c r="O48" s="15"/>
-      <c r="P48" s="15"/>
-    </row>
-    <row r="49" spans="1:16">
+      <c r="Q48" s="20"/>
+    </row>
+    <row r="49" spans="1:17">
       <c r="A49" s="15" t="s">
         <v>316</v>
       </c>
@@ -9728,7 +9713,7 @@
       <c r="K49" s="15">
         <v>138</v>
       </c>
-      <c r="L49" t="s">
+      <c r="L49" s="15" t="s">
         <v>334</v>
       </c>
       <c r="M49" s="15">
@@ -9737,10 +9722,9 @@
       <c r="N49" s="15">
         <v>0.94</v>
       </c>
-      <c r="O49" s="15"/>
-      <c r="P49" s="15"/>
-    </row>
-    <row r="50" spans="1:16">
+      <c r="Q49" s="20"/>
+    </row>
+    <row r="50" spans="1:17">
       <c r="A50" s="15" t="s">
         <v>220</v>
       </c>
@@ -9772,7 +9756,7 @@
       <c r="K50" s="15">
         <v>138</v>
       </c>
-      <c r="L50" t="s">
+      <c r="L50" s="15" t="s">
         <v>334</v>
       </c>
       <c r="M50" s="15">
@@ -9781,10 +9765,9 @@
       <c r="N50" s="15">
         <v>0.94</v>
       </c>
-      <c r="O50" s="15"/>
-      <c r="P50" s="15"/>
-    </row>
-    <row r="51" spans="1:16">
+      <c r="Q50" s="20"/>
+    </row>
+    <row r="51" spans="1:17">
       <c r="A51" s="15" t="s">
         <v>317</v>
       </c>
@@ -9816,7 +9799,7 @@
       <c r="K51" s="15">
         <v>138</v>
       </c>
-      <c r="L51" t="s">
+      <c r="L51" s="15" t="s">
         <v>334</v>
       </c>
       <c r="M51" s="15">
@@ -9825,10 +9808,9 @@
       <c r="N51" s="15">
         <v>0.94</v>
       </c>
-      <c r="O51" s="15"/>
-      <c r="P51" s="15"/>
-    </row>
-    <row r="52" spans="1:16">
+      <c r="Q51" s="20"/>
+    </row>
+    <row r="52" spans="1:17">
       <c r="A52" s="15" t="s">
         <v>318</v>
       </c>
@@ -9860,7 +9842,7 @@
       <c r="K52" s="15">
         <v>138</v>
       </c>
-      <c r="L52" t="s">
+      <c r="L52" s="15" t="s">
         <v>334</v>
       </c>
       <c r="M52" s="15">
@@ -9869,10 +9851,9 @@
       <c r="N52" s="15">
         <v>0.94</v>
       </c>
-      <c r="O52" s="15"/>
-      <c r="P52" s="15"/>
-    </row>
-    <row r="53" spans="1:16">
+      <c r="Q52" s="20"/>
+    </row>
+    <row r="53" spans="1:17">
       <c r="A53" s="15" t="s">
         <v>319</v>
       </c>
@@ -9904,7 +9885,7 @@
       <c r="K53" s="15">
         <v>138</v>
       </c>
-      <c r="L53" t="s">
+      <c r="L53" s="15" t="s">
         <v>334</v>
       </c>
       <c r="M53" s="15">
@@ -9913,10 +9894,9 @@
       <c r="N53" s="15">
         <v>0.94</v>
       </c>
-      <c r="O53" s="15"/>
-      <c r="P53" s="15"/>
-    </row>
-    <row r="54" spans="1:16">
+      <c r="Q53" s="20"/>
+    </row>
+    <row r="54" spans="1:17">
       <c r="A54" s="15" t="s">
         <v>320</v>
       </c>
@@ -9948,7 +9928,7 @@
       <c r="K54" s="15">
         <v>138</v>
       </c>
-      <c r="L54" t="s">
+      <c r="L54" s="15" t="s">
         <v>334</v>
       </c>
       <c r="M54" s="15">
@@ -9957,10 +9937,9 @@
       <c r="N54" s="15">
         <v>0.94</v>
       </c>
-      <c r="O54" s="15"/>
-      <c r="P54" s="15"/>
-    </row>
-    <row r="55" spans="1:16">
+      <c r="Q54" s="20"/>
+    </row>
+    <row r="55" spans="1:17">
       <c r="A55" s="15" t="s">
         <v>321</v>
       </c>
@@ -9992,7 +9971,7 @@
       <c r="K55" s="15">
         <v>138</v>
       </c>
-      <c r="L55" t="s">
+      <c r="L55" s="15" t="s">
         <v>334</v>
       </c>
       <c r="M55" s="15">
@@ -10001,10 +9980,9 @@
       <c r="N55" s="15">
         <v>0.94</v>
       </c>
-      <c r="O55" s="15"/>
-      <c r="P55" s="15"/>
-    </row>
-    <row r="56" spans="1:16">
+      <c r="Q55" s="20"/>
+    </row>
+    <row r="56" spans="1:17">
       <c r="A56" s="15" t="s">
         <v>322</v>
       </c>
@@ -10036,7 +10014,7 @@
       <c r="K56" s="15">
         <v>138</v>
       </c>
-      <c r="L56" t="s">
+      <c r="L56" s="15" t="s">
         <v>334</v>
       </c>
       <c r="M56" s="15">
@@ -10045,10 +10023,9 @@
       <c r="N56" s="15">
         <v>0.94</v>
       </c>
-      <c r="O56" s="15"/>
-      <c r="P56" s="15"/>
-    </row>
-    <row r="57" spans="1:16">
+      <c r="Q56" s="20"/>
+    </row>
+    <row r="57" spans="1:17">
       <c r="A57" s="15" t="s">
         <v>323</v>
       </c>
@@ -10080,7 +10057,7 @@
       <c r="K57" s="15">
         <v>138</v>
       </c>
-      <c r="L57" t="s">
+      <c r="L57" s="15" t="s">
         <v>334</v>
       </c>
       <c r="M57" s="15">
@@ -10089,10 +10066,9 @@
       <c r="N57" s="15">
         <v>0.94</v>
       </c>
-      <c r="O57" s="15"/>
-      <c r="P57" s="15"/>
-    </row>
-    <row r="58" spans="1:16">
+      <c r="Q57" s="20"/>
+    </row>
+    <row r="58" spans="1:17">
       <c r="A58" s="15" t="s">
         <v>324</v>
       </c>
@@ -10124,7 +10100,7 @@
       <c r="K58" s="15">
         <v>138</v>
       </c>
-      <c r="L58" t="s">
+      <c r="L58" s="15" t="s">
         <v>334</v>
       </c>
       <c r="M58" s="15">
@@ -10133,10 +10109,9 @@
       <c r="N58" s="15">
         <v>0.94</v>
       </c>
-      <c r="O58" s="15"/>
-      <c r="P58" s="15"/>
-    </row>
-    <row r="59" spans="1:16">
+      <c r="Q58" s="20"/>
+    </row>
+    <row r="59" spans="1:17">
       <c r="A59" s="15" t="s">
         <v>325</v>
       </c>
@@ -10168,7 +10143,7 @@
       <c r="K59" s="15">
         <v>138</v>
       </c>
-      <c r="L59" t="s">
+      <c r="L59" s="15" t="s">
         <v>334</v>
       </c>
       <c r="M59" s="15">
@@ -10177,10 +10152,9 @@
       <c r="N59" s="15">
         <v>0.94</v>
       </c>
-      <c r="O59" s="15"/>
-      <c r="P59" s="15"/>
-    </row>
-    <row r="60" spans="1:16">
+      <c r="Q59" s="20"/>
+    </row>
+    <row r="60" spans="1:17">
       <c r="A60" s="15" t="s">
         <v>326</v>
       </c>
@@ -10212,7 +10186,7 @@
       <c r="K60" s="15">
         <v>138</v>
       </c>
-      <c r="L60" t="s">
+      <c r="L60" s="15" t="s">
         <v>334</v>
       </c>
       <c r="M60" s="15">
@@ -10221,10 +10195,9 @@
       <c r="N60" s="15">
         <v>0.94</v>
       </c>
-      <c r="O60" s="15"/>
-      <c r="P60" s="15"/>
-    </row>
-    <row r="61" spans="1:16">
+      <c r="Q60" s="20"/>
+    </row>
+    <row r="61" spans="1:17">
       <c r="A61" s="15" t="s">
         <v>327</v>
       </c>
@@ -10256,7 +10229,7 @@
       <c r="K61" s="15">
         <v>138</v>
       </c>
-      <c r="L61" t="s">
+      <c r="L61" s="15" t="s">
         <v>334</v>
       </c>
       <c r="M61" s="15">
@@ -10265,10 +10238,9 @@
       <c r="N61" s="15">
         <v>0.94</v>
       </c>
-      <c r="O61" s="15"/>
-      <c r="P61" s="15"/>
-    </row>
-    <row r="62" spans="1:16">
+      <c r="Q61" s="20"/>
+    </row>
+    <row r="62" spans="1:17">
       <c r="A62" s="15" t="s">
         <v>328</v>
       </c>
@@ -10300,7 +10272,7 @@
       <c r="K62" s="15">
         <v>138</v>
       </c>
-      <c r="L62" t="s">
+      <c r="L62" s="15" t="s">
         <v>334</v>
       </c>
       <c r="M62" s="15">
@@ -10309,10 +10281,9 @@
       <c r="N62" s="15">
         <v>0.94</v>
       </c>
-      <c r="O62" s="15"/>
-      <c r="P62" s="15"/>
-    </row>
-    <row r="63" spans="1:16">
+      <c r="Q62" s="20"/>
+    </row>
+    <row r="63" spans="1:17">
       <c r="A63" s="15" t="s">
         <v>213</v>
       </c>
@@ -10344,7 +10315,7 @@
       <c r="K63" s="15">
         <v>138</v>
       </c>
-      <c r="L63" t="s">
+      <c r="L63" s="15" t="s">
         <v>334</v>
       </c>
       <c r="M63" s="15">
@@ -10353,10 +10324,9 @@
       <c r="N63" s="15">
         <v>0.94</v>
       </c>
-      <c r="O63" s="15"/>
-      <c r="P63" s="15"/>
-    </row>
-    <row r="64" spans="1:16">
+      <c r="Q63" s="20"/>
+    </row>
+    <row r="64" spans="1:17">
       <c r="A64" s="15" t="s">
         <v>329</v>
       </c>
@@ -10388,7 +10358,7 @@
       <c r="K64" s="15">
         <v>345</v>
       </c>
-      <c r="L64" t="s">
+      <c r="L64" s="15" t="s">
         <v>334</v>
       </c>
       <c r="M64" s="15">
@@ -10397,10 +10367,9 @@
       <c r="N64" s="15">
         <v>0.94</v>
       </c>
-      <c r="O64" s="15"/>
-      <c r="P64" s="15"/>
-    </row>
-    <row r="65" spans="1:16">
+      <c r="Q64" s="20"/>
+    </row>
+    <row r="65" spans="1:17">
       <c r="A65" s="15" t="s">
         <v>330</v>
       </c>
@@ -10432,7 +10401,7 @@
       <c r="K65" s="15">
         <v>345</v>
       </c>
-      <c r="L65" t="s">
+      <c r="L65" s="15" t="s">
         <v>334</v>
       </c>
       <c r="M65" s="15">
@@ -10441,10 +10410,9 @@
       <c r="N65" s="15">
         <v>0.94</v>
       </c>
-      <c r="O65" s="15"/>
-      <c r="P65" s="15"/>
-    </row>
-    <row r="66" spans="1:16">
+      <c r="Q65" s="20"/>
+    </row>
+    <row r="66" spans="1:17">
       <c r="A66" s="15" t="s">
         <v>216</v>
       </c>
@@ -10476,7 +10444,7 @@
       <c r="K66" s="15">
         <v>345</v>
       </c>
-      <c r="L66" t="s">
+      <c r="L66" s="15" t="s">
         <v>334</v>
       </c>
       <c r="M66" s="15">
@@ -10485,10 +10453,9 @@
       <c r="N66" s="15">
         <v>0.94</v>
       </c>
-      <c r="O66" s="15"/>
-      <c r="P66" s="15"/>
-    </row>
-    <row r="67" spans="1:16">
+      <c r="Q66" s="20"/>
+    </row>
+    <row r="67" spans="1:17">
       <c r="A67" s="15" t="s">
         <v>214</v>
       </c>
@@ -10520,7 +10487,7 @@
       <c r="K67" s="15">
         <v>138</v>
       </c>
-      <c r="L67" t="s">
+      <c r="L67" s="15" t="s">
         <v>334</v>
       </c>
       <c r="M67" s="15">
@@ -10529,10 +10496,9 @@
       <c r="N67" s="15">
         <v>0.94</v>
       </c>
-      <c r="O67" s="15"/>
-      <c r="P67" s="15"/>
-    </row>
-    <row r="68" spans="1:16">
+      <c r="Q67" s="20"/>
+    </row>
+    <row r="68" spans="1:17">
       <c r="A68" s="15" t="s">
         <v>215</v>
       </c>
@@ -10564,7 +10530,7 @@
       <c r="K68" s="15">
         <v>138</v>
       </c>
-      <c r="L68" t="s">
+      <c r="L68" s="15" t="s">
         <v>334</v>
       </c>
       <c r="M68" s="15">
@@ -10573,10 +10539,9 @@
       <c r="N68" s="15">
         <v>0.94</v>
       </c>
-      <c r="O68" s="15"/>
-      <c r="P68" s="15"/>
-    </row>
-    <row r="69" spans="1:16">
+      <c r="Q68" s="20"/>
+    </row>
+    <row r="69" spans="1:17">
       <c r="A69" s="15" t="s">
         <v>217</v>
       </c>
@@ -10608,8 +10573,8 @@
       <c r="K69" s="15">
         <v>345</v>
       </c>
-      <c r="L69" t="s">
-        <v>334</v>
+      <c r="L69" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M69" s="15">
         <v>1.06</v>
@@ -10617,10 +10582,9 @@
       <c r="N69" s="15">
         <v>0.94</v>
       </c>
-      <c r="O69" s="15"/>
-      <c r="P69" s="15"/>
-    </row>
-    <row r="70" spans="1:16">
+      <c r="Q69" s="20"/>
+    </row>
+    <row r="70" spans="1:17">
       <c r="A70" s="15" t="s">
         <v>219</v>
       </c>
@@ -10652,8 +10616,8 @@
       <c r="K70" s="15">
         <v>138</v>
       </c>
-      <c r="L70" t="s">
-        <v>334</v>
+      <c r="L70" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M70" s="15">
         <v>1.06</v>
@@ -10661,10 +10625,9 @@
       <c r="N70" s="15">
         <v>0.94</v>
       </c>
-      <c r="O70" s="15"/>
-      <c r="P70" s="15"/>
-    </row>
-    <row r="71" spans="1:16">
+      <c r="Q70" s="20"/>
+    </row>
+    <row r="71" spans="1:17">
       <c r="A71" s="15" t="s">
         <v>221</v>
       </c>
@@ -10696,8 +10659,8 @@
       <c r="K71" s="15">
         <v>138</v>
       </c>
-      <c r="L71" t="s">
-        <v>334</v>
+      <c r="L71" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M71" s="15">
         <v>1.06</v>
@@ -10705,10 +10668,9 @@
       <c r="N71" s="15">
         <v>0.94</v>
       </c>
-      <c r="O71" s="15"/>
-      <c r="P71" s="15"/>
-    </row>
-    <row r="72" spans="1:16">
+      <c r="Q71" s="20"/>
+    </row>
+    <row r="72" spans="1:17">
       <c r="A72" s="15" t="s">
         <v>223</v>
       </c>
@@ -10740,8 +10702,8 @@
       <c r="K72" s="15">
         <v>138</v>
       </c>
-      <c r="L72" t="s">
-        <v>334</v>
+      <c r="L72" s="15" t="s">
+        <v>333</v>
       </c>
       <c r="M72" s="15">
         <v>1.06</v>
@@ -10749,10 +10711,9 @@
       <c r="N72" s="15">
         <v>0.94</v>
       </c>
-      <c r="O72" s="15"/>
-      <c r="P72" s="15"/>
-    </row>
-    <row r="73" spans="1:16">
+      <c r="Q72" s="20"/>
+    </row>
+    <row r="73" spans="1:17">
       <c r="A73" s="15" t="s">
         <v>224</v>
       </c>
@@ -10784,8 +10745,8 @@
       <c r="K73" s="15">
         <v>138</v>
       </c>
-      <c r="L73" t="s">
-        <v>334</v>
+      <c r="L73" s="15" t="s">
+        <v>333</v>
       </c>
       <c r="M73" s="15">
         <v>1.06</v>
@@ -10793,10 +10754,9 @@
       <c r="N73" s="15">
         <v>0.94</v>
       </c>
-      <c r="O73" s="15"/>
-      <c r="P73" s="15"/>
-    </row>
-    <row r="74" spans="1:16">
+      <c r="Q73" s="20"/>
+    </row>
+    <row r="74" spans="1:17">
       <c r="A74" s="15" t="s">
         <v>225</v>
       </c>
@@ -10828,8 +10788,8 @@
       <c r="K74" s="15">
         <v>138</v>
       </c>
-      <c r="L74" t="s">
-        <v>334</v>
+      <c r="L74" s="15" t="s">
+        <v>333</v>
       </c>
       <c r="M74" s="15">
         <v>1.06</v>
@@ -10837,10 +10797,9 @@
       <c r="N74" s="15">
         <v>0.94</v>
       </c>
-      <c r="O74" s="15"/>
-      <c r="P74" s="15"/>
-    </row>
-    <row r="75" spans="1:16">
+      <c r="Q74" s="20"/>
+    </row>
+    <row r="75" spans="1:17">
       <c r="A75" s="15" t="s">
         <v>226</v>
       </c>
@@ -10872,8 +10831,8 @@
       <c r="K75" s="15">
         <v>138</v>
       </c>
-      <c r="L75" t="s">
-        <v>334</v>
+      <c r="L75" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M75" s="15">
         <v>1.06</v>
@@ -10881,10 +10840,9 @@
       <c r="N75" s="15">
         <v>0.94</v>
       </c>
-      <c r="O75" s="15"/>
-      <c r="P75" s="15"/>
-    </row>
-    <row r="76" spans="1:16">
+      <c r="Q75" s="20"/>
+    </row>
+    <row r="76" spans="1:17">
       <c r="A76" s="15" t="s">
         <v>227</v>
       </c>
@@ -10916,8 +10874,8 @@
       <c r="K76" s="15">
         <v>138</v>
       </c>
-      <c r="L76" t="s">
-        <v>334</v>
+      <c r="L76" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M76" s="15">
         <v>1.06</v>
@@ -10925,10 +10883,9 @@
       <c r="N76" s="15">
         <v>0.94</v>
       </c>
-      <c r="O76" s="15"/>
-      <c r="P76" s="15"/>
-    </row>
-    <row r="77" spans="1:16">
+      <c r="Q76" s="20"/>
+    </row>
+    <row r="77" spans="1:17">
       <c r="A77" s="15" t="s">
         <v>228</v>
       </c>
@@ -10960,8 +10917,8 @@
       <c r="K77" s="15">
         <v>138</v>
       </c>
-      <c r="L77" t="s">
-        <v>334</v>
+      <c r="L77" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M77" s="15">
         <v>1.06</v>
@@ -10969,10 +10926,9 @@
       <c r="N77" s="15">
         <v>0.94</v>
       </c>
-      <c r="O77" s="15"/>
-      <c r="P77" s="15"/>
-    </row>
-    <row r="78" spans="1:16">
+      <c r="Q77" s="20"/>
+    </row>
+    <row r="78" spans="1:17">
       <c r="A78" s="15" t="s">
         <v>229</v>
       </c>
@@ -11004,8 +10960,8 @@
       <c r="K78" s="15">
         <v>138</v>
       </c>
-      <c r="L78" t="s">
-        <v>334</v>
+      <c r="L78" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M78" s="15">
         <v>1.06</v>
@@ -11013,10 +10969,9 @@
       <c r="N78" s="15">
         <v>0.94</v>
       </c>
-      <c r="O78" s="15"/>
-      <c r="P78" s="15"/>
-    </row>
-    <row r="79" spans="1:16">
+      <c r="Q78" s="20"/>
+    </row>
+    <row r="79" spans="1:17">
       <c r="A79" s="15" t="s">
         <v>230</v>
       </c>
@@ -11048,8 +11003,8 @@
       <c r="K79" s="15">
         <v>138</v>
       </c>
-      <c r="L79" t="s">
-        <v>334</v>
+      <c r="L79" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M79" s="15">
         <v>1.06</v>
@@ -11057,10 +11012,9 @@
       <c r="N79" s="15">
         <v>0.94</v>
       </c>
-      <c r="O79" s="15"/>
-      <c r="P79" s="15"/>
-    </row>
-    <row r="80" spans="1:16">
+      <c r="Q79" s="20"/>
+    </row>
+    <row r="80" spans="1:17">
       <c r="A80" s="15" t="s">
         <v>231</v>
       </c>
@@ -11092,8 +11046,8 @@
       <c r="K80" s="15">
         <v>138</v>
       </c>
-      <c r="L80" t="s">
-        <v>334</v>
+      <c r="L80" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M80" s="15">
         <v>1.06</v>
@@ -11101,10 +11055,9 @@
       <c r="N80" s="15">
         <v>0.94</v>
       </c>
-      <c r="O80" s="15"/>
-      <c r="P80" s="15"/>
-    </row>
-    <row r="81" spans="1:16">
+      <c r="Q80" s="20"/>
+    </row>
+    <row r="81" spans="1:17">
       <c r="A81" s="15" t="s">
         <v>232</v>
       </c>
@@ -11136,8 +11089,8 @@
       <c r="K81" s="15">
         <v>138</v>
       </c>
-      <c r="L81" t="s">
-        <v>334</v>
+      <c r="L81" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M81" s="15">
         <v>1.06</v>
@@ -11145,10 +11098,9 @@
       <c r="N81" s="15">
         <v>0.94</v>
       </c>
-      <c r="O81" s="15"/>
-      <c r="P81" s="15"/>
-    </row>
-    <row r="82" spans="1:16">
+      <c r="Q81" s="20"/>
+    </row>
+    <row r="82" spans="1:17">
       <c r="A82" s="15" t="s">
         <v>233</v>
       </c>
@@ -11180,8 +11132,8 @@
       <c r="K82" s="15">
         <v>345</v>
       </c>
-      <c r="L82" t="s">
-        <v>332</v>
+      <c r="L82" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M82" s="15">
         <v>1.06</v>
@@ -11189,10 +11141,9 @@
       <c r="N82" s="15">
         <v>0.94</v>
       </c>
-      <c r="O82" s="15"/>
-      <c r="P82" s="15"/>
-    </row>
-    <row r="83" spans="1:16">
+      <c r="Q82" s="20"/>
+    </row>
+    <row r="83" spans="1:17">
       <c r="A83" s="15" t="s">
         <v>234</v>
       </c>
@@ -11224,8 +11175,8 @@
       <c r="K83" s="15">
         <v>138</v>
       </c>
-      <c r="L83" t="s">
-        <v>332</v>
+      <c r="L83" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M83" s="15">
         <v>1.06</v>
@@ -11233,10 +11184,9 @@
       <c r="N83" s="15">
         <v>0.94</v>
       </c>
-      <c r="O83" s="15"/>
-      <c r="P83" s="15"/>
-    </row>
-    <row r="84" spans="1:16">
+      <c r="Q83" s="20"/>
+    </row>
+    <row r="84" spans="1:17">
       <c r="A84" s="15" t="s">
         <v>235</v>
       </c>
@@ -11268,8 +11218,8 @@
       <c r="K84" s="15">
         <v>138</v>
       </c>
-      <c r="L84" t="s">
-        <v>332</v>
+      <c r="L84" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M84" s="15">
         <v>1.06</v>
@@ -11277,10 +11227,9 @@
       <c r="N84" s="15">
         <v>0.94</v>
       </c>
-      <c r="O84" s="15"/>
-      <c r="P84" s="15"/>
-    </row>
-    <row r="85" spans="1:16">
+      <c r="Q84" s="20"/>
+    </row>
+    <row r="85" spans="1:17">
       <c r="A85" s="15" t="s">
         <v>236</v>
       </c>
@@ -11312,8 +11261,8 @@
       <c r="K85" s="15">
         <v>138</v>
       </c>
-      <c r="L85" t="s">
-        <v>332</v>
+      <c r="L85" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M85" s="15">
         <v>1.06</v>
@@ -11321,10 +11270,9 @@
       <c r="N85" s="15">
         <v>0.94</v>
       </c>
-      <c r="O85" s="15"/>
-      <c r="P85" s="15"/>
-    </row>
-    <row r="86" spans="1:16">
+      <c r="Q85" s="20"/>
+    </row>
+    <row r="86" spans="1:17">
       <c r="A86" s="15" t="s">
         <v>237</v>
       </c>
@@ -11356,8 +11304,8 @@
       <c r="K86" s="15">
         <v>138</v>
       </c>
-      <c r="L86" t="s">
-        <v>332</v>
+      <c r="L86" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M86" s="15">
         <v>1.06</v>
@@ -11365,10 +11313,9 @@
       <c r="N86" s="15">
         <v>0.94</v>
       </c>
-      <c r="O86" s="15"/>
-      <c r="P86" s="15"/>
-    </row>
-    <row r="87" spans="1:16">
+      <c r="Q86" s="20"/>
+    </row>
+    <row r="87" spans="1:17">
       <c r="A87" s="15" t="s">
         <v>238</v>
       </c>
@@ -11400,8 +11347,8 @@
       <c r="K87" s="15">
         <v>138</v>
       </c>
-      <c r="L87" t="s">
-        <v>332</v>
+      <c r="L87" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M87" s="15">
         <v>1.06</v>
@@ -11409,10 +11356,9 @@
       <c r="N87" s="15">
         <v>0.94</v>
       </c>
-      <c r="O87" s="15"/>
-      <c r="P87" s="15"/>
-    </row>
-    <row r="88" spans="1:16">
+      <c r="Q87" s="20"/>
+    </row>
+    <row r="88" spans="1:17">
       <c r="A88" s="15" t="s">
         <v>239</v>
       </c>
@@ -11444,8 +11390,8 @@
       <c r="K88" s="15">
         <v>161</v>
       </c>
-      <c r="L88" t="s">
-        <v>332</v>
+      <c r="L88" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M88" s="15">
         <v>1.06</v>
@@ -11453,10 +11399,9 @@
       <c r="N88" s="15">
         <v>0.94</v>
       </c>
-      <c r="O88" s="15"/>
-      <c r="P88" s="15"/>
-    </row>
-    <row r="89" spans="1:16">
+      <c r="Q88" s="20"/>
+    </row>
+    <row r="89" spans="1:17">
       <c r="A89" s="15" t="s">
         <v>240</v>
       </c>
@@ -11488,8 +11433,8 @@
       <c r="K89" s="15">
         <v>138</v>
       </c>
-      <c r="L89" t="s">
-        <v>332</v>
+      <c r="L89" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M89" s="15">
         <v>1.06</v>
@@ -11497,10 +11442,9 @@
       <c r="N89" s="15">
         <v>0.94</v>
       </c>
-      <c r="O89" s="15"/>
-      <c r="P89" s="15"/>
-    </row>
-    <row r="90" spans="1:16">
+      <c r="Q89" s="20"/>
+    </row>
+    <row r="90" spans="1:17">
       <c r="A90" s="15" t="s">
         <v>241</v>
       </c>
@@ -11532,8 +11476,8 @@
       <c r="K90" s="15">
         <v>138</v>
       </c>
-      <c r="L90" t="s">
-        <v>332</v>
+      <c r="L90" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M90" s="15">
         <v>1.06</v>
@@ -11541,10 +11485,9 @@
       <c r="N90" s="15">
         <v>0.94</v>
       </c>
-      <c r="O90" s="15"/>
-      <c r="P90" s="15"/>
-    </row>
-    <row r="91" spans="1:16">
+      <c r="Q90" s="20"/>
+    </row>
+    <row r="91" spans="1:17">
       <c r="A91" s="15" t="s">
         <v>242</v>
       </c>
@@ -11576,8 +11519,8 @@
       <c r="K91" s="15">
         <v>138</v>
       </c>
-      <c r="L91" t="s">
-        <v>332</v>
+      <c r="L91" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M91" s="15">
         <v>1.06</v>
@@ -11585,10 +11528,9 @@
       <c r="N91" s="15">
         <v>0.94</v>
       </c>
-      <c r="O91" s="15"/>
-      <c r="P91" s="15"/>
-    </row>
-    <row r="92" spans="1:16">
+      <c r="Q91" s="20"/>
+    </row>
+    <row r="92" spans="1:17">
       <c r="A92" s="15" t="s">
         <v>243</v>
       </c>
@@ -11620,8 +11562,8 @@
       <c r="K92" s="15">
         <v>138</v>
       </c>
-      <c r="L92" t="s">
-        <v>333</v>
+      <c r="L92" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M92" s="15">
         <v>1.06</v>
@@ -11629,10 +11571,9 @@
       <c r="N92" s="15">
         <v>0.94</v>
       </c>
-      <c r="O92" s="15"/>
-      <c r="P92" s="15"/>
-    </row>
-    <row r="93" spans="1:16">
+      <c r="Q92" s="20"/>
+    </row>
+    <row r="93" spans="1:17">
       <c r="A93" s="15" t="s">
         <v>244</v>
       </c>
@@ -11664,8 +11605,8 @@
       <c r="K93" s="15">
         <v>138</v>
       </c>
-      <c r="L93" t="s">
-        <v>333</v>
+      <c r="L93" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M93" s="15">
         <v>1.06</v>
@@ -11673,10 +11614,9 @@
       <c r="N93" s="15">
         <v>0.94</v>
       </c>
-      <c r="O93" s="15"/>
-      <c r="P93" s="15"/>
-    </row>
-    <row r="94" spans="1:16">
+      <c r="Q93" s="20"/>
+    </row>
+    <row r="94" spans="1:17">
       <c r="A94" s="15" t="s">
         <v>245</v>
       </c>
@@ -11708,8 +11648,8 @@
       <c r="K94" s="15">
         <v>138</v>
       </c>
-      <c r="L94" t="s">
-        <v>334</v>
+      <c r="L94" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M94" s="15">
         <v>1.06</v>
@@ -11717,10 +11657,9 @@
       <c r="N94" s="15">
         <v>0.94</v>
       </c>
-      <c r="O94" s="15"/>
-      <c r="P94" s="15"/>
-    </row>
-    <row r="95" spans="1:16">
+      <c r="Q94" s="20"/>
+    </row>
+    <row r="95" spans="1:17">
       <c r="A95" s="15" t="s">
         <v>246</v>
       </c>
@@ -11752,8 +11691,8 @@
       <c r="K95" s="15">
         <v>138</v>
       </c>
-      <c r="L95" t="s">
-        <v>334</v>
+      <c r="L95" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M95" s="15">
         <v>1.06</v>
@@ -11761,10 +11700,9 @@
       <c r="N95" s="15">
         <v>0.94</v>
       </c>
-      <c r="O95" s="15"/>
-      <c r="P95" s="15"/>
-    </row>
-    <row r="96" spans="1:16">
+      <c r="Q95" s="20"/>
+    </row>
+    <row r="96" spans="1:17">
       <c r="A96" s="15" t="s">
         <v>247</v>
       </c>
@@ -11796,8 +11734,8 @@
       <c r="K96" s="15">
         <v>138</v>
       </c>
-      <c r="L96" t="s">
-        <v>334</v>
+      <c r="L96" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M96" s="15">
         <v>1.06</v>
@@ -11805,10 +11743,9 @@
       <c r="N96" s="15">
         <v>0.94</v>
       </c>
-      <c r="O96" s="15"/>
-      <c r="P96" s="15"/>
-    </row>
-    <row r="97" spans="1:16">
+      <c r="Q96" s="20"/>
+    </row>
+    <row r="97" spans="1:17">
       <c r="A97" s="15" t="s">
         <v>248</v>
       </c>
@@ -11840,8 +11777,8 @@
       <c r="K97" s="15">
         <v>138</v>
       </c>
-      <c r="L97" t="s">
-        <v>334</v>
+      <c r="L97" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M97" s="15">
         <v>1.06</v>
@@ -11849,10 +11786,9 @@
       <c r="N97" s="15">
         <v>0.94</v>
       </c>
-      <c r="O97" s="15"/>
-      <c r="P97" s="15"/>
-    </row>
-    <row r="98" spans="1:16">
+      <c r="Q97" s="20"/>
+    </row>
+    <row r="98" spans="1:17">
       <c r="A98" s="15" t="s">
         <v>249</v>
       </c>
@@ -11884,8 +11820,8 @@
       <c r="K98" s="15">
         <v>138</v>
       </c>
-      <c r="L98" t="s">
-        <v>334</v>
+      <c r="L98" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M98" s="15">
         <v>1.06</v>
@@ -11893,10 +11829,9 @@
       <c r="N98" s="15">
         <v>0.94</v>
       </c>
-      <c r="O98" s="15"/>
-      <c r="P98" s="15"/>
-    </row>
-    <row r="99" spans="1:16">
+      <c r="Q98" s="20"/>
+    </row>
+    <row r="99" spans="1:17">
       <c r="A99" s="15" t="s">
         <v>250</v>
       </c>
@@ -11928,8 +11863,8 @@
       <c r="K99" s="15">
         <v>138</v>
       </c>
-      <c r="L99" t="s">
-        <v>334</v>
+      <c r="L99" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M99" s="15">
         <v>1.06</v>
@@ -11937,10 +11872,9 @@
       <c r="N99" s="15">
         <v>0.94</v>
       </c>
-      <c r="O99" s="15"/>
-      <c r="P99" s="15"/>
-    </row>
-    <row r="100" spans="1:16">
+      <c r="Q99" s="20"/>
+    </row>
+    <row r="100" spans="1:17">
       <c r="A100" s="15" t="s">
         <v>251</v>
       </c>
@@ -11972,8 +11906,8 @@
       <c r="K100" s="15">
         <v>138</v>
       </c>
-      <c r="L100" t="s">
-        <v>334</v>
+      <c r="L100" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M100" s="15">
         <v>1.06</v>
@@ -11981,10 +11915,9 @@
       <c r="N100" s="15">
         <v>0.94</v>
       </c>
-      <c r="O100" s="15"/>
-      <c r="P100" s="15"/>
-    </row>
-    <row r="101" spans="1:16">
+      <c r="Q100" s="20"/>
+    </row>
+    <row r="101" spans="1:17">
       <c r="A101" s="15" t="s">
         <v>252</v>
       </c>
@@ -12016,8 +11949,8 @@
       <c r="K101" s="15">
         <v>138</v>
       </c>
-      <c r="L101" t="s">
-        <v>334</v>
+      <c r="L101" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M101" s="15">
         <v>1.06</v>
@@ -12025,10 +11958,9 @@
       <c r="N101" s="15">
         <v>0.94</v>
       </c>
-      <c r="O101" s="15"/>
-      <c r="P101" s="15"/>
-    </row>
-    <row r="102" spans="1:16">
+      <c r="Q101" s="20"/>
+    </row>
+    <row r="102" spans="1:17">
       <c r="A102" s="15" t="s">
         <v>253</v>
       </c>
@@ -12060,8 +11992,8 @@
       <c r="K102" s="15">
         <v>138</v>
       </c>
-      <c r="L102" t="s">
-        <v>334</v>
+      <c r="L102" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M102" s="15">
         <v>1.06</v>
@@ -12069,10 +12001,9 @@
       <c r="N102" s="15">
         <v>0.94</v>
       </c>
-      <c r="O102" s="15"/>
-      <c r="P102" s="15"/>
-    </row>
-    <row r="103" spans="1:16">
+      <c r="Q102" s="20"/>
+    </row>
+    <row r="103" spans="1:17">
       <c r="A103" s="15" t="s">
         <v>254</v>
       </c>
@@ -12104,8 +12035,8 @@
       <c r="K103" s="15">
         <v>138</v>
       </c>
-      <c r="L103" t="s">
-        <v>334</v>
+      <c r="L103" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M103" s="15">
         <v>1.06</v>
@@ -12113,10 +12044,9 @@
       <c r="N103" s="15">
         <v>0.94</v>
       </c>
-      <c r="O103" s="15"/>
-      <c r="P103" s="15"/>
-    </row>
-    <row r="104" spans="1:16">
+      <c r="Q103" s="20"/>
+    </row>
+    <row r="104" spans="1:17">
       <c r="A104" s="15" t="s">
         <v>255</v>
       </c>
@@ -12148,8 +12078,8 @@
       <c r="K104" s="15">
         <v>138</v>
       </c>
-      <c r="L104" t="s">
-        <v>334</v>
+      <c r="L104" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M104" s="15">
         <v>1.06</v>
@@ -12157,10 +12087,9 @@
       <c r="N104" s="15">
         <v>0.94</v>
       </c>
-      <c r="O104" s="15"/>
-      <c r="P104" s="15"/>
-    </row>
-    <row r="105" spans="1:16">
+      <c r="Q104" s="20"/>
+    </row>
+    <row r="105" spans="1:17">
       <c r="A105" s="15" t="s">
         <v>256</v>
       </c>
@@ -12192,8 +12121,8 @@
       <c r="K105" s="15">
         <v>138</v>
       </c>
-      <c r="L105" t="s">
-        <v>334</v>
+      <c r="L105" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M105" s="15">
         <v>1.06</v>
@@ -12201,10 +12130,9 @@
       <c r="N105" s="15">
         <v>0.94</v>
       </c>
-      <c r="O105" s="15"/>
-      <c r="P105" s="15"/>
-    </row>
-    <row r="106" spans="1:16">
+      <c r="Q105" s="20"/>
+    </row>
+    <row r="106" spans="1:17">
       <c r="A106" s="15" t="s">
         <v>257</v>
       </c>
@@ -12236,8 +12164,8 @@
       <c r="K106" s="15">
         <v>138</v>
       </c>
-      <c r="L106" t="s">
-        <v>334</v>
+      <c r="L106" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M106" s="15">
         <v>1.06</v>
@@ -12245,10 +12173,9 @@
       <c r="N106" s="15">
         <v>0.94</v>
       </c>
-      <c r="O106" s="15"/>
-      <c r="P106" s="15"/>
-    </row>
-    <row r="107" spans="1:16">
+      <c r="Q106" s="20"/>
+    </row>
+    <row r="107" spans="1:17">
       <c r="A107" s="15" t="s">
         <v>258</v>
       </c>
@@ -12280,8 +12207,8 @@
       <c r="K107" s="15">
         <v>138</v>
       </c>
-      <c r="L107" t="s">
-        <v>334</v>
+      <c r="L107" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M107" s="15">
         <v>1.06</v>
@@ -12289,10 +12216,9 @@
       <c r="N107" s="15">
         <v>0.94</v>
       </c>
-      <c r="O107" s="15"/>
-      <c r="P107" s="15"/>
-    </row>
-    <row r="108" spans="1:16">
+      <c r="Q107" s="20"/>
+    </row>
+    <row r="108" spans="1:17">
       <c r="A108" s="15" t="s">
         <v>259</v>
       </c>
@@ -12324,8 +12250,8 @@
       <c r="K108" s="15">
         <v>138</v>
       </c>
-      <c r="L108" t="s">
-        <v>334</v>
+      <c r="L108" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M108" s="15">
         <v>1.06</v>
@@ -12333,10 +12259,9 @@
       <c r="N108" s="15">
         <v>0.94</v>
       </c>
-      <c r="O108" s="15"/>
-      <c r="P108" s="15"/>
-    </row>
-    <row r="109" spans="1:16">
+      <c r="Q108" s="20"/>
+    </row>
+    <row r="109" spans="1:17">
       <c r="A109" s="15" t="s">
         <v>260</v>
       </c>
@@ -12368,8 +12293,8 @@
       <c r="K109" s="15">
         <v>138</v>
       </c>
-      <c r="L109" t="s">
-        <v>334</v>
+      <c r="L109" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M109" s="15">
         <v>1.06</v>
@@ -12377,10 +12302,9 @@
       <c r="N109" s="15">
         <v>0.94</v>
       </c>
-      <c r="O109" s="15"/>
-      <c r="P109" s="15"/>
-    </row>
-    <row r="110" spans="1:16">
+      <c r="Q109" s="20"/>
+    </row>
+    <row r="110" spans="1:17">
       <c r="A110" s="15" t="s">
         <v>261</v>
       </c>
@@ -12412,8 +12336,8 @@
       <c r="K110" s="15">
         <v>138</v>
       </c>
-      <c r="L110" t="s">
-        <v>334</v>
+      <c r="L110" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M110" s="15">
         <v>1.06</v>
@@ -12421,10 +12345,9 @@
       <c r="N110" s="15">
         <v>0.94</v>
       </c>
-      <c r="O110" s="15"/>
-      <c r="P110" s="15"/>
-    </row>
-    <row r="111" spans="1:16">
+      <c r="Q110" s="20"/>
+    </row>
+    <row r="111" spans="1:17">
       <c r="A111" s="15" t="s">
         <v>262</v>
       </c>
@@ -12456,8 +12379,8 @@
       <c r="K111" s="15">
         <v>138</v>
       </c>
-      <c r="L111" t="s">
-        <v>334</v>
+      <c r="L111" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M111" s="15">
         <v>1.06</v>
@@ -12465,10 +12388,9 @@
       <c r="N111" s="15">
         <v>0.94</v>
       </c>
-      <c r="O111" s="15"/>
-      <c r="P111" s="15"/>
-    </row>
-    <row r="112" spans="1:16">
+      <c r="Q111" s="20"/>
+    </row>
+    <row r="112" spans="1:17">
       <c r="A112" s="15" t="s">
         <v>263</v>
       </c>
@@ -12500,8 +12422,8 @@
       <c r="K112" s="15">
         <v>138</v>
       </c>
-      <c r="L112" t="s">
-        <v>334</v>
+      <c r="L112" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M112" s="15">
         <v>1.06</v>
@@ -12509,10 +12431,9 @@
       <c r="N112" s="15">
         <v>0.94</v>
       </c>
-      <c r="O112" s="15"/>
-      <c r="P112" s="15"/>
-    </row>
-    <row r="113" spans="1:16">
+      <c r="Q112" s="20"/>
+    </row>
+    <row r="113" spans="1:17">
       <c r="A113" s="15" t="s">
         <v>264</v>
       </c>
@@ -12544,8 +12465,8 @@
       <c r="K113" s="15">
         <v>138</v>
       </c>
-      <c r="L113" t="s">
-        <v>334</v>
+      <c r="L113" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M113" s="15">
         <v>1.06</v>
@@ -12553,10 +12474,9 @@
       <c r="N113" s="15">
         <v>0.94</v>
       </c>
-      <c r="O113" s="15"/>
-      <c r="P113" s="15"/>
-    </row>
-    <row r="114" spans="1:16">
+      <c r="Q113" s="20"/>
+    </row>
+    <row r="114" spans="1:17">
       <c r="A114" s="15" t="s">
         <v>266</v>
       </c>
@@ -12588,8 +12508,8 @@
       <c r="K114" s="15">
         <v>138</v>
       </c>
-      <c r="L114" t="s">
-        <v>332</v>
+      <c r="L114" s="15" t="s">
+        <v>333</v>
       </c>
       <c r="M114" s="15">
         <v>1.06</v>
@@ -12597,10 +12517,9 @@
       <c r="N114" s="15">
         <v>0.94</v>
       </c>
-      <c r="O114" s="15"/>
-      <c r="P114" s="15"/>
-    </row>
-    <row r="115" spans="1:16">
+      <c r="Q114" s="20"/>
+    </row>
+    <row r="115" spans="1:17">
       <c r="A115" s="15" t="s">
         <v>268</v>
       </c>
@@ -12632,8 +12551,8 @@
       <c r="K115" s="15">
         <v>138</v>
       </c>
-      <c r="L115" t="s">
-        <v>332</v>
+      <c r="L115" s="15" t="s">
+        <v>333</v>
       </c>
       <c r="M115" s="15">
         <v>1.06</v>
@@ -12641,10 +12560,9 @@
       <c r="N115" s="15">
         <v>0.94</v>
       </c>
-      <c r="O115" s="15"/>
-      <c r="P115" s="15"/>
-    </row>
-    <row r="116" spans="1:16">
+      <c r="Q115" s="20"/>
+    </row>
+    <row r="116" spans="1:17">
       <c r="A116" s="15" t="s">
         <v>270</v>
       </c>
@@ -12676,8 +12594,8 @@
       <c r="K116" s="15">
         <v>138</v>
       </c>
-      <c r="L116" t="s">
-        <v>332</v>
+      <c r="L116" s="15" t="s">
+        <v>333</v>
       </c>
       <c r="M116" s="15">
         <v>1.06</v>
@@ -12685,10 +12603,9 @@
       <c r="N116" s="15">
         <v>0.94</v>
       </c>
-      <c r="O116" s="15"/>
-      <c r="P116" s="15"/>
-    </row>
-    <row r="117" spans="1:16">
+      <c r="Q116" s="20"/>
+    </row>
+    <row r="117" spans="1:17">
       <c r="A117" s="15" t="s">
         <v>271</v>
       </c>
@@ -12720,8 +12637,8 @@
       <c r="K117" s="15">
         <v>138</v>
       </c>
-      <c r="L117" t="s">
-        <v>332</v>
+      <c r="L117" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M117" s="15">
         <v>1.06</v>
@@ -12729,10 +12646,9 @@
       <c r="N117" s="15">
         <v>0.94</v>
       </c>
-      <c r="O117" s="15"/>
-      <c r="P117" s="15"/>
-    </row>
-    <row r="118" spans="1:16">
+      <c r="Q117" s="20"/>
+    </row>
+    <row r="118" spans="1:17">
       <c r="A118" s="15" t="s">
         <v>273</v>
       </c>
@@ -12764,8 +12680,8 @@
       <c r="K118" s="15">
         <v>138</v>
       </c>
-      <c r="L118" t="s">
-        <v>333</v>
+      <c r="L118" s="15" t="s">
+        <v>332</v>
       </c>
       <c r="M118" s="15">
         <v>1.06</v>
@@ -12773,10 +12689,9 @@
       <c r="N118" s="15">
         <v>0.94</v>
       </c>
-      <c r="O118" s="15"/>
-      <c r="P118" s="15"/>
-    </row>
-    <row r="119" spans="1:16">
+      <c r="Q118" s="20"/>
+    </row>
+    <row r="119" spans="1:17">
       <c r="A119" s="15" t="s">
         <v>274</v>
       </c>
@@ -12808,8 +12723,8 @@
       <c r="K119" s="15">
         <v>138</v>
       </c>
-      <c r="L119" t="s">
-        <v>332</v>
+      <c r="L119" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M119" s="15">
         <v>1.06</v>
@@ -12817,11 +12732,70 @@
       <c r="N119" s="15">
         <v>0.94</v>
       </c>
-      <c r="O119" s="15"/>
-      <c r="P119" s="15"/>
+      <c r="Q119" s="20"/>
+    </row>
+    <row r="130" spans="17:17" ht="23.25">
+      <c r="Q130" s="21"/>
+    </row>
+    <row r="131" spans="17:17">
+      <c r="Q131" s="22"/>
+    </row>
+    <row r="132" spans="17:17">
+      <c r="Q132" s="22"/>
+    </row>
+    <row r="133" spans="17:17">
+      <c r="Q133" s="22"/>
+    </row>
+    <row r="134" spans="17:17">
+      <c r="Q134" s="22"/>
+    </row>
+    <row r="135" spans="17:17">
+      <c r="Q135" s="22"/>
+    </row>
+    <row r="136" spans="17:17">
+      <c r="Q136" s="22"/>
+    </row>
+    <row r="137" spans="17:17">
+      <c r="Q137" s="22"/>
+    </row>
+    <row r="138" spans="17:17">
+      <c r="Q138" s="22"/>
+    </row>
+    <row r="139" spans="17:17">
+      <c r="Q139" s="22"/>
+    </row>
+    <row r="140" spans="17:17">
+      <c r="Q140" s="22"/>
+    </row>
+    <row r="143" spans="17:17">
+      <c r="Q143" s="22"/>
+    </row>
+    <row r="144" spans="17:17">
+      <c r="Q144" s="22"/>
+    </row>
+    <row r="145" spans="17:17">
+      <c r="Q145" s="22"/>
+    </row>
+    <row r="146" spans="17:17">
+      <c r="Q146" s="22"/>
+    </row>
+    <row r="147" spans="17:17">
+      <c r="Q147" s="22"/>
+    </row>
+    <row r="148" spans="17:17">
+      <c r="Q148" s="22"/>
+    </row>
+    <row r="149" spans="17:17">
+      <c r="Q149" s="22"/>
+    </row>
+    <row r="150" spans="17:17">
+      <c r="Q150" s="22"/>
+    </row>
+    <row r="152" spans="17:17">
+      <c r="Q152" s="23"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="6" type="noConversion"/>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
add dc lines, transformers, and parallel processing (#73)
</commit_message>
<xml_diff>
--- a/test/inputs/case118/case118.xlsx
+++ b/test/inputs/case118/case118.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nomyk\Desktop\Network Reduction Model\NetworkReduction.jl\test\inputs\case118\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{529FD465-F4B0-4217-AB4C-5A3279106415}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D02B6407-E370-4E89-9E9F-B95C3D4D8089}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1015" uniqueCount="337">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1015" uniqueCount="338">
   <si>
     <t>Line_name</t>
   </si>
@@ -1050,6 +1050,9 @@
   </si>
   <si>
     <t>IsRepresentative</t>
+  </si>
+  <si>
+    <t>Z4</t>
   </si>
 </sst>
 </file>
@@ -1059,7 +1062,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1094,11 +1097,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
-      <name val="Segoe UI"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -1107,6 +1105,27 @@
     <font>
       <sz val="11"/>
       <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1194,12 +1213,13 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1"/>
@@ -1220,14 +1240,24 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="7" fillId="2" borderId="0" xfId="2" applyNumberFormat="1"/>
-    <xf numFmtId="2" fontId="7" fillId="2" borderId="4" xfId="2" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="6" fillId="2" borderId="0" xfId="2" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="6" fillId="2" borderId="4" xfId="2" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="3"/>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="4">
     <cellStyle name="Good" xfId="2" builtinId="26"/>
+    <cellStyle name="Hyperlink" xfId="3" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Standard 2" xfId="1" xr:uid="{4781E190-0CBC-4ACB-9E92-DBE0057C370D}"/>
   </cellStyles>
@@ -1567,7 +1597,7 @@
       <c r="D2" s="12" t="s">
         <v>276</v>
       </c>
-      <c r="E2" s="17">
+      <c r="E2" s="16">
         <v>138</v>
       </c>
       <c r="F2" s="10">
@@ -1599,7 +1629,7 @@
       <c r="D3" s="10" t="s">
         <v>277</v>
       </c>
-      <c r="E3" s="18">
+      <c r="E3" s="17">
         <v>138</v>
       </c>
       <c r="F3" s="10">
@@ -1631,7 +1661,7 @@
       <c r="D4" s="10" t="s">
         <v>279</v>
       </c>
-      <c r="E4" s="18">
+      <c r="E4" s="17">
         <v>138</v>
       </c>
       <c r="F4" s="10">
@@ -1663,7 +1693,7 @@
       <c r="D5" s="10" t="s">
         <v>279</v>
       </c>
-      <c r="E5" s="18">
+      <c r="E5" s="17">
         <v>138</v>
       </c>
       <c r="F5" s="10">
@@ -1695,7 +1725,7 @@
       <c r="D6" s="10" t="s">
         <v>280</v>
       </c>
-      <c r="E6" s="18">
+      <c r="E6" s="17">
         <v>138</v>
       </c>
       <c r="F6" s="10">
@@ -1727,7 +1757,7 @@
       <c r="D7" s="10" t="s">
         <v>281</v>
       </c>
-      <c r="E7" s="18">
+      <c r="E7" s="17">
         <v>138</v>
       </c>
       <c r="F7" s="10">
@@ -1759,7 +1789,7 @@
       <c r="D8" s="10" t="s">
         <v>283</v>
       </c>
-      <c r="E8" s="18">
+      <c r="E8" s="17">
         <v>345</v>
       </c>
       <c r="F8" s="10">
@@ -1791,19 +1821,19 @@
       <c r="D9" s="10" t="s">
         <v>279</v>
       </c>
-      <c r="E9" s="18">
+      <c r="E9" s="17">
         <v>345</v>
       </c>
       <c r="F9" s="10">
         <v>1506.1311370164149</v>
       </c>
-      <c r="G9" s="19">
+      <c r="G9" s="18">
         <v>0</v>
       </c>
       <c r="H9" s="13">
         <v>31.779675000000001</v>
       </c>
-      <c r="I9" s="20">
+      <c r="I9" s="19">
         <v>0</v>
       </c>
       <c r="J9" s="13">
@@ -1823,7 +1853,7 @@
       <c r="D10" s="10" t="s">
         <v>284</v>
       </c>
-      <c r="E10" s="18">
+      <c r="E10" s="17">
         <v>345</v>
       </c>
       <c r="F10" s="10">
@@ -1855,7 +1885,7 @@
       <c r="D11" s="10" t="s">
         <v>285</v>
       </c>
-      <c r="E11" s="18">
+      <c r="E11" s="17">
         <v>138</v>
       </c>
       <c r="F11" s="10">
@@ -1887,7 +1917,7 @@
       <c r="D12" s="10" t="s">
         <v>285</v>
       </c>
-      <c r="E12" s="18">
+      <c r="E12" s="17">
         <v>138</v>
       </c>
       <c r="F12" s="10">
@@ -1919,7 +1949,7 @@
       <c r="D13" s="10" t="s">
         <v>272</v>
       </c>
-      <c r="E13" s="18">
+      <c r="E13" s="17">
         <v>138</v>
       </c>
       <c r="F13" s="10">
@@ -1951,7 +1981,7 @@
       <c r="D14" s="10" t="s">
         <v>272</v>
       </c>
-      <c r="E14" s="18">
+      <c r="E14" s="17">
         <v>138</v>
       </c>
       <c r="F14" s="10">
@@ -1983,7 +2013,7 @@
       <c r="D15" s="10" t="s">
         <v>272</v>
       </c>
-      <c r="E15" s="18">
+      <c r="E15" s="17">
         <v>138</v>
       </c>
       <c r="F15" s="10">
@@ -2015,7 +2045,7 @@
       <c r="D16" s="10" t="s">
         <v>272</v>
       </c>
-      <c r="E16" s="18">
+      <c r="E16" s="17">
         <v>138</v>
       </c>
       <c r="F16" s="10">
@@ -2047,7 +2077,7 @@
       <c r="D17" s="10" t="s">
         <v>286</v>
       </c>
-      <c r="E17" s="18">
+      <c r="E17" s="17">
         <v>138</v>
       </c>
       <c r="F17" s="10">
@@ -2079,7 +2109,7 @@
       <c r="D18" s="10" t="s">
         <v>287</v>
       </c>
-      <c r="E18" s="18">
+      <c r="E18" s="17">
         <v>138</v>
       </c>
       <c r="F18" s="10">
@@ -2111,7 +2141,7 @@
       <c r="D19" s="10" t="s">
         <v>288</v>
       </c>
-      <c r="E19" s="18">
+      <c r="E19" s="17">
         <v>138</v>
       </c>
       <c r="F19" s="10">
@@ -2143,7 +2173,7 @@
       <c r="D20" s="10" t="s">
         <v>288</v>
       </c>
-      <c r="E20" s="18">
+      <c r="E20" s="17">
         <v>138</v>
       </c>
       <c r="F20" s="10">
@@ -2175,7 +2205,7 @@
       <c r="D21" s="10" t="s">
         <v>289</v>
       </c>
-      <c r="E21" s="18">
+      <c r="E21" s="17">
         <v>138</v>
       </c>
       <c r="F21" s="10">
@@ -2207,7 +2237,7 @@
       <c r="D22" s="10" t="s">
         <v>265</v>
       </c>
-      <c r="E22" s="18">
+      <c r="E22" s="17">
         <v>138</v>
       </c>
       <c r="F22" s="10">
@@ -2239,7 +2269,7 @@
       <c r="D23" s="10" t="s">
         <v>265</v>
       </c>
-      <c r="E23" s="18">
+      <c r="E23" s="17">
         <v>138</v>
       </c>
       <c r="F23" s="10">
@@ -2271,7 +2301,7 @@
       <c r="D24" s="10" t="s">
         <v>290</v>
       </c>
-      <c r="E24" s="18">
+      <c r="E24" s="17">
         <v>138</v>
       </c>
       <c r="F24" s="10">
@@ -2303,7 +2333,7 @@
       <c r="D25" s="10" t="s">
         <v>291</v>
       </c>
-      <c r="E25" s="18">
+      <c r="E25" s="17">
         <v>138</v>
       </c>
       <c r="F25" s="10">
@@ -2335,7 +2365,7 @@
       <c r="D26" s="10" t="s">
         <v>292</v>
       </c>
-      <c r="E26" s="18">
+      <c r="E26" s="17">
         <v>138</v>
       </c>
       <c r="F26" s="10">
@@ -2367,7 +2397,7 @@
       <c r="D27" s="10" t="s">
         <v>291</v>
       </c>
-      <c r="E27" s="18">
+      <c r="E27" s="17">
         <v>138</v>
       </c>
       <c r="F27" s="10">
@@ -2399,7 +2429,7 @@
       <c r="D28" s="10" t="s">
         <v>293</v>
       </c>
-      <c r="E28" s="18">
+      <c r="E28" s="17">
         <v>138</v>
       </c>
       <c r="F28" s="10">
@@ -2431,7 +2461,7 @@
       <c r="D29" s="10" t="s">
         <v>294</v>
       </c>
-      <c r="E29" s="18">
+      <c r="E29" s="17">
         <v>138</v>
       </c>
       <c r="F29" s="10">
@@ -2463,7 +2493,7 @@
       <c r="D30" s="10" t="s">
         <v>295</v>
       </c>
-      <c r="E30" s="18">
+      <c r="E30" s="17">
         <v>138</v>
       </c>
       <c r="F30" s="10">
@@ -2495,7 +2525,7 @@
       <c r="D31" s="10" t="s">
         <v>222</v>
       </c>
-      <c r="E31" s="18">
+      <c r="E31" s="17">
         <v>138</v>
       </c>
       <c r="F31" s="10">
@@ -2527,7 +2557,7 @@
       <c r="D32" s="10" t="s">
         <v>296</v>
       </c>
-      <c r="E32" s="18">
+      <c r="E32" s="17">
         <v>138</v>
       </c>
       <c r="F32" s="10">
@@ -2559,19 +2589,19 @@
       <c r="D33" s="10" t="s">
         <v>296</v>
       </c>
-      <c r="E33" s="18">
+      <c r="E33" s="17">
         <v>345</v>
       </c>
       <c r="F33" s="10">
         <v>920.41347262114243</v>
       </c>
-      <c r="G33" s="19">
+      <c r="G33" s="18">
         <v>0</v>
       </c>
       <c r="H33" s="13">
         <v>45.467550000000003</v>
       </c>
-      <c r="I33" s="20">
+      <c r="I33" s="19">
         <v>0</v>
       </c>
       <c r="J33" s="13">
@@ -2591,7 +2621,7 @@
       <c r="D34" s="10" t="s">
         <v>269</v>
       </c>
-      <c r="E34" s="18">
+      <c r="E34" s="17">
         <v>138</v>
       </c>
       <c r="F34" s="10">
@@ -2623,7 +2653,7 @@
       <c r="D35" s="10" t="s">
         <v>298</v>
       </c>
-      <c r="E35" s="18">
+      <c r="E35" s="17">
         <v>138</v>
       </c>
       <c r="F35" s="10">
@@ -2655,7 +2685,7 @@
       <c r="D36" s="10" t="s">
         <v>299</v>
       </c>
-      <c r="E36" s="18">
+      <c r="E36" s="17">
         <v>138</v>
       </c>
       <c r="F36" s="10">
@@ -2687,19 +2717,19 @@
       <c r="D37" s="10" t="s">
         <v>265</v>
       </c>
-      <c r="E37" s="18">
+      <c r="E37" s="17">
         <v>345</v>
       </c>
       <c r="F37" s="10">
         <v>920.41347262114243</v>
       </c>
-      <c r="G37" s="19">
+      <c r="G37" s="18">
         <v>0</v>
       </c>
       <c r="H37" s="13">
         <v>46.181699999999999</v>
       </c>
-      <c r="I37" s="20">
+      <c r="I37" s="19">
         <v>0</v>
       </c>
       <c r="J37" s="13">
@@ -2719,7 +2749,7 @@
       <c r="D38" s="10" t="s">
         <v>300</v>
       </c>
-      <c r="E38" s="18">
+      <c r="E38" s="17">
         <v>345</v>
       </c>
       <c r="F38" s="10">
@@ -2751,7 +2781,7 @@
       <c r="D39" s="10" t="s">
         <v>300</v>
       </c>
-      <c r="E39" s="18">
+      <c r="E39" s="17">
         <v>345</v>
       </c>
       <c r="F39" s="10">
@@ -2783,7 +2813,7 @@
       <c r="D40" s="10" t="s">
         <v>301</v>
       </c>
-      <c r="E40" s="18">
+      <c r="E40" s="17">
         <v>138</v>
       </c>
       <c r="F40" s="10">
@@ -2815,7 +2845,7 @@
       <c r="D41" s="10" t="s">
         <v>301</v>
       </c>
-      <c r="E41" s="18">
+      <c r="E41" s="17">
         <v>138</v>
       </c>
       <c r="F41" s="10">
@@ -2847,7 +2877,7 @@
       <c r="D42" s="10" t="s">
         <v>267</v>
       </c>
-      <c r="E42" s="18">
+      <c r="E42" s="17">
         <v>138</v>
       </c>
       <c r="F42" s="10">
@@ -2879,7 +2909,7 @@
       <c r="D43" s="10" t="s">
         <v>267</v>
       </c>
-      <c r="E43" s="18">
+      <c r="E43" s="17">
         <v>138</v>
       </c>
       <c r="F43" s="10">
@@ -2911,7 +2941,7 @@
       <c r="D44" s="10" t="s">
         <v>267</v>
       </c>
-      <c r="E44" s="18">
+      <c r="E44" s="17">
         <v>138</v>
       </c>
       <c r="F44" s="10">
@@ -2943,7 +2973,7 @@
       <c r="D45" s="10" t="s">
         <v>302</v>
       </c>
-      <c r="E45" s="18">
+      <c r="E45" s="17">
         <v>138</v>
       </c>
       <c r="F45" s="10">
@@ -2975,7 +3005,7 @@
       <c r="D46" s="10" t="s">
         <v>303</v>
       </c>
-      <c r="E46" s="18">
+      <c r="E46" s="17">
         <v>138</v>
       </c>
       <c r="F46" s="10">
@@ -3007,7 +3037,7 @@
       <c r="D47" s="10" t="s">
         <v>305</v>
       </c>
-      <c r="E47" s="18">
+      <c r="E47" s="17">
         <v>138</v>
       </c>
       <c r="F47" s="10">
@@ -3039,7 +3069,7 @@
       <c r="D48" s="10" t="s">
         <v>306</v>
       </c>
-      <c r="E48" s="18">
+      <c r="E48" s="17">
         <v>138</v>
       </c>
       <c r="F48" s="10">
@@ -3071,7 +3101,7 @@
       <c r="D49" s="10" t="s">
         <v>306</v>
       </c>
-      <c r="E49" s="18">
+      <c r="E49" s="17">
         <v>138</v>
       </c>
       <c r="F49" s="10">
@@ -3103,7 +3133,7 @@
       <c r="D50" s="10" t="s">
         <v>305</v>
       </c>
-      <c r="E50" s="18">
+      <c r="E50" s="17">
         <v>138</v>
       </c>
       <c r="F50" s="10">
@@ -3135,7 +3165,7 @@
       <c r="D51" s="10" t="s">
         <v>306</v>
       </c>
-      <c r="E51" s="18">
+      <c r="E51" s="17">
         <v>138</v>
       </c>
       <c r="F51" s="10">
@@ -3167,19 +3197,19 @@
       <c r="D52" s="10" t="s">
         <v>306</v>
       </c>
-      <c r="E52" s="18">
+      <c r="E52" s="17">
         <v>345</v>
       </c>
       <c r="F52" s="10">
         <v>920.41347262114243</v>
       </c>
-      <c r="G52" s="19">
+      <c r="G52" s="18">
         <v>0</v>
       </c>
       <c r="H52" s="13">
         <v>44.634374999999999</v>
       </c>
-      <c r="I52" s="20">
+      <c r="I52" s="19">
         <v>0</v>
       </c>
       <c r="J52" s="13">
@@ -3199,7 +3229,7 @@
       <c r="D53" s="10" t="s">
         <v>308</v>
       </c>
-      <c r="E53" s="18">
+      <c r="E53" s="17">
         <v>138</v>
       </c>
       <c r="F53" s="10">
@@ -3231,7 +3261,7 @@
       <c r="D54" s="10" t="s">
         <v>309</v>
       </c>
-      <c r="E54" s="18">
+      <c r="E54" s="17">
         <v>138</v>
       </c>
       <c r="F54" s="10">
@@ -3263,7 +3293,7 @@
       <c r="D55" s="10" t="s">
         <v>307</v>
       </c>
-      <c r="E55" s="18">
+      <c r="E55" s="17">
         <v>345</v>
       </c>
       <c r="F55" s="10">
@@ -3295,7 +3325,7 @@
       <c r="D56" s="10" t="s">
         <v>309</v>
       </c>
-      <c r="E56" s="18">
+      <c r="E56" s="17">
         <v>138</v>
       </c>
       <c r="F56" s="10">
@@ -3327,7 +3357,7 @@
       <c r="D57" s="10" t="s">
         <v>310</v>
       </c>
-      <c r="E57" s="18">
+      <c r="E57" s="17">
         <v>138</v>
       </c>
       <c r="F57" s="10">
@@ -3359,7 +3389,7 @@
       <c r="D58" s="10" t="s">
         <v>311</v>
       </c>
-      <c r="E58" s="18">
+      <c r="E58" s="17">
         <v>138</v>
       </c>
       <c r="F58" s="10">
@@ -3391,7 +3421,7 @@
       <c r="D59" s="10" t="s">
         <v>311</v>
       </c>
-      <c r="E59" s="18">
+      <c r="E59" s="17">
         <v>138</v>
       </c>
       <c r="F59" s="10">
@@ -3423,7 +3453,7 @@
       <c r="D60" s="10" t="s">
         <v>313</v>
       </c>
-      <c r="E60" s="18">
+      <c r="E60" s="17">
         <v>138</v>
       </c>
       <c r="F60" s="10">
@@ -3455,7 +3485,7 @@
       <c r="D61" s="10" t="s">
         <v>312</v>
       </c>
-      <c r="E61" s="18">
+      <c r="E61" s="17">
         <v>138</v>
       </c>
       <c r="F61" s="10">
@@ -3487,7 +3517,7 @@
       <c r="D62" s="10" t="s">
         <v>314</v>
       </c>
-      <c r="E62" s="18">
+      <c r="E62" s="17">
         <v>138</v>
       </c>
       <c r="F62" s="10">
@@ -3519,7 +3549,7 @@
       <c r="D63" s="10" t="s">
         <v>315</v>
       </c>
-      <c r="E63" s="18">
+      <c r="E63" s="17">
         <v>138</v>
       </c>
       <c r="F63" s="10">
@@ -3551,7 +3581,7 @@
       <c r="D64" s="10" t="s">
         <v>218</v>
       </c>
-      <c r="E64" s="18">
+      <c r="E64" s="17">
         <v>138</v>
       </c>
       <c r="F64" s="10">
@@ -3583,7 +3613,7 @@
       <c r="D65" s="10" t="s">
         <v>316</v>
       </c>
-      <c r="E65" s="18">
+      <c r="E65" s="17">
         <v>138</v>
       </c>
       <c r="F65" s="10">
@@ -3615,7 +3645,7 @@
       <c r="D66" s="10" t="s">
         <v>220</v>
       </c>
-      <c r="E66" s="18">
+      <c r="E66" s="17">
         <v>138</v>
       </c>
       <c r="F66" s="10">
@@ -3647,7 +3677,7 @@
       <c r="D67" s="10" t="s">
         <v>220</v>
       </c>
-      <c r="E67" s="18">
+      <c r="E67" s="17">
         <v>138</v>
       </c>
       <c r="F67" s="10">
@@ -3679,7 +3709,7 @@
       <c r="D68" s="10" t="s">
         <v>220</v>
       </c>
-      <c r="E68" s="18">
+      <c r="E68" s="17">
         <v>138</v>
       </c>
       <c r="F68" s="10">
@@ -3711,7 +3741,7 @@
       <c r="D69" s="10" t="s">
         <v>220</v>
       </c>
-      <c r="E69" s="18">
+      <c r="E69" s="17">
         <v>138</v>
       </c>
       <c r="F69" s="10">
@@ -3743,7 +3773,7 @@
       <c r="D70" s="10" t="s">
         <v>220</v>
       </c>
-      <c r="E70" s="18">
+      <c r="E70" s="17">
         <v>138</v>
       </c>
       <c r="F70" s="10">
@@ -3775,7 +3805,7 @@
       <c r="D71" s="10" t="s">
         <v>317</v>
       </c>
-      <c r="E71" s="18">
+      <c r="E71" s="17">
         <v>138</v>
       </c>
       <c r="F71" s="10">
@@ -3807,7 +3837,7 @@
       <c r="D72" s="10" t="s">
         <v>318</v>
       </c>
-      <c r="E72" s="18">
+      <c r="E72" s="17">
         <v>138</v>
       </c>
       <c r="F72" s="10">
@@ -3839,7 +3869,7 @@
       <c r="D73" s="10" t="s">
         <v>319</v>
       </c>
-      <c r="E73" s="18">
+      <c r="E73" s="17">
         <v>138</v>
       </c>
       <c r="F73" s="10">
@@ -3871,7 +3901,7 @@
       <c r="D74" s="10" t="s">
         <v>320</v>
       </c>
-      <c r="E74" s="18">
+      <c r="E74" s="17">
         <v>138</v>
       </c>
       <c r="F74" s="10">
@@ -3903,7 +3933,7 @@
       <c r="D75" s="10" t="s">
         <v>321</v>
       </c>
-      <c r="E75" s="18">
+      <c r="E75" s="17">
         <v>138</v>
       </c>
       <c r="F75" s="10">
@@ -3935,7 +3965,7 @@
       <c r="D76" s="10" t="s">
         <v>321</v>
       </c>
-      <c r="E76" s="18">
+      <c r="E76" s="17">
         <v>138</v>
       </c>
       <c r="F76" s="10">
@@ -3967,7 +3997,7 @@
       <c r="D77" s="10" t="s">
         <v>321</v>
       </c>
-      <c r="E77" s="18">
+      <c r="E77" s="17">
         <v>138</v>
       </c>
       <c r="F77" s="10">
@@ -3999,7 +4029,7 @@
       <c r="D78" s="10" t="s">
         <v>322</v>
       </c>
-      <c r="E78" s="18">
+      <c r="E78" s="17">
         <v>138</v>
       </c>
       <c r="F78" s="10">
@@ -4031,7 +4061,7 @@
       <c r="D79" s="10" t="s">
         <v>323</v>
       </c>
-      <c r="E79" s="18">
+      <c r="E79" s="17">
         <v>138</v>
       </c>
       <c r="F79" s="10">
@@ -4063,7 +4093,7 @@
       <c r="D80" s="10" t="s">
         <v>323</v>
       </c>
-      <c r="E80" s="18">
+      <c r="E80" s="17">
         <v>138</v>
       </c>
       <c r="F80" s="10">
@@ -4095,7 +4125,7 @@
       <c r="D81" s="10" t="s">
         <v>324</v>
       </c>
-      <c r="E81" s="18">
+      <c r="E81" s="17">
         <v>138</v>
       </c>
       <c r="F81" s="10">
@@ -4127,7 +4157,7 @@
       <c r="D82" s="10" t="s">
         <v>324</v>
       </c>
-      <c r="E82" s="18">
+      <c r="E82" s="17">
         <v>138</v>
       </c>
       <c r="F82" s="10">
@@ -4159,7 +4189,7 @@
       <c r="D83" s="10" t="s">
         <v>325</v>
       </c>
-      <c r="E83" s="18">
+      <c r="E83" s="17">
         <v>138</v>
       </c>
       <c r="F83" s="10">
@@ -4191,7 +4221,7 @@
       <c r="D84" s="10" t="s">
         <v>325</v>
       </c>
-      <c r="E84" s="18">
+      <c r="E84" s="17">
         <v>138</v>
       </c>
       <c r="F84" s="10">
@@ -4223,7 +4253,7 @@
       <c r="D85" s="10" t="s">
         <v>326</v>
       </c>
-      <c r="E85" s="18">
+      <c r="E85" s="17">
         <v>138</v>
       </c>
       <c r="F85" s="10">
@@ -4255,7 +4285,7 @@
       <c r="D86" s="10" t="s">
         <v>326</v>
       </c>
-      <c r="E86" s="18">
+      <c r="E86" s="17">
         <v>138</v>
       </c>
       <c r="F86" s="10">
@@ -4287,7 +4317,7 @@
       <c r="D87" s="10" t="s">
         <v>326</v>
       </c>
-      <c r="E87" s="18">
+      <c r="E87" s="17">
         <v>138</v>
       </c>
       <c r="F87" s="10">
@@ -4319,7 +4349,7 @@
       <c r="D88" s="10" t="s">
         <v>326</v>
       </c>
-      <c r="E88" s="18">
+      <c r="E88" s="17">
         <v>138</v>
       </c>
       <c r="F88" s="10">
@@ -4351,7 +4381,7 @@
       <c r="D89" s="10" t="s">
         <v>327</v>
       </c>
-      <c r="E89" s="18">
+      <c r="E89" s="17">
         <v>138</v>
       </c>
       <c r="F89" s="10">
@@ -4383,7 +4413,7 @@
       <c r="D90" s="10" t="s">
         <v>328</v>
       </c>
-      <c r="E90" s="18">
+      <c r="E90" s="17">
         <v>138</v>
       </c>
       <c r="F90" s="10">
@@ -4415,7 +4445,7 @@
       <c r="D91" s="10" t="s">
         <v>328</v>
       </c>
-      <c r="E91" s="18">
+      <c r="E91" s="17">
         <v>138</v>
       </c>
       <c r="F91" s="10">
@@ -4447,7 +4477,7 @@
       <c r="D92" s="10" t="s">
         <v>213</v>
       </c>
-      <c r="E92" s="18">
+      <c r="E92" s="17">
         <v>138</v>
       </c>
       <c r="F92" s="10">
@@ -4479,7 +4509,7 @@
       <c r="D93" s="10" t="s">
         <v>213</v>
       </c>
-      <c r="E93" s="18">
+      <c r="E93" s="17">
         <v>138</v>
       </c>
       <c r="F93" s="10">
@@ -4511,19 +4541,19 @@
       <c r="D94" s="10" t="s">
         <v>326</v>
       </c>
-      <c r="E94" s="18">
+      <c r="E94" s="17">
         <v>345</v>
       </c>
       <c r="F94" s="10">
         <v>920.41347262114243</v>
       </c>
-      <c r="G94" s="19">
+      <c r="G94" s="18">
         <v>0</v>
       </c>
       <c r="H94" s="13">
         <v>45.943650000000005</v>
       </c>
-      <c r="I94" s="20">
+      <c r="I94" s="19">
         <v>0</v>
       </c>
       <c r="J94" s="13">
@@ -4543,7 +4573,7 @@
       <c r="D95" s="10" t="s">
         <v>330</v>
       </c>
-      <c r="E95" s="18">
+      <c r="E95" s="17">
         <v>345</v>
       </c>
       <c r="F95" s="10">
@@ -4575,19 +4605,19 @@
       <c r="D96" s="10" t="s">
         <v>328</v>
       </c>
-      <c r="E96" s="18">
+      <c r="E96" s="17">
         <v>345</v>
       </c>
       <c r="F96" s="10">
         <v>920.41347262114243</v>
       </c>
-      <c r="G96" s="19">
+      <c r="G96" s="18">
         <v>0</v>
       </c>
       <c r="H96" s="13">
         <v>31.898699999999998</v>
       </c>
-      <c r="I96" s="20">
+      <c r="I96" s="19">
         <v>0</v>
       </c>
       <c r="J96" s="13">
@@ -4607,7 +4637,7 @@
       <c r="D97" s="10" t="s">
         <v>216</v>
       </c>
-      <c r="E97" s="18">
+      <c r="E97" s="17">
         <v>345</v>
       </c>
       <c r="F97" s="10">
@@ -4639,7 +4669,7 @@
       <c r="D98" s="10" t="s">
         <v>216</v>
       </c>
-      <c r="E98" s="18">
+      <c r="E98" s="17">
         <v>345</v>
       </c>
       <c r="F98" s="10">
@@ -4671,7 +4701,7 @@
       <c r="D99" s="10" t="s">
         <v>214</v>
       </c>
-      <c r="E99" s="18">
+      <c r="E99" s="17">
         <v>138</v>
       </c>
       <c r="F99" s="10">
@@ -4703,7 +4733,7 @@
       <c r="D100" s="10" t="s">
         <v>214</v>
       </c>
-      <c r="E100" s="18">
+      <c r="E100" s="17">
         <v>138</v>
       </c>
       <c r="F100" s="10">
@@ -4735,7 +4765,7 @@
       <c r="D101" s="10" t="s">
         <v>214</v>
       </c>
-      <c r="E101" s="18">
+      <c r="E101" s="17">
         <v>138</v>
       </c>
       <c r="F101" s="10">
@@ -4767,7 +4797,7 @@
       <c r="D102" s="10" t="s">
         <v>215</v>
       </c>
-      <c r="E102" s="18">
+      <c r="E102" s="17">
         <v>138</v>
       </c>
       <c r="F102" s="10">
@@ -4799,19 +4829,19 @@
       <c r="D103" s="10" t="s">
         <v>214</v>
       </c>
-      <c r="E103" s="18">
+      <c r="E103" s="17">
         <v>345</v>
       </c>
       <c r="F103" s="10">
         <v>1506.1311370164149</v>
       </c>
-      <c r="G103" s="19">
+      <c r="G103" s="18">
         <v>0</v>
       </c>
       <c r="H103" s="13">
         <v>44.039250000000003</v>
       </c>
-      <c r="I103" s="20">
+      <c r="I103" s="19">
         <v>0</v>
       </c>
       <c r="J103" s="13">
@@ -4831,7 +4861,7 @@
       <c r="D104" s="10" t="s">
         <v>215</v>
       </c>
-      <c r="E104" s="18">
+      <c r="E104" s="17">
         <v>138</v>
       </c>
       <c r="F104" s="10">
@@ -4863,7 +4893,7 @@
       <c r="D105" s="10" t="s">
         <v>217</v>
       </c>
-      <c r="E105" s="18">
+      <c r="E105" s="17">
         <v>345</v>
       </c>
       <c r="F105" s="10">
@@ -4895,7 +4925,7 @@
       <c r="D106" s="10" t="s">
         <v>219</v>
       </c>
-      <c r="E106" s="18">
+      <c r="E106" s="17">
         <v>138</v>
       </c>
       <c r="F106" s="10">
@@ -4927,7 +4957,7 @@
       <c r="D107" s="10" t="s">
         <v>219</v>
       </c>
-      <c r="E107" s="18">
+      <c r="E107" s="17">
         <v>138</v>
       </c>
       <c r="F107" s="10">
@@ -4959,19 +4989,19 @@
       <c r="D108" s="10" t="s">
         <v>219</v>
       </c>
-      <c r="E108" s="18">
+      <c r="E108" s="17">
         <v>345</v>
       </c>
       <c r="F108" s="10">
         <v>1506.1311370164149</v>
       </c>
-      <c r="G108" s="19">
+      <c r="G108" s="18">
         <v>0</v>
       </c>
       <c r="H108" s="13">
         <v>44.039250000000003</v>
       </c>
-      <c r="I108" s="20">
+      <c r="I108" s="19">
         <v>0</v>
       </c>
       <c r="J108" s="13">
@@ -4991,7 +5021,7 @@
       <c r="D109" s="10" t="s">
         <v>221</v>
       </c>
-      <c r="E109" s="18">
+      <c r="E109" s="17">
         <v>138</v>
       </c>
       <c r="F109" s="10">
@@ -5023,7 +5053,7 @@
       <c r="D110" s="10" t="s">
         <v>221</v>
       </c>
-      <c r="E110" s="18">
+      <c r="E110" s="17">
         <v>138</v>
       </c>
       <c r="F110" s="10">
@@ -5055,7 +5085,7 @@
       <c r="D111" s="10" t="s">
         <v>223</v>
       </c>
-      <c r="E111" s="18">
+      <c r="E111" s="17">
         <v>138</v>
       </c>
       <c r="F111" s="10">
@@ -5087,7 +5117,7 @@
       <c r="D112" s="10" t="s">
         <v>224</v>
       </c>
-      <c r="E112" s="18">
+      <c r="E112" s="17">
         <v>138</v>
       </c>
       <c r="F112" s="10">
@@ -5119,7 +5149,7 @@
       <c r="D113" s="10" t="s">
         <v>224</v>
       </c>
-      <c r="E113" s="18">
+      <c r="E113" s="17">
         <v>138</v>
       </c>
       <c r="F113" s="10">
@@ -5151,7 +5181,7 @@
       <c r="D114" s="10" t="s">
         <v>225</v>
       </c>
-      <c r="E114" s="18">
+      <c r="E114" s="17">
         <v>138</v>
       </c>
       <c r="F114" s="10">
@@ -5183,7 +5213,7 @@
       <c r="D115" s="10" t="s">
         <v>226</v>
       </c>
-      <c r="E115" s="18">
+      <c r="E115" s="17">
         <v>138</v>
       </c>
       <c r="F115" s="10">
@@ -5215,7 +5245,7 @@
       <c r="D116" s="10" t="s">
         <v>227</v>
       </c>
-      <c r="E116" s="18">
+      <c r="E116" s="17">
         <v>138</v>
       </c>
       <c r="F116" s="10">
@@ -5247,7 +5277,7 @@
       <c r="D117" s="10" t="s">
         <v>227</v>
       </c>
-      <c r="E117" s="18">
+      <c r="E117" s="17">
         <v>138</v>
       </c>
       <c r="F117" s="10">
@@ -5279,7 +5309,7 @@
       <c r="D118" s="10" t="s">
         <v>227</v>
       </c>
-      <c r="E118" s="18">
+      <c r="E118" s="17">
         <v>138</v>
       </c>
       <c r="F118" s="10">
@@ -5311,7 +5341,7 @@
       <c r="D119" s="10" t="s">
         <v>229</v>
       </c>
-      <c r="E119" s="18">
+      <c r="E119" s="17">
         <v>138</v>
       </c>
       <c r="F119" s="10">
@@ -5343,7 +5373,7 @@
       <c r="D120" s="10" t="s">
         <v>229</v>
       </c>
-      <c r="E120" s="18">
+      <c r="E120" s="17">
         <v>138</v>
       </c>
       <c r="F120" s="10">
@@ -5375,7 +5405,7 @@
       <c r="D121" s="10" t="s">
         <v>229</v>
       </c>
-      <c r="E121" s="18">
+      <c r="E121" s="17">
         <v>138</v>
       </c>
       <c r="F121" s="10">
@@ -5407,7 +5437,7 @@
       <c r="D122" s="10" t="s">
         <v>230</v>
       </c>
-      <c r="E122" s="18">
+      <c r="E122" s="17">
         <v>138</v>
       </c>
       <c r="F122" s="10">
@@ -5439,7 +5469,7 @@
       <c r="D123" s="10" t="s">
         <v>231</v>
       </c>
-      <c r="E123" s="18">
+      <c r="E123" s="17">
         <v>138</v>
       </c>
       <c r="F123" s="10">
@@ -5471,7 +5501,7 @@
       <c r="D124" s="10" t="s">
         <v>232</v>
       </c>
-      <c r="E124" s="18">
+      <c r="E124" s="17">
         <v>138</v>
       </c>
       <c r="F124" s="10">
@@ -5503,7 +5533,7 @@
       <c r="D125" s="10" t="s">
         <v>232</v>
       </c>
-      <c r="E125" s="18">
+      <c r="E125" s="17">
         <v>138</v>
       </c>
       <c r="F125" s="10">
@@ -5535,7 +5565,7 @@
       <c r="D126" s="10" t="s">
         <v>232</v>
       </c>
-      <c r="E126" s="18">
+      <c r="E126" s="17">
         <v>138</v>
       </c>
       <c r="F126" s="10">
@@ -5567,7 +5597,7 @@
       <c r="D127" s="10" t="s">
         <v>233</v>
       </c>
-      <c r="E127" s="18">
+      <c r="E127" s="17">
         <v>345</v>
       </c>
       <c r="F127" s="10">
@@ -5599,19 +5629,19 @@
       <c r="D128" s="10" t="s">
         <v>232</v>
       </c>
-      <c r="E128" s="18">
+      <c r="E128" s="17">
         <v>345</v>
       </c>
       <c r="F128" s="10">
         <v>1506.1311370164149</v>
       </c>
-      <c r="G128" s="19">
+      <c r="G128" s="18">
         <v>0</v>
       </c>
       <c r="H128" s="13">
         <v>44.039250000000003</v>
       </c>
-      <c r="I128" s="20">
+      <c r="I128" s="19">
         <v>0</v>
       </c>
       <c r="J128" s="13">
@@ -5631,7 +5661,7 @@
       <c r="D129" s="10" t="s">
         <v>234</v>
       </c>
-      <c r="E129" s="18">
+      <c r="E129" s="17">
         <v>138</v>
       </c>
       <c r="F129" s="10">
@@ -5663,7 +5693,7 @@
       <c r="D130" s="10" t="s">
         <v>235</v>
       </c>
-      <c r="E130" s="18">
+      <c r="E130" s="17">
         <v>138</v>
       </c>
       <c r="F130" s="10">
@@ -5695,7 +5725,7 @@
       <c r="D131" s="10" t="s">
         <v>236</v>
       </c>
-      <c r="E131" s="18">
+      <c r="E131" s="17">
         <v>138</v>
       </c>
       <c r="F131" s="10">
@@ -5727,7 +5757,7 @@
       <c r="D132" s="10" t="s">
         <v>237</v>
       </c>
-      <c r="E132" s="18">
+      <c r="E132" s="17">
         <v>138</v>
       </c>
       <c r="F132" s="10">
@@ -5759,7 +5789,7 @@
       <c r="D133" s="10" t="s">
         <v>237</v>
       </c>
-      <c r="E133" s="18">
+      <c r="E133" s="17">
         <v>138</v>
       </c>
       <c r="F133" s="10">
@@ -5791,7 +5821,7 @@
       <c r="D134" s="10" t="s">
         <v>238</v>
       </c>
-      <c r="E134" s="18">
+      <c r="E134" s="17">
         <v>138</v>
       </c>
       <c r="F134" s="10">
@@ -5823,7 +5853,7 @@
       <c r="D135" s="10" t="s">
         <v>239</v>
       </c>
-      <c r="E135" s="18">
+      <c r="E135" s="17">
         <v>138</v>
       </c>
       <c r="F135" s="10">
@@ -5855,7 +5885,7 @@
       <c r="D136" s="10" t="s">
         <v>240</v>
       </c>
-      <c r="E136" s="18">
+      <c r="E136" s="17">
         <v>138</v>
       </c>
       <c r="F136" s="10">
@@ -5887,7 +5917,7 @@
       <c r="D137" s="10" t="s">
         <v>241</v>
       </c>
-      <c r="E137" s="18">
+      <c r="E137" s="17">
         <v>138</v>
       </c>
       <c r="F137" s="10">
@@ -5919,7 +5949,7 @@
       <c r="D138" s="10" t="s">
         <v>241</v>
       </c>
-      <c r="E138" s="18">
+      <c r="E138" s="17">
         <v>138</v>
       </c>
       <c r="F138" s="10">
@@ -5951,7 +5981,7 @@
       <c r="D139" s="10" t="s">
         <v>242</v>
       </c>
-      <c r="E139" s="18">
+      <c r="E139" s="17">
         <v>138</v>
       </c>
       <c r="F139" s="10">
@@ -5983,7 +6013,7 @@
       <c r="D140" s="10" t="s">
         <v>242</v>
       </c>
-      <c r="E140" s="18">
+      <c r="E140" s="17">
         <v>138</v>
       </c>
       <c r="F140" s="10">
@@ -6015,7 +6045,7 @@
       <c r="D141" s="10" t="s">
         <v>243</v>
       </c>
-      <c r="E141" s="18">
+      <c r="E141" s="17">
         <v>138</v>
       </c>
       <c r="F141" s="10">
@@ -6047,7 +6077,7 @@
       <c r="D142" s="10" t="s">
         <v>244</v>
       </c>
-      <c r="E142" s="18">
+      <c r="E142" s="17">
         <v>138</v>
       </c>
       <c r="F142" s="10">
@@ -6079,7 +6109,7 @@
       <c r="D143" s="10" t="s">
         <v>244</v>
       </c>
-      <c r="E143" s="18">
+      <c r="E143" s="17">
         <v>138</v>
       </c>
       <c r="F143" s="10">
@@ -6111,7 +6141,7 @@
       <c r="D144" s="10" t="s">
         <v>244</v>
       </c>
-      <c r="E144" s="18">
+      <c r="E144" s="17">
         <v>138</v>
       </c>
       <c r="F144" s="10">
@@ -6143,7 +6173,7 @@
       <c r="D145" s="10" t="s">
         <v>245</v>
       </c>
-      <c r="E145" s="18">
+      <c r="E145" s="17">
         <v>138</v>
       </c>
       <c r="F145" s="10">
@@ -6175,7 +6205,7 @@
       <c r="D146" s="10" t="s">
         <v>246</v>
       </c>
-      <c r="E146" s="18">
+      <c r="E146" s="17">
         <v>138</v>
       </c>
       <c r="F146" s="10">
@@ -6207,7 +6237,7 @@
       <c r="D147" s="10" t="s">
         <v>246</v>
       </c>
-      <c r="E147" s="18">
+      <c r="E147" s="17">
         <v>138</v>
       </c>
       <c r="F147" s="10">
@@ -6239,7 +6269,7 @@
       <c r="D148" s="10" t="s">
         <v>247</v>
       </c>
-      <c r="E148" s="18">
+      <c r="E148" s="17">
         <v>138</v>
       </c>
       <c r="F148" s="10">
@@ -6271,7 +6301,7 @@
       <c r="D149" s="10" t="s">
         <v>248</v>
       </c>
-      <c r="E149" s="18">
+      <c r="E149" s="17">
         <v>138</v>
       </c>
       <c r="F149" s="10">
@@ -6303,7 +6333,7 @@
       <c r="D150" s="10" t="s">
         <v>248</v>
       </c>
-      <c r="E150" s="18">
+      <c r="E150" s="17">
         <v>138</v>
       </c>
       <c r="F150" s="10">
@@ -6335,7 +6365,7 @@
       <c r="D151" s="10" t="s">
         <v>248</v>
       </c>
-      <c r="E151" s="18">
+      <c r="E151" s="17">
         <v>138</v>
       </c>
       <c r="F151" s="10">
@@ -6367,7 +6397,7 @@
       <c r="D152" s="10" t="s">
         <v>249</v>
       </c>
-      <c r="E152" s="18">
+      <c r="E152" s="17">
         <v>138</v>
       </c>
       <c r="F152" s="10">
@@ -6399,7 +6429,7 @@
       <c r="D153" s="10" t="s">
         <v>250</v>
       </c>
-      <c r="E153" s="18">
+      <c r="E153" s="17">
         <v>138</v>
       </c>
       <c r="F153" s="10">
@@ -6431,7 +6461,7 @@
       <c r="D154" s="10" t="s">
         <v>251</v>
       </c>
-      <c r="E154" s="18">
+      <c r="E154" s="17">
         <v>138</v>
       </c>
       <c r="F154" s="10">
@@ -6463,7 +6493,7 @@
       <c r="D155" s="10" t="s">
         <v>252</v>
       </c>
-      <c r="E155" s="18">
+      <c r="E155" s="17">
         <v>138</v>
       </c>
       <c r="F155" s="10">
@@ -6495,7 +6525,7 @@
       <c r="D156" s="10" t="s">
         <v>252</v>
       </c>
-      <c r="E156" s="18">
+      <c r="E156" s="17">
         <v>138</v>
       </c>
       <c r="F156" s="10">
@@ -6527,7 +6557,7 @@
       <c r="D157" s="10" t="s">
         <v>248</v>
       </c>
-      <c r="E157" s="18">
+      <c r="E157" s="17">
         <v>138</v>
       </c>
       <c r="F157" s="10">
@@ -6559,7 +6589,7 @@
       <c r="D158" s="10" t="s">
         <v>249</v>
       </c>
-      <c r="E158" s="18">
+      <c r="E158" s="17">
         <v>138</v>
       </c>
       <c r="F158" s="10">
@@ -6591,7 +6621,7 @@
       <c r="D159" s="10" t="s">
         <v>252</v>
       </c>
-      <c r="E159" s="18">
+      <c r="E159" s="17">
         <v>138</v>
       </c>
       <c r="F159" s="10">
@@ -6623,7 +6653,7 @@
       <c r="D160" s="10" t="s">
         <v>252</v>
       </c>
-      <c r="E160" s="18">
+      <c r="E160" s="17">
         <v>138</v>
       </c>
       <c r="F160" s="10">
@@ -6655,7 +6685,7 @@
       <c r="D161" s="10" t="s">
         <v>253</v>
       </c>
-      <c r="E161" s="18">
+      <c r="E161" s="17">
         <v>138</v>
       </c>
       <c r="F161" s="10">
@@ -6687,7 +6717,7 @@
       <c r="D162" s="10" t="s">
         <v>254</v>
       </c>
-      <c r="E162" s="18">
+      <c r="E162" s="17">
         <v>138</v>
       </c>
       <c r="F162" s="10">
@@ -6719,7 +6749,7 @@
       <c r="D163" s="10" t="s">
         <v>254</v>
       </c>
-      <c r="E163" s="18">
+      <c r="E163" s="17">
         <v>138</v>
       </c>
       <c r="F163" s="10">
@@ -6751,7 +6781,7 @@
       <c r="D164" s="10" t="s">
         <v>255</v>
       </c>
-      <c r="E164" s="18">
+      <c r="E164" s="17">
         <v>138</v>
       </c>
       <c r="F164" s="10">
@@ -6783,7 +6813,7 @@
       <c r="D165" s="10" t="s">
         <v>256</v>
       </c>
-      <c r="E165" s="18">
+      <c r="E165" s="17">
         <v>138</v>
       </c>
       <c r="F165" s="10">
@@ -6815,7 +6845,7 @@
       <c r="D166" s="10" t="s">
         <v>256</v>
       </c>
-      <c r="E166" s="18">
+      <c r="E166" s="17">
         <v>138</v>
       </c>
       <c r="F166" s="10">
@@ -6847,7 +6877,7 @@
       <c r="D167" s="10" t="s">
         <v>257</v>
       </c>
-      <c r="E167" s="18">
+      <c r="E167" s="17">
         <v>138</v>
       </c>
       <c r="F167" s="10">
@@ -6879,7 +6909,7 @@
       <c r="D168" s="10" t="s">
         <v>258</v>
       </c>
-      <c r="E168" s="18">
+      <c r="E168" s="17">
         <v>138</v>
       </c>
       <c r="F168" s="10">
@@ -6911,7 +6941,7 @@
       <c r="D169" s="10" t="s">
         <v>257</v>
       </c>
-      <c r="E169" s="18">
+      <c r="E169" s="17">
         <v>138</v>
       </c>
       <c r="F169" s="10">
@@ -6943,7 +6973,7 @@
       <c r="D170" s="10" t="s">
         <v>258</v>
       </c>
-      <c r="E170" s="18">
+      <c r="E170" s="17">
         <v>138</v>
       </c>
       <c r="F170" s="10">
@@ -6975,7 +7005,7 @@
       <c r="D171" s="10" t="s">
         <v>259</v>
       </c>
-      <c r="E171" s="18">
+      <c r="E171" s="17">
         <v>138</v>
       </c>
       <c r="F171" s="10">
@@ -7007,7 +7037,7 @@
       <c r="D172" s="10" t="s">
         <v>260</v>
       </c>
-      <c r="E172" s="18">
+      <c r="E172" s="17">
         <v>138</v>
       </c>
       <c r="F172" s="10">
@@ -7039,7 +7069,7 @@
       <c r="D173" s="10" t="s">
         <v>259</v>
       </c>
-      <c r="E173" s="18">
+      <c r="E173" s="17">
         <v>138</v>
       </c>
       <c r="F173" s="10">
@@ -7071,7 +7101,7 @@
       <c r="D174" s="10" t="s">
         <v>261</v>
       </c>
-      <c r="E174" s="18">
+      <c r="E174" s="17">
         <v>138</v>
       </c>
       <c r="F174" s="10">
@@ -7103,7 +7133,7 @@
       <c r="D175" s="10" t="s">
         <v>262</v>
       </c>
-      <c r="E175" s="18">
+      <c r="E175" s="17">
         <v>138</v>
       </c>
       <c r="F175" s="10">
@@ -7135,7 +7165,7 @@
       <c r="D176" s="10" t="s">
         <v>262</v>
       </c>
-      <c r="E176" s="18">
+      <c r="E176" s="17">
         <v>138</v>
       </c>
       <c r="F176" s="10">
@@ -7167,7 +7197,7 @@
       <c r="D177" s="10" t="s">
         <v>263</v>
       </c>
-      <c r="E177" s="18">
+      <c r="E177" s="17">
         <v>138</v>
       </c>
       <c r="F177" s="10">
@@ -7199,7 +7229,7 @@
       <c r="D178" s="10" t="s">
         <v>264</v>
       </c>
-      <c r="E178" s="18">
+      <c r="E178" s="17">
         <v>138</v>
       </c>
       <c r="F178" s="10">
@@ -7231,7 +7261,7 @@
       <c r="D179" s="10" t="s">
         <v>266</v>
       </c>
-      <c r="E179" s="18">
+      <c r="E179" s="17">
         <v>138</v>
       </c>
       <c r="F179" s="10">
@@ -7263,7 +7293,7 @@
       <c r="D180" s="10" t="s">
         <v>266</v>
       </c>
-      <c r="E180" s="18">
+      <c r="E180" s="17">
         <v>138</v>
       </c>
       <c r="F180" s="10">
@@ -7295,7 +7325,7 @@
       <c r="D181" s="10" t="s">
         <v>268</v>
       </c>
-      <c r="E181" s="18">
+      <c r="E181" s="17">
         <v>138</v>
       </c>
       <c r="F181" s="10">
@@ -7327,7 +7357,7 @@
       <c r="D182" s="10" t="s">
         <v>270</v>
       </c>
-      <c r="E182" s="18">
+      <c r="E182" s="17">
         <v>138</v>
       </c>
       <c r="F182" s="10">
@@ -7359,7 +7389,7 @@
       <c r="D183" s="10" t="s">
         <v>270</v>
       </c>
-      <c r="E183" s="18">
+      <c r="E183" s="17">
         <v>138</v>
       </c>
       <c r="F183" s="10">
@@ -7391,7 +7421,7 @@
       <c r="D184" s="10" t="s">
         <v>271</v>
       </c>
-      <c r="E184" s="18">
+      <c r="E184" s="17">
         <v>345</v>
       </c>
       <c r="F184" s="10">
@@ -7423,7 +7453,7 @@
       <c r="D185" s="10" t="s">
         <v>273</v>
       </c>
-      <c r="E185" s="18">
+      <c r="E185" s="17">
         <v>138</v>
       </c>
       <c r="F185" s="10">
@@ -7455,7 +7485,7 @@
       <c r="D186" s="10" t="s">
         <v>274</v>
       </c>
-      <c r="E186" s="18">
+      <c r="E186" s="17">
         <v>138</v>
       </c>
       <c r="F186" s="10">
@@ -7571,14 +7601,15 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABBA67B1-483C-4642-AA56-A1B87583E7BE}">
-  <dimension ref="A1:P119"/>
+  <dimension ref="A1:Q152"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.5703125" customWidth="1"/>
     <col min="2" max="2" width="16.42578125" customWidth="1"/>
+    <col min="17" max="17" width="71.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16">
+    <row r="1" spans="1:17">
       <c r="A1" t="s">
         <v>11</v>
       </c>
@@ -7627,8 +7658,9 @@
       <c r="P1" s="9" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="2" spans="1:16">
+      <c r="Q1" s="20"/>
+    </row>
+    <row r="2" spans="1:17">
       <c r="A2" s="15" t="s">
         <v>275</v>
       </c>
@@ -7660,7 +7692,7 @@
       <c r="K2" s="15">
         <v>138</v>
       </c>
-      <c r="L2" t="s">
+      <c r="L2" s="15" t="s">
         <v>332</v>
       </c>
       <c r="M2" s="15">
@@ -7669,10 +7701,9 @@
       <c r="N2" s="15">
         <v>0.94</v>
       </c>
-      <c r="O2" s="15"/>
-      <c r="P2" s="15"/>
-    </row>
-    <row r="3" spans="1:16" ht="17.25">
+      <c r="Q2" s="20"/>
+    </row>
+    <row r="3" spans="1:17">
       <c r="A3" s="15" t="s">
         <v>276</v>
       </c>
@@ -7704,7 +7735,7 @@
       <c r="K3" s="15">
         <v>138</v>
       </c>
-      <c r="L3" t="s">
+      <c r="L3" s="15" t="s">
         <v>332</v>
       </c>
       <c r="M3" s="15">
@@ -7713,10 +7744,9 @@
       <c r="N3" s="15">
         <v>0.94</v>
       </c>
-      <c r="O3" s="16"/>
-      <c r="P3" s="15"/>
-    </row>
-    <row r="4" spans="1:16">
+      <c r="Q3" s="20"/>
+    </row>
+    <row r="4" spans="1:17">
       <c r="A4" s="15" t="s">
         <v>277</v>
       </c>
@@ -7748,7 +7778,7 @@
       <c r="K4" s="15">
         <v>138</v>
       </c>
-      <c r="L4" t="s">
+      <c r="L4" s="15" t="s">
         <v>332</v>
       </c>
       <c r="M4" s="15">
@@ -7757,10 +7787,9 @@
       <c r="N4" s="15">
         <v>0.94</v>
       </c>
-      <c r="O4" s="15"/>
-      <c r="P4" s="15"/>
-    </row>
-    <row r="5" spans="1:16">
+      <c r="Q4" s="20"/>
+    </row>
+    <row r="5" spans="1:17">
       <c r="A5" s="15" t="s">
         <v>278</v>
       </c>
@@ -7792,7 +7821,7 @@
       <c r="K5" s="15">
         <v>138</v>
       </c>
-      <c r="L5" t="s">
+      <c r="L5" s="15" t="s">
         <v>332</v>
       </c>
       <c r="M5" s="15">
@@ -7801,10 +7830,9 @@
       <c r="N5" s="15">
         <v>0.94</v>
       </c>
-      <c r="O5" s="15"/>
-      <c r="P5" s="15"/>
-    </row>
-    <row r="6" spans="1:16">
+      <c r="Q5" s="20"/>
+    </row>
+    <row r="6" spans="1:17">
       <c r="A6" s="15" t="s">
         <v>279</v>
       </c>
@@ -7836,7 +7864,7 @@
       <c r="K6" s="15">
         <v>138</v>
       </c>
-      <c r="L6" t="s">
+      <c r="L6" s="15" t="s">
         <v>332</v>
       </c>
       <c r="M6" s="15">
@@ -7845,10 +7873,9 @@
       <c r="N6" s="15">
         <v>0.94</v>
       </c>
-      <c r="O6" s="15"/>
-      <c r="P6" s="15"/>
-    </row>
-    <row r="7" spans="1:16">
+      <c r="Q6" s="20"/>
+    </row>
+    <row r="7" spans="1:17">
       <c r="A7" s="15" t="s">
         <v>280</v>
       </c>
@@ -7880,7 +7907,7 @@
       <c r="K7" s="15">
         <v>138</v>
       </c>
-      <c r="L7" t="s">
+      <c r="L7" s="15" t="s">
         <v>332</v>
       </c>
       <c r="M7" s="15">
@@ -7889,10 +7916,9 @@
       <c r="N7" s="15">
         <v>0.94</v>
       </c>
-      <c r="O7" s="15"/>
-      <c r="P7" s="15"/>
-    </row>
-    <row r="8" spans="1:16">
+      <c r="Q7" s="20"/>
+    </row>
+    <row r="8" spans="1:17">
       <c r="A8" s="15" t="s">
         <v>281</v>
       </c>
@@ -7924,7 +7950,7 @@
       <c r="K8" s="15">
         <v>138</v>
       </c>
-      <c r="L8" t="s">
+      <c r="L8" s="15" t="s">
         <v>332</v>
       </c>
       <c r="M8" s="15">
@@ -7933,10 +7959,9 @@
       <c r="N8" s="15">
         <v>0.94</v>
       </c>
-      <c r="O8" s="15"/>
-      <c r="P8" s="15"/>
-    </row>
-    <row r="9" spans="1:16">
+      <c r="Q8" s="20"/>
+    </row>
+    <row r="9" spans="1:17">
       <c r="A9" s="15" t="s">
         <v>282</v>
       </c>
@@ -7968,7 +7993,7 @@
       <c r="K9" s="15">
         <v>345</v>
       </c>
-      <c r="L9" t="s">
+      <c r="L9" s="15" t="s">
         <v>332</v>
       </c>
       <c r="M9" s="15">
@@ -7977,10 +8002,9 @@
       <c r="N9" s="15">
         <v>0.94</v>
       </c>
-      <c r="O9" s="15"/>
-      <c r="P9" s="15"/>
-    </row>
-    <row r="10" spans="1:16">
+      <c r="Q9" s="20"/>
+    </row>
+    <row r="10" spans="1:17">
       <c r="A10" s="15" t="s">
         <v>283</v>
       </c>
@@ -8012,7 +8036,7 @@
       <c r="K10" s="15">
         <v>345</v>
       </c>
-      <c r="L10" t="s">
+      <c r="L10" s="15" t="s">
         <v>332</v>
       </c>
       <c r="M10" s="15">
@@ -8021,10 +8045,9 @@
       <c r="N10" s="15">
         <v>0.94</v>
       </c>
-      <c r="O10" s="15"/>
-      <c r="P10" s="15"/>
-    </row>
-    <row r="11" spans="1:16">
+      <c r="Q10" s="20"/>
+    </row>
+    <row r="11" spans="1:17">
       <c r="A11" s="15" t="s">
         <v>284</v>
       </c>
@@ -8056,7 +8079,7 @@
       <c r="K11" s="15">
         <v>345</v>
       </c>
-      <c r="L11" t="s">
+      <c r="L11" s="15" t="s">
         <v>332</v>
       </c>
       <c r="M11" s="15">
@@ -8065,10 +8088,9 @@
       <c r="N11" s="15">
         <v>0.94</v>
       </c>
-      <c r="O11" s="15"/>
-      <c r="P11" s="15"/>
-    </row>
-    <row r="12" spans="1:16">
+      <c r="Q11" s="20"/>
+    </row>
+    <row r="12" spans="1:17">
       <c r="A12" s="15" t="s">
         <v>285</v>
       </c>
@@ -8100,7 +8122,7 @@
       <c r="K12" s="15">
         <v>138</v>
       </c>
-      <c r="L12" t="s">
+      <c r="L12" s="15" t="s">
         <v>332</v>
       </c>
       <c r="M12" s="15">
@@ -8109,10 +8131,9 @@
       <c r="N12" s="15">
         <v>0.94</v>
       </c>
-      <c r="O12" s="15"/>
-      <c r="P12" s="15"/>
-    </row>
-    <row r="13" spans="1:16">
+      <c r="Q12" s="20"/>
+    </row>
+    <row r="13" spans="1:17">
       <c r="A13" s="15" t="s">
         <v>272</v>
       </c>
@@ -8144,7 +8165,7 @@
       <c r="K13" s="15">
         <v>138</v>
       </c>
-      <c r="L13" t="s">
+      <c r="L13" s="15" t="s">
         <v>332</v>
       </c>
       <c r="M13" s="15">
@@ -8153,10 +8174,9 @@
       <c r="N13" s="15">
         <v>0.94</v>
       </c>
-      <c r="O13" s="15"/>
-      <c r="P13" s="15"/>
-    </row>
-    <row r="14" spans="1:16">
+      <c r="Q13" s="20"/>
+    </row>
+    <row r="14" spans="1:17">
       <c r="A14" s="15" t="s">
         <v>286</v>
       </c>
@@ -8188,7 +8208,7 @@
       <c r="K14" s="15">
         <v>138</v>
       </c>
-      <c r="L14" t="s">
+      <c r="L14" s="15" t="s">
         <v>332</v>
       </c>
       <c r="M14" s="15">
@@ -8197,10 +8217,9 @@
       <c r="N14" s="15">
         <v>0.94</v>
       </c>
-      <c r="O14" s="15"/>
-      <c r="P14" s="15"/>
-    </row>
-    <row r="15" spans="1:16">
+      <c r="Q14" s="20"/>
+    </row>
+    <row r="15" spans="1:17">
       <c r="A15" s="15" t="s">
         <v>287</v>
       </c>
@@ -8232,7 +8251,7 @@
       <c r="K15" s="15">
         <v>138</v>
       </c>
-      <c r="L15" t="s">
+      <c r="L15" s="15" t="s">
         <v>332</v>
       </c>
       <c r="M15" s="15">
@@ -8241,10 +8260,9 @@
       <c r="N15" s="15">
         <v>0.94</v>
       </c>
-      <c r="O15" s="15"/>
-      <c r="P15" s="15"/>
-    </row>
-    <row r="16" spans="1:16">
+      <c r="Q15" s="20"/>
+    </row>
+    <row r="16" spans="1:17">
       <c r="A16" s="15" t="s">
         <v>288</v>
       </c>
@@ -8276,7 +8294,7 @@
       <c r="K16" s="15">
         <v>138</v>
       </c>
-      <c r="L16" t="s">
+      <c r="L16" s="15" t="s">
         <v>332</v>
       </c>
       <c r="M16" s="15">
@@ -8285,10 +8303,9 @@
       <c r="N16" s="15">
         <v>0.94</v>
       </c>
-      <c r="O16" s="15"/>
-      <c r="P16" s="15"/>
-    </row>
-    <row r="17" spans="1:16">
+      <c r="Q16" s="20"/>
+    </row>
+    <row r="17" spans="1:17">
       <c r="A17" s="15" t="s">
         <v>289</v>
       </c>
@@ -8320,7 +8337,7 @@
       <c r="K17" s="15">
         <v>138</v>
       </c>
-      <c r="L17" t="s">
+      <c r="L17" s="15" t="s">
         <v>332</v>
       </c>
       <c r="M17" s="15">
@@ -8329,10 +8346,9 @@
       <c r="N17" s="15">
         <v>0.94</v>
       </c>
-      <c r="O17" s="15"/>
-      <c r="P17" s="15"/>
-    </row>
-    <row r="18" spans="1:16">
+      <c r="Q17" s="20"/>
+    </row>
+    <row r="18" spans="1:17">
       <c r="A18" s="15" t="s">
         <v>265</v>
       </c>
@@ -8364,8 +8380,8 @@
       <c r="K18" s="15">
         <v>138</v>
       </c>
-      <c r="L18" t="s">
-        <v>332</v>
+      <c r="L18" s="15" t="s">
+        <v>333</v>
       </c>
       <c r="M18" s="15">
         <v>1.06</v>
@@ -8373,10 +8389,9 @@
       <c r="N18" s="15">
         <v>0.94</v>
       </c>
-      <c r="O18" s="15"/>
-      <c r="P18" s="15"/>
-    </row>
-    <row r="19" spans="1:16">
+      <c r="Q18" s="20"/>
+    </row>
+    <row r="19" spans="1:17">
       <c r="A19" s="15" t="s">
         <v>290</v>
       </c>
@@ -8408,8 +8423,8 @@
       <c r="K19" s="15">
         <v>138</v>
       </c>
-      <c r="L19" t="s">
-        <v>332</v>
+      <c r="L19" s="15" t="s">
+        <v>333</v>
       </c>
       <c r="M19" s="15">
         <v>1.06</v>
@@ -8417,10 +8432,9 @@
       <c r="N19" s="15">
         <v>0.94</v>
       </c>
-      <c r="O19" s="15"/>
-      <c r="P19" s="15"/>
-    </row>
-    <row r="20" spans="1:16">
+      <c r="Q19" s="20"/>
+    </row>
+    <row r="20" spans="1:17">
       <c r="A20" s="15" t="s">
         <v>291</v>
       </c>
@@ -8452,8 +8466,8 @@
       <c r="K20" s="15">
         <v>138</v>
       </c>
-      <c r="L20" t="s">
-        <v>332</v>
+      <c r="L20" s="15" t="s">
+        <v>333</v>
       </c>
       <c r="M20" s="15">
         <v>1.06</v>
@@ -8461,10 +8475,9 @@
       <c r="N20" s="15">
         <v>0.94</v>
       </c>
-      <c r="O20" s="15"/>
-      <c r="P20" s="15"/>
-    </row>
-    <row r="21" spans="1:16">
+      <c r="Q20" s="20"/>
+    </row>
+    <row r="21" spans="1:17">
       <c r="A21" s="15" t="s">
         <v>292</v>
       </c>
@@ -8496,8 +8509,8 @@
       <c r="K21" s="15">
         <v>138</v>
       </c>
-      <c r="L21" t="s">
-        <v>332</v>
+      <c r="L21" s="15" t="s">
+        <v>333</v>
       </c>
       <c r="M21" s="15">
         <v>1.06</v>
@@ -8505,10 +8518,9 @@
       <c r="N21" s="15">
         <v>0.94</v>
       </c>
-      <c r="O21" s="15"/>
-      <c r="P21" s="15"/>
-    </row>
-    <row r="22" spans="1:16">
+      <c r="Q21" s="20"/>
+    </row>
+    <row r="22" spans="1:17">
       <c r="A22" s="15" t="s">
         <v>293</v>
       </c>
@@ -8540,8 +8552,8 @@
       <c r="K22" s="15">
         <v>138</v>
       </c>
-      <c r="L22" t="s">
-        <v>332</v>
+      <c r="L22" s="15" t="s">
+        <v>333</v>
       </c>
       <c r="M22" s="15">
         <v>1.06</v>
@@ -8549,10 +8561,9 @@
       <c r="N22" s="15">
         <v>0.94</v>
       </c>
-      <c r="O22" s="15"/>
-      <c r="P22" s="15"/>
-    </row>
-    <row r="23" spans="1:16">
+      <c r="Q22" s="20"/>
+    </row>
+    <row r="23" spans="1:17">
       <c r="A23" s="15" t="s">
         <v>294</v>
       </c>
@@ -8584,8 +8595,8 @@
       <c r="K23" s="15">
         <v>138</v>
       </c>
-      <c r="L23" t="s">
-        <v>332</v>
+      <c r="L23" s="15" t="s">
+        <v>333</v>
       </c>
       <c r="M23" s="15">
         <v>1.06</v>
@@ -8593,10 +8604,9 @@
       <c r="N23" s="15">
         <v>0.94</v>
       </c>
-      <c r="O23" s="15"/>
-      <c r="P23" s="15"/>
-    </row>
-    <row r="24" spans="1:16">
+      <c r="Q23" s="20"/>
+    </row>
+    <row r="24" spans="1:17">
       <c r="A24" s="15" t="s">
         <v>295</v>
       </c>
@@ -8628,8 +8638,8 @@
       <c r="K24" s="15">
         <v>138</v>
       </c>
-      <c r="L24" t="s">
-        <v>332</v>
+      <c r="L24" s="15" t="s">
+        <v>333</v>
       </c>
       <c r="M24" s="15">
         <v>1.06</v>
@@ -8637,10 +8647,9 @@
       <c r="N24" s="15">
         <v>0.94</v>
       </c>
-      <c r="O24" s="15"/>
-      <c r="P24" s="15"/>
-    </row>
-    <row r="25" spans="1:16">
+      <c r="Q24" s="20"/>
+    </row>
+    <row r="25" spans="1:17">
       <c r="A25" s="15" t="s">
         <v>222</v>
       </c>
@@ -8672,8 +8681,8 @@
       <c r="K25" s="15">
         <v>138</v>
       </c>
-      <c r="L25" t="s">
-        <v>332</v>
+      <c r="L25" s="15" t="s">
+        <v>333</v>
       </c>
       <c r="M25" s="15">
         <v>1.06</v>
@@ -8681,10 +8690,9 @@
       <c r="N25" s="15">
         <v>0.94</v>
       </c>
-      <c r="O25" s="15"/>
-      <c r="P25" s="15"/>
-    </row>
-    <row r="26" spans="1:16">
+      <c r="Q25" s="20"/>
+    </row>
+    <row r="26" spans="1:17">
       <c r="A26" s="15" t="s">
         <v>296</v>
       </c>
@@ -8716,8 +8724,8 @@
       <c r="K26" s="15">
         <v>138</v>
       </c>
-      <c r="L26" t="s">
-        <v>332</v>
+      <c r="L26" s="15" t="s">
+        <v>333</v>
       </c>
       <c r="M26" s="15">
         <v>1.06</v>
@@ -8725,10 +8733,9 @@
       <c r="N26" s="15">
         <v>0.94</v>
       </c>
-      <c r="O26" s="15"/>
-      <c r="P26" s="15"/>
-    </row>
-    <row r="27" spans="1:16">
+      <c r="Q26" s="20"/>
+    </row>
+    <row r="27" spans="1:17">
       <c r="A27" s="15" t="s">
         <v>297</v>
       </c>
@@ -8760,8 +8767,8 @@
       <c r="K27" s="15">
         <v>345</v>
       </c>
-      <c r="L27" t="s">
-        <v>332</v>
+      <c r="L27" s="15" t="s">
+        <v>333</v>
       </c>
       <c r="M27" s="15">
         <v>1.06</v>
@@ -8769,10 +8776,9 @@
       <c r="N27" s="15">
         <v>0.94</v>
       </c>
-      <c r="O27" s="15"/>
-      <c r="P27" s="15"/>
-    </row>
-    <row r="28" spans="1:16">
+      <c r="Q27" s="20"/>
+    </row>
+    <row r="28" spans="1:17">
       <c r="A28" s="15" t="s">
         <v>269</v>
       </c>
@@ -8804,8 +8810,8 @@
       <c r="K28" s="15">
         <v>138</v>
       </c>
-      <c r="L28" t="s">
-        <v>332</v>
+      <c r="L28" s="15" t="s">
+        <v>333</v>
       </c>
       <c r="M28" s="15">
         <v>1.06</v>
@@ -8813,10 +8819,9 @@
       <c r="N28" s="15">
         <v>0.94</v>
       </c>
-      <c r="O28" s="15"/>
-      <c r="P28" s="15"/>
-    </row>
-    <row r="29" spans="1:16">
+      <c r="Q28" s="20"/>
+    </row>
+    <row r="29" spans="1:17">
       <c r="A29" s="15" t="s">
         <v>298</v>
       </c>
@@ -8848,8 +8853,8 @@
       <c r="K29" s="15">
         <v>138</v>
       </c>
-      <c r="L29" t="s">
-        <v>332</v>
+      <c r="L29" s="15" t="s">
+        <v>333</v>
       </c>
       <c r="M29" s="15">
         <v>1.06</v>
@@ -8857,10 +8862,9 @@
       <c r="N29" s="15">
         <v>0.94</v>
       </c>
-      <c r="O29" s="15"/>
-      <c r="P29" s="15"/>
-    </row>
-    <row r="30" spans="1:16">
+      <c r="Q29" s="20"/>
+    </row>
+    <row r="30" spans="1:17">
       <c r="A30" s="15" t="s">
         <v>299</v>
       </c>
@@ -8892,8 +8896,8 @@
       <c r="K30" s="15">
         <v>138</v>
       </c>
-      <c r="L30" t="s">
-        <v>332</v>
+      <c r="L30" s="15" t="s">
+        <v>333</v>
       </c>
       <c r="M30" s="15">
         <v>1.06</v>
@@ -8901,10 +8905,9 @@
       <c r="N30" s="15">
         <v>0.94</v>
       </c>
-      <c r="O30" s="15"/>
-      <c r="P30" s="15"/>
-    </row>
-    <row r="31" spans="1:16">
+      <c r="Q30" s="20"/>
+    </row>
+    <row r="31" spans="1:17">
       <c r="A31" s="15" t="s">
         <v>300</v>
       </c>
@@ -8936,8 +8939,8 @@
       <c r="K31" s="15">
         <v>345</v>
       </c>
-      <c r="L31" t="s">
-        <v>332</v>
+      <c r="L31" s="15" t="s">
+        <v>333</v>
       </c>
       <c r="M31" s="15">
         <v>1.06</v>
@@ -8945,10 +8948,9 @@
       <c r="N31" s="15">
         <v>0.94</v>
       </c>
-      <c r="O31" s="15"/>
-      <c r="P31" s="15"/>
-    </row>
-    <row r="32" spans="1:16">
+      <c r="Q31" s="20"/>
+    </row>
+    <row r="32" spans="1:17">
       <c r="A32" s="15" t="s">
         <v>301</v>
       </c>
@@ -8980,8 +8982,8 @@
       <c r="K32" s="15">
         <v>138</v>
       </c>
-      <c r="L32" t="s">
-        <v>332</v>
+      <c r="L32" s="15" t="s">
+        <v>333</v>
       </c>
       <c r="M32" s="15">
         <v>1.06</v>
@@ -8989,10 +8991,9 @@
       <c r="N32" s="15">
         <v>0.94</v>
       </c>
-      <c r="O32" s="15"/>
-      <c r="P32" s="15"/>
-    </row>
-    <row r="33" spans="1:16">
+      <c r="Q32" s="20"/>
+    </row>
+    <row r="33" spans="1:17">
       <c r="A33" s="15" t="s">
         <v>267</v>
       </c>
@@ -9024,8 +9025,8 @@
       <c r="K33" s="15">
         <v>138</v>
       </c>
-      <c r="L33" t="s">
-        <v>332</v>
+      <c r="L33" s="15" t="s">
+        <v>333</v>
       </c>
       <c r="M33" s="15">
         <v>1.06</v>
@@ -9033,10 +9034,9 @@
       <c r="N33" s="15">
         <v>0.94</v>
       </c>
-      <c r="O33" s="15"/>
-      <c r="P33" s="15"/>
-    </row>
-    <row r="34" spans="1:16">
+      <c r="Q33" s="20"/>
+    </row>
+    <row r="34" spans="1:17">
       <c r="A34" s="15" t="s">
         <v>302</v>
       </c>
@@ -9068,8 +9068,8 @@
       <c r="K34" s="15">
         <v>138</v>
       </c>
-      <c r="L34" t="s">
-        <v>332</v>
+      <c r="L34" s="15" t="s">
+        <v>333</v>
       </c>
       <c r="M34" s="15">
         <v>1.06</v>
@@ -9077,10 +9077,9 @@
       <c r="N34" s="15">
         <v>0.94</v>
       </c>
-      <c r="O34" s="15"/>
-      <c r="P34" s="15"/>
-    </row>
-    <row r="35" spans="1:16">
+      <c r="Q34" s="20"/>
+    </row>
+    <row r="35" spans="1:17">
       <c r="A35" s="15" t="s">
         <v>303</v>
       </c>
@@ -9112,7 +9111,7 @@
       <c r="K35" s="15">
         <v>138</v>
       </c>
-      <c r="L35" t="s">
+      <c r="L35" s="15" t="s">
         <v>333</v>
       </c>
       <c r="M35" s="15">
@@ -9121,10 +9120,9 @@
       <c r="N35" s="15">
         <v>0.94</v>
       </c>
-      <c r="O35" s="15"/>
-      <c r="P35" s="15"/>
-    </row>
-    <row r="36" spans="1:16">
+      <c r="Q35" s="20"/>
+    </row>
+    <row r="36" spans="1:17">
       <c r="A36" s="15" t="s">
         <v>304</v>
       </c>
@@ -9156,7 +9154,7 @@
       <c r="K36" s="15">
         <v>138</v>
       </c>
-      <c r="L36" t="s">
+      <c r="L36" s="15" t="s">
         <v>333</v>
       </c>
       <c r="M36" s="15">
@@ -9165,10 +9163,9 @@
       <c r="N36" s="15">
         <v>0.94</v>
       </c>
-      <c r="O36" s="15"/>
-      <c r="P36" s="15"/>
-    </row>
-    <row r="37" spans="1:16">
+      <c r="Q36" s="20"/>
+    </row>
+    <row r="37" spans="1:17">
       <c r="A37" s="15" t="s">
         <v>305</v>
       </c>
@@ -9200,7 +9197,7 @@
       <c r="K37" s="15">
         <v>138</v>
       </c>
-      <c r="L37" t="s">
+      <c r="L37" s="15" t="s">
         <v>333</v>
       </c>
       <c r="M37" s="15">
@@ -9209,10 +9206,9 @@
       <c r="N37" s="15">
         <v>0.94</v>
       </c>
-      <c r="O37" s="15"/>
-      <c r="P37" s="15"/>
-    </row>
-    <row r="38" spans="1:16">
+      <c r="Q37" s="20"/>
+    </row>
+    <row r="38" spans="1:17">
       <c r="A38" s="15" t="s">
         <v>306</v>
       </c>
@@ -9244,7 +9240,7 @@
       <c r="K38" s="15">
         <v>138</v>
       </c>
-      <c r="L38" t="s">
+      <c r="L38" s="15" t="s">
         <v>333</v>
       </c>
       <c r="M38" s="15">
@@ -9253,10 +9249,9 @@
       <c r="N38" s="15">
         <v>0.94</v>
       </c>
-      <c r="O38" s="15"/>
-      <c r="P38" s="15"/>
-    </row>
-    <row r="39" spans="1:16">
+      <c r="Q38" s="20"/>
+    </row>
+    <row r="39" spans="1:17">
       <c r="A39" s="15" t="s">
         <v>307</v>
       </c>
@@ -9288,7 +9283,7 @@
       <c r="K39" s="15">
         <v>345</v>
       </c>
-      <c r="L39" t="s">
+      <c r="L39" s="15" t="s">
         <v>333</v>
       </c>
       <c r="M39" s="15">
@@ -9297,10 +9292,9 @@
       <c r="N39" s="15">
         <v>0.94</v>
       </c>
-      <c r="O39" s="15"/>
-      <c r="P39" s="15"/>
-    </row>
-    <row r="40" spans="1:16">
+      <c r="Q39" s="20"/>
+    </row>
+    <row r="40" spans="1:17">
       <c r="A40" s="15" t="s">
         <v>308</v>
       </c>
@@ -9332,7 +9326,7 @@
       <c r="K40" s="15">
         <v>138</v>
       </c>
-      <c r="L40" t="s">
+      <c r="L40" s="15" t="s">
         <v>333</v>
       </c>
       <c r="M40" s="15">
@@ -9341,10 +9335,9 @@
       <c r="N40" s="15">
         <v>0.94</v>
       </c>
-      <c r="O40" s="15"/>
-      <c r="P40" s="15"/>
-    </row>
-    <row r="41" spans="1:16">
+      <c r="Q40" s="20"/>
+    </row>
+    <row r="41" spans="1:17">
       <c r="A41" s="15" t="s">
         <v>309</v>
       </c>
@@ -9376,7 +9369,7 @@
       <c r="K41" s="15">
         <v>138</v>
       </c>
-      <c r="L41" t="s">
+      <c r="L41" s="15" t="s">
         <v>333</v>
       </c>
       <c r="M41" s="15">
@@ -9385,10 +9378,9 @@
       <c r="N41" s="15">
         <v>0.94</v>
       </c>
-      <c r="O41" s="15"/>
-      <c r="P41" s="15"/>
-    </row>
-    <row r="42" spans="1:16">
+      <c r="Q41" s="20"/>
+    </row>
+    <row r="42" spans="1:17">
       <c r="A42" s="15" t="s">
         <v>310</v>
       </c>
@@ -9420,8 +9412,8 @@
       <c r="K42" s="15">
         <v>138</v>
       </c>
-      <c r="L42" t="s">
-        <v>333</v>
+      <c r="L42" s="15" t="s">
+        <v>334</v>
       </c>
       <c r="M42" s="15">
         <v>1.06</v>
@@ -9429,10 +9421,9 @@
       <c r="N42" s="15">
         <v>0.94</v>
       </c>
-      <c r="O42" s="15"/>
-      <c r="P42" s="15"/>
-    </row>
-    <row r="43" spans="1:16">
+      <c r="Q42" s="20"/>
+    </row>
+    <row r="43" spans="1:17">
       <c r="A43" s="15" t="s">
         <v>311</v>
       </c>
@@ -9464,8 +9455,8 @@
       <c r="K43" s="15">
         <v>138</v>
       </c>
-      <c r="L43" t="s">
-        <v>333</v>
+      <c r="L43" s="15" t="s">
+        <v>334</v>
       </c>
       <c r="M43" s="15">
         <v>1.06</v>
@@ -9473,10 +9464,9 @@
       <c r="N43" s="15">
         <v>0.94</v>
       </c>
-      <c r="O43" s="15"/>
-      <c r="P43" s="15"/>
-    </row>
-    <row r="44" spans="1:16">
+      <c r="Q43" s="20"/>
+    </row>
+    <row r="44" spans="1:17">
       <c r="A44" s="15" t="s">
         <v>312</v>
       </c>
@@ -9508,8 +9498,8 @@
       <c r="K44" s="15">
         <v>138</v>
       </c>
-      <c r="L44" t="s">
-        <v>333</v>
+      <c r="L44" s="15" t="s">
+        <v>334</v>
       </c>
       <c r="M44" s="15">
         <v>1.06</v>
@@ -9517,10 +9507,9 @@
       <c r="N44" s="15">
         <v>0.94</v>
       </c>
-      <c r="O44" s="15"/>
-      <c r="P44" s="15"/>
-    </row>
-    <row r="45" spans="1:16">
+      <c r="Q44" s="20"/>
+    </row>
+    <row r="45" spans="1:17">
       <c r="A45" s="15" t="s">
         <v>313</v>
       </c>
@@ -9552,7 +9541,7 @@
       <c r="K45" s="15">
         <v>138</v>
       </c>
-      <c r="L45" t="s">
+      <c r="L45" s="15" t="s">
         <v>334</v>
       </c>
       <c r="M45" s="15">
@@ -9561,10 +9550,9 @@
       <c r="N45" s="15">
         <v>0.94</v>
       </c>
-      <c r="O45" s="15"/>
-      <c r="P45" s="15"/>
-    </row>
-    <row r="46" spans="1:16">
+      <c r="Q45" s="20"/>
+    </row>
+    <row r="46" spans="1:17">
       <c r="A46" s="15" t="s">
         <v>314</v>
       </c>
@@ -9596,7 +9584,7 @@
       <c r="K46" s="15">
         <v>138</v>
       </c>
-      <c r="L46" t="s">
+      <c r="L46" s="15" t="s">
         <v>334</v>
       </c>
       <c r="M46" s="15">
@@ -9605,10 +9593,9 @@
       <c r="N46" s="15">
         <v>0.94</v>
       </c>
-      <c r="O46" s="15"/>
-      <c r="P46" s="15"/>
-    </row>
-    <row r="47" spans="1:16">
+      <c r="Q46" s="20"/>
+    </row>
+    <row r="47" spans="1:17">
       <c r="A47" s="15" t="s">
         <v>315</v>
       </c>
@@ -9640,7 +9627,7 @@
       <c r="K47" s="15">
         <v>138</v>
       </c>
-      <c r="L47" t="s">
+      <c r="L47" s="15" t="s">
         <v>334</v>
       </c>
       <c r="M47" s="15">
@@ -9649,10 +9636,9 @@
       <c r="N47" s="15">
         <v>0.94</v>
       </c>
-      <c r="O47" s="15"/>
-      <c r="P47" s="15"/>
-    </row>
-    <row r="48" spans="1:16">
+      <c r="Q47" s="20"/>
+    </row>
+    <row r="48" spans="1:17">
       <c r="A48" s="15" t="s">
         <v>218</v>
       </c>
@@ -9684,7 +9670,7 @@
       <c r="K48" s="15">
         <v>138</v>
       </c>
-      <c r="L48" t="s">
+      <c r="L48" s="15" t="s">
         <v>334</v>
       </c>
       <c r="M48" s="15">
@@ -9693,10 +9679,9 @@
       <c r="N48" s="15">
         <v>0.94</v>
       </c>
-      <c r="O48" s="15"/>
-      <c r="P48" s="15"/>
-    </row>
-    <row r="49" spans="1:16">
+      <c r="Q48" s="20"/>
+    </row>
+    <row r="49" spans="1:17">
       <c r="A49" s="15" t="s">
         <v>316</v>
       </c>
@@ -9728,7 +9713,7 @@
       <c r="K49" s="15">
         <v>138</v>
       </c>
-      <c r="L49" t="s">
+      <c r="L49" s="15" t="s">
         <v>334</v>
       </c>
       <c r="M49" s="15">
@@ -9737,10 +9722,9 @@
       <c r="N49" s="15">
         <v>0.94</v>
       </c>
-      <c r="O49" s="15"/>
-      <c r="P49" s="15"/>
-    </row>
-    <row r="50" spans="1:16">
+      <c r="Q49" s="20"/>
+    </row>
+    <row r="50" spans="1:17">
       <c r="A50" s="15" t="s">
         <v>220</v>
       </c>
@@ -9772,7 +9756,7 @@
       <c r="K50" s="15">
         <v>138</v>
       </c>
-      <c r="L50" t="s">
+      <c r="L50" s="15" t="s">
         <v>334</v>
       </c>
       <c r="M50" s="15">
@@ -9781,10 +9765,9 @@
       <c r="N50" s="15">
         <v>0.94</v>
       </c>
-      <c r="O50" s="15"/>
-      <c r="P50" s="15"/>
-    </row>
-    <row r="51" spans="1:16">
+      <c r="Q50" s="20"/>
+    </row>
+    <row r="51" spans="1:17">
       <c r="A51" s="15" t="s">
         <v>317</v>
       </c>
@@ -9816,7 +9799,7 @@
       <c r="K51" s="15">
         <v>138</v>
       </c>
-      <c r="L51" t="s">
+      <c r="L51" s="15" t="s">
         <v>334</v>
       </c>
       <c r="M51" s="15">
@@ -9825,10 +9808,9 @@
       <c r="N51" s="15">
         <v>0.94</v>
       </c>
-      <c r="O51" s="15"/>
-      <c r="P51" s="15"/>
-    </row>
-    <row r="52" spans="1:16">
+      <c r="Q51" s="20"/>
+    </row>
+    <row r="52" spans="1:17">
       <c r="A52" s="15" t="s">
         <v>318</v>
       </c>
@@ -9860,7 +9842,7 @@
       <c r="K52" s="15">
         <v>138</v>
       </c>
-      <c r="L52" t="s">
+      <c r="L52" s="15" t="s">
         <v>334</v>
       </c>
       <c r="M52" s="15">
@@ -9869,10 +9851,9 @@
       <c r="N52" s="15">
         <v>0.94</v>
       </c>
-      <c r="O52" s="15"/>
-      <c r="P52" s="15"/>
-    </row>
-    <row r="53" spans="1:16">
+      <c r="Q52" s="20"/>
+    </row>
+    <row r="53" spans="1:17">
       <c r="A53" s="15" t="s">
         <v>319</v>
       </c>
@@ -9904,7 +9885,7 @@
       <c r="K53" s="15">
         <v>138</v>
       </c>
-      <c r="L53" t="s">
+      <c r="L53" s="15" t="s">
         <v>334</v>
       </c>
       <c r="M53" s="15">
@@ -9913,10 +9894,9 @@
       <c r="N53" s="15">
         <v>0.94</v>
       </c>
-      <c r="O53" s="15"/>
-      <c r="P53" s="15"/>
-    </row>
-    <row r="54" spans="1:16">
+      <c r="Q53" s="20"/>
+    </row>
+    <row r="54" spans="1:17">
       <c r="A54" s="15" t="s">
         <v>320</v>
       </c>
@@ -9948,7 +9928,7 @@
       <c r="K54" s="15">
         <v>138</v>
       </c>
-      <c r="L54" t="s">
+      <c r="L54" s="15" t="s">
         <v>334</v>
       </c>
       <c r="M54" s="15">
@@ -9957,10 +9937,9 @@
       <c r="N54" s="15">
         <v>0.94</v>
       </c>
-      <c r="O54" s="15"/>
-      <c r="P54" s="15"/>
-    </row>
-    <row r="55" spans="1:16">
+      <c r="Q54" s="20"/>
+    </row>
+    <row r="55" spans="1:17">
       <c r="A55" s="15" t="s">
         <v>321</v>
       </c>
@@ -9992,7 +9971,7 @@
       <c r="K55" s="15">
         <v>138</v>
       </c>
-      <c r="L55" t="s">
+      <c r="L55" s="15" t="s">
         <v>334</v>
       </c>
       <c r="M55" s="15">
@@ -10001,10 +9980,9 @@
       <c r="N55" s="15">
         <v>0.94</v>
       </c>
-      <c r="O55" s="15"/>
-      <c r="P55" s="15"/>
-    </row>
-    <row r="56" spans="1:16">
+      <c r="Q55" s="20"/>
+    </row>
+    <row r="56" spans="1:17">
       <c r="A56" s="15" t="s">
         <v>322</v>
       </c>
@@ -10036,7 +10014,7 @@
       <c r="K56" s="15">
         <v>138</v>
       </c>
-      <c r="L56" t="s">
+      <c r="L56" s="15" t="s">
         <v>334</v>
       </c>
       <c r="M56" s="15">
@@ -10045,10 +10023,9 @@
       <c r="N56" s="15">
         <v>0.94</v>
       </c>
-      <c r="O56" s="15"/>
-      <c r="P56" s="15"/>
-    </row>
-    <row r="57" spans="1:16">
+      <c r="Q56" s="20"/>
+    </row>
+    <row r="57" spans="1:17">
       <c r="A57" s="15" t="s">
         <v>323</v>
       </c>
@@ -10080,7 +10057,7 @@
       <c r="K57" s="15">
         <v>138</v>
       </c>
-      <c r="L57" t="s">
+      <c r="L57" s="15" t="s">
         <v>334</v>
       </c>
       <c r="M57" s="15">
@@ -10089,10 +10066,9 @@
       <c r="N57" s="15">
         <v>0.94</v>
       </c>
-      <c r="O57" s="15"/>
-      <c r="P57" s="15"/>
-    </row>
-    <row r="58" spans="1:16">
+      <c r="Q57" s="20"/>
+    </row>
+    <row r="58" spans="1:17">
       <c r="A58" s="15" t="s">
         <v>324</v>
       </c>
@@ -10124,7 +10100,7 @@
       <c r="K58" s="15">
         <v>138</v>
       </c>
-      <c r="L58" t="s">
+      <c r="L58" s="15" t="s">
         <v>334</v>
       </c>
       <c r="M58" s="15">
@@ -10133,10 +10109,9 @@
       <c r="N58" s="15">
         <v>0.94</v>
       </c>
-      <c r="O58" s="15"/>
-      <c r="P58" s="15"/>
-    </row>
-    <row r="59" spans="1:16">
+      <c r="Q58" s="20"/>
+    </row>
+    <row r="59" spans="1:17">
       <c r="A59" s="15" t="s">
         <v>325</v>
       </c>
@@ -10168,7 +10143,7 @@
       <c r="K59" s="15">
         <v>138</v>
       </c>
-      <c r="L59" t="s">
+      <c r="L59" s="15" t="s">
         <v>334</v>
       </c>
       <c r="M59" s="15">
@@ -10177,10 +10152,9 @@
       <c r="N59" s="15">
         <v>0.94</v>
       </c>
-      <c r="O59" s="15"/>
-      <c r="P59" s="15"/>
-    </row>
-    <row r="60" spans="1:16">
+      <c r="Q59" s="20"/>
+    </row>
+    <row r="60" spans="1:17">
       <c r="A60" s="15" t="s">
         <v>326</v>
       </c>
@@ -10212,7 +10186,7 @@
       <c r="K60" s="15">
         <v>138</v>
       </c>
-      <c r="L60" t="s">
+      <c r="L60" s="15" t="s">
         <v>334</v>
       </c>
       <c r="M60" s="15">
@@ -10221,10 +10195,9 @@
       <c r="N60" s="15">
         <v>0.94</v>
       </c>
-      <c r="O60" s="15"/>
-      <c r="P60" s="15"/>
-    </row>
-    <row r="61" spans="1:16">
+      <c r="Q60" s="20"/>
+    </row>
+    <row r="61" spans="1:17">
       <c r="A61" s="15" t="s">
         <v>327</v>
       </c>
@@ -10256,7 +10229,7 @@
       <c r="K61" s="15">
         <v>138</v>
       </c>
-      <c r="L61" t="s">
+      <c r="L61" s="15" t="s">
         <v>334</v>
       </c>
       <c r="M61" s="15">
@@ -10265,10 +10238,9 @@
       <c r="N61" s="15">
         <v>0.94</v>
       </c>
-      <c r="O61" s="15"/>
-      <c r="P61" s="15"/>
-    </row>
-    <row r="62" spans="1:16">
+      <c r="Q61" s="20"/>
+    </row>
+    <row r="62" spans="1:17">
       <c r="A62" s="15" t="s">
         <v>328</v>
       </c>
@@ -10300,7 +10272,7 @@
       <c r="K62" s="15">
         <v>138</v>
       </c>
-      <c r="L62" t="s">
+      <c r="L62" s="15" t="s">
         <v>334</v>
       </c>
       <c r="M62" s="15">
@@ -10309,10 +10281,9 @@
       <c r="N62" s="15">
         <v>0.94</v>
       </c>
-      <c r="O62" s="15"/>
-      <c r="P62" s="15"/>
-    </row>
-    <row r="63" spans="1:16">
+      <c r="Q62" s="20"/>
+    </row>
+    <row r="63" spans="1:17">
       <c r="A63" s="15" t="s">
         <v>213</v>
       </c>
@@ -10344,7 +10315,7 @@
       <c r="K63" s="15">
         <v>138</v>
       </c>
-      <c r="L63" t="s">
+      <c r="L63" s="15" t="s">
         <v>334</v>
       </c>
       <c r="M63" s="15">
@@ -10353,10 +10324,9 @@
       <c r="N63" s="15">
         <v>0.94</v>
       </c>
-      <c r="O63" s="15"/>
-      <c r="P63" s="15"/>
-    </row>
-    <row r="64" spans="1:16">
+      <c r="Q63" s="20"/>
+    </row>
+    <row r="64" spans="1:17">
       <c r="A64" s="15" t="s">
         <v>329</v>
       </c>
@@ -10388,7 +10358,7 @@
       <c r="K64" s="15">
         <v>345</v>
       </c>
-      <c r="L64" t="s">
+      <c r="L64" s="15" t="s">
         <v>334</v>
       </c>
       <c r="M64" s="15">
@@ -10397,10 +10367,9 @@
       <c r="N64" s="15">
         <v>0.94</v>
       </c>
-      <c r="O64" s="15"/>
-      <c r="P64" s="15"/>
-    </row>
-    <row r="65" spans="1:16">
+      <c r="Q64" s="20"/>
+    </row>
+    <row r="65" spans="1:17">
       <c r="A65" s="15" t="s">
         <v>330</v>
       </c>
@@ -10432,7 +10401,7 @@
       <c r="K65" s="15">
         <v>345</v>
       </c>
-      <c r="L65" t="s">
+      <c r="L65" s="15" t="s">
         <v>334</v>
       </c>
       <c r="M65" s="15">
@@ -10441,10 +10410,9 @@
       <c r="N65" s="15">
         <v>0.94</v>
       </c>
-      <c r="O65" s="15"/>
-      <c r="P65" s="15"/>
-    </row>
-    <row r="66" spans="1:16">
+      <c r="Q65" s="20"/>
+    </row>
+    <row r="66" spans="1:17">
       <c r="A66" s="15" t="s">
         <v>216</v>
       </c>
@@ -10476,7 +10444,7 @@
       <c r="K66" s="15">
         <v>345</v>
       </c>
-      <c r="L66" t="s">
+      <c r="L66" s="15" t="s">
         <v>334</v>
       </c>
       <c r="M66" s="15">
@@ -10485,10 +10453,9 @@
       <c r="N66" s="15">
         <v>0.94</v>
       </c>
-      <c r="O66" s="15"/>
-      <c r="P66" s="15"/>
-    </row>
-    <row r="67" spans="1:16">
+      <c r="Q66" s="20"/>
+    </row>
+    <row r="67" spans="1:17">
       <c r="A67" s="15" t="s">
         <v>214</v>
       </c>
@@ -10520,7 +10487,7 @@
       <c r="K67" s="15">
         <v>138</v>
       </c>
-      <c r="L67" t="s">
+      <c r="L67" s="15" t="s">
         <v>334</v>
       </c>
       <c r="M67" s="15">
@@ -10529,10 +10496,9 @@
       <c r="N67" s="15">
         <v>0.94</v>
       </c>
-      <c r="O67" s="15"/>
-      <c r="P67" s="15"/>
-    </row>
-    <row r="68" spans="1:16">
+      <c r="Q67" s="20"/>
+    </row>
+    <row r="68" spans="1:17">
       <c r="A68" s="15" t="s">
         <v>215</v>
       </c>
@@ -10564,7 +10530,7 @@
       <c r="K68" s="15">
         <v>138</v>
       </c>
-      <c r="L68" t="s">
+      <c r="L68" s="15" t="s">
         <v>334</v>
       </c>
       <c r="M68" s="15">
@@ -10573,10 +10539,9 @@
       <c r="N68" s="15">
         <v>0.94</v>
       </c>
-      <c r="O68" s="15"/>
-      <c r="P68" s="15"/>
-    </row>
-    <row r="69" spans="1:16">
+      <c r="Q68" s="20"/>
+    </row>
+    <row r="69" spans="1:17">
       <c r="A69" s="15" t="s">
         <v>217</v>
       </c>
@@ -10608,8 +10573,8 @@
       <c r="K69" s="15">
         <v>345</v>
       </c>
-      <c r="L69" t="s">
-        <v>334</v>
+      <c r="L69" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M69" s="15">
         <v>1.06</v>
@@ -10617,10 +10582,9 @@
       <c r="N69" s="15">
         <v>0.94</v>
       </c>
-      <c r="O69" s="15"/>
-      <c r="P69" s="15"/>
-    </row>
-    <row r="70" spans="1:16">
+      <c r="Q69" s="20"/>
+    </row>
+    <row r="70" spans="1:17">
       <c r="A70" s="15" t="s">
         <v>219</v>
       </c>
@@ -10652,8 +10616,8 @@
       <c r="K70" s="15">
         <v>138</v>
       </c>
-      <c r="L70" t="s">
-        <v>334</v>
+      <c r="L70" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M70" s="15">
         <v>1.06</v>
@@ -10661,10 +10625,9 @@
       <c r="N70" s="15">
         <v>0.94</v>
       </c>
-      <c r="O70" s="15"/>
-      <c r="P70" s="15"/>
-    </row>
-    <row r="71" spans="1:16">
+      <c r="Q70" s="20"/>
+    </row>
+    <row r="71" spans="1:17">
       <c r="A71" s="15" t="s">
         <v>221</v>
       </c>
@@ -10696,8 +10659,8 @@
       <c r="K71" s="15">
         <v>138</v>
       </c>
-      <c r="L71" t="s">
-        <v>334</v>
+      <c r="L71" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M71" s="15">
         <v>1.06</v>
@@ -10705,10 +10668,9 @@
       <c r="N71" s="15">
         <v>0.94</v>
       </c>
-      <c r="O71" s="15"/>
-      <c r="P71" s="15"/>
-    </row>
-    <row r="72" spans="1:16">
+      <c r="Q71" s="20"/>
+    </row>
+    <row r="72" spans="1:17">
       <c r="A72" s="15" t="s">
         <v>223</v>
       </c>
@@ -10740,8 +10702,8 @@
       <c r="K72" s="15">
         <v>138</v>
       </c>
-      <c r="L72" t="s">
-        <v>334</v>
+      <c r="L72" s="15" t="s">
+        <v>333</v>
       </c>
       <c r="M72" s="15">
         <v>1.06</v>
@@ -10749,10 +10711,9 @@
       <c r="N72" s="15">
         <v>0.94</v>
       </c>
-      <c r="O72" s="15"/>
-      <c r="P72" s="15"/>
-    </row>
-    <row r="73" spans="1:16">
+      <c r="Q72" s="20"/>
+    </row>
+    <row r="73" spans="1:17">
       <c r="A73" s="15" t="s">
         <v>224</v>
       </c>
@@ -10784,8 +10745,8 @@
       <c r="K73" s="15">
         <v>138</v>
       </c>
-      <c r="L73" t="s">
-        <v>334</v>
+      <c r="L73" s="15" t="s">
+        <v>333</v>
       </c>
       <c r="M73" s="15">
         <v>1.06</v>
@@ -10793,10 +10754,9 @@
       <c r="N73" s="15">
         <v>0.94</v>
       </c>
-      <c r="O73" s="15"/>
-      <c r="P73" s="15"/>
-    </row>
-    <row r="74" spans="1:16">
+      <c r="Q73" s="20"/>
+    </row>
+    <row r="74" spans="1:17">
       <c r="A74" s="15" t="s">
         <v>225</v>
       </c>
@@ -10828,8 +10788,8 @@
       <c r="K74" s="15">
         <v>138</v>
       </c>
-      <c r="L74" t="s">
-        <v>334</v>
+      <c r="L74" s="15" t="s">
+        <v>333</v>
       </c>
       <c r="M74" s="15">
         <v>1.06</v>
@@ -10837,10 +10797,9 @@
       <c r="N74" s="15">
         <v>0.94</v>
       </c>
-      <c r="O74" s="15"/>
-      <c r="P74" s="15"/>
-    </row>
-    <row r="75" spans="1:16">
+      <c r="Q74" s="20"/>
+    </row>
+    <row r="75" spans="1:17">
       <c r="A75" s="15" t="s">
         <v>226</v>
       </c>
@@ -10872,8 +10831,8 @@
       <c r="K75" s="15">
         <v>138</v>
       </c>
-      <c r="L75" t="s">
-        <v>334</v>
+      <c r="L75" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M75" s="15">
         <v>1.06</v>
@@ -10881,10 +10840,9 @@
       <c r="N75" s="15">
         <v>0.94</v>
       </c>
-      <c r="O75" s="15"/>
-      <c r="P75" s="15"/>
-    </row>
-    <row r="76" spans="1:16">
+      <c r="Q75" s="20"/>
+    </row>
+    <row r="76" spans="1:17">
       <c r="A76" s="15" t="s">
         <v>227</v>
       </c>
@@ -10916,8 +10874,8 @@
       <c r="K76" s="15">
         <v>138</v>
       </c>
-      <c r="L76" t="s">
-        <v>334</v>
+      <c r="L76" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M76" s="15">
         <v>1.06</v>
@@ -10925,10 +10883,9 @@
       <c r="N76" s="15">
         <v>0.94</v>
       </c>
-      <c r="O76" s="15"/>
-      <c r="P76" s="15"/>
-    </row>
-    <row r="77" spans="1:16">
+      <c r="Q76" s="20"/>
+    </row>
+    <row r="77" spans="1:17">
       <c r="A77" s="15" t="s">
         <v>228</v>
       </c>
@@ -10960,8 +10917,8 @@
       <c r="K77" s="15">
         <v>138</v>
       </c>
-      <c r="L77" t="s">
-        <v>334</v>
+      <c r="L77" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M77" s="15">
         <v>1.06</v>
@@ -10969,10 +10926,9 @@
       <c r="N77" s="15">
         <v>0.94</v>
       </c>
-      <c r="O77" s="15"/>
-      <c r="P77" s="15"/>
-    </row>
-    <row r="78" spans="1:16">
+      <c r="Q77" s="20"/>
+    </row>
+    <row r="78" spans="1:17">
       <c r="A78" s="15" t="s">
         <v>229</v>
       </c>
@@ -11004,8 +10960,8 @@
       <c r="K78" s="15">
         <v>138</v>
       </c>
-      <c r="L78" t="s">
-        <v>334</v>
+      <c r="L78" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M78" s="15">
         <v>1.06</v>
@@ -11013,10 +10969,9 @@
       <c r="N78" s="15">
         <v>0.94</v>
       </c>
-      <c r="O78" s="15"/>
-      <c r="P78" s="15"/>
-    </row>
-    <row r="79" spans="1:16">
+      <c r="Q78" s="20"/>
+    </row>
+    <row r="79" spans="1:17">
       <c r="A79" s="15" t="s">
         <v>230</v>
       </c>
@@ -11048,8 +11003,8 @@
       <c r="K79" s="15">
         <v>138</v>
       </c>
-      <c r="L79" t="s">
-        <v>334</v>
+      <c r="L79" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M79" s="15">
         <v>1.06</v>
@@ -11057,10 +11012,9 @@
       <c r="N79" s="15">
         <v>0.94</v>
       </c>
-      <c r="O79" s="15"/>
-      <c r="P79" s="15"/>
-    </row>
-    <row r="80" spans="1:16">
+      <c r="Q79" s="20"/>
+    </row>
+    <row r="80" spans="1:17">
       <c r="A80" s="15" t="s">
         <v>231</v>
       </c>
@@ -11092,8 +11046,8 @@
       <c r="K80" s="15">
         <v>138</v>
       </c>
-      <c r="L80" t="s">
-        <v>334</v>
+      <c r="L80" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M80" s="15">
         <v>1.06</v>
@@ -11101,10 +11055,9 @@
       <c r="N80" s="15">
         <v>0.94</v>
       </c>
-      <c r="O80" s="15"/>
-      <c r="P80" s="15"/>
-    </row>
-    <row r="81" spans="1:16">
+      <c r="Q80" s="20"/>
+    </row>
+    <row r="81" spans="1:17">
       <c r="A81" s="15" t="s">
         <v>232</v>
       </c>
@@ -11136,8 +11089,8 @@
       <c r="K81" s="15">
         <v>138</v>
       </c>
-      <c r="L81" t="s">
-        <v>334</v>
+      <c r="L81" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M81" s="15">
         <v>1.06</v>
@@ -11145,10 +11098,9 @@
       <c r="N81" s="15">
         <v>0.94</v>
       </c>
-      <c r="O81" s="15"/>
-      <c r="P81" s="15"/>
-    </row>
-    <row r="82" spans="1:16">
+      <c r="Q81" s="20"/>
+    </row>
+    <row r="82" spans="1:17">
       <c r="A82" s="15" t="s">
         <v>233</v>
       </c>
@@ -11180,8 +11132,8 @@
       <c r="K82" s="15">
         <v>345</v>
       </c>
-      <c r="L82" t="s">
-        <v>332</v>
+      <c r="L82" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M82" s="15">
         <v>1.06</v>
@@ -11189,10 +11141,9 @@
       <c r="N82" s="15">
         <v>0.94</v>
       </c>
-      <c r="O82" s="15"/>
-      <c r="P82" s="15"/>
-    </row>
-    <row r="83" spans="1:16">
+      <c r="Q82" s="20"/>
+    </row>
+    <row r="83" spans="1:17">
       <c r="A83" s="15" t="s">
         <v>234</v>
       </c>
@@ -11224,8 +11175,8 @@
       <c r="K83" s="15">
         <v>138</v>
       </c>
-      <c r="L83" t="s">
-        <v>332</v>
+      <c r="L83" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M83" s="15">
         <v>1.06</v>
@@ -11233,10 +11184,9 @@
       <c r="N83" s="15">
         <v>0.94</v>
       </c>
-      <c r="O83" s="15"/>
-      <c r="P83" s="15"/>
-    </row>
-    <row r="84" spans="1:16">
+      <c r="Q83" s="20"/>
+    </row>
+    <row r="84" spans="1:17">
       <c r="A84" s="15" t="s">
         <v>235</v>
       </c>
@@ -11268,8 +11218,8 @@
       <c r="K84" s="15">
         <v>138</v>
       </c>
-      <c r="L84" t="s">
-        <v>332</v>
+      <c r="L84" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M84" s="15">
         <v>1.06</v>
@@ -11277,10 +11227,9 @@
       <c r="N84" s="15">
         <v>0.94</v>
       </c>
-      <c r="O84" s="15"/>
-      <c r="P84" s="15"/>
-    </row>
-    <row r="85" spans="1:16">
+      <c r="Q84" s="20"/>
+    </row>
+    <row r="85" spans="1:17">
       <c r="A85" s="15" t="s">
         <v>236</v>
       </c>
@@ -11312,8 +11261,8 @@
       <c r="K85" s="15">
         <v>138</v>
       </c>
-      <c r="L85" t="s">
-        <v>332</v>
+      <c r="L85" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M85" s="15">
         <v>1.06</v>
@@ -11321,10 +11270,9 @@
       <c r="N85" s="15">
         <v>0.94</v>
       </c>
-      <c r="O85" s="15"/>
-      <c r="P85" s="15"/>
-    </row>
-    <row r="86" spans="1:16">
+      <c r="Q85" s="20"/>
+    </row>
+    <row r="86" spans="1:17">
       <c r="A86" s="15" t="s">
         <v>237</v>
       </c>
@@ -11356,8 +11304,8 @@
       <c r="K86" s="15">
         <v>138</v>
       </c>
-      <c r="L86" t="s">
-        <v>332</v>
+      <c r="L86" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M86" s="15">
         <v>1.06</v>
@@ -11365,10 +11313,9 @@
       <c r="N86" s="15">
         <v>0.94</v>
       </c>
-      <c r="O86" s="15"/>
-      <c r="P86" s="15"/>
-    </row>
-    <row r="87" spans="1:16">
+      <c r="Q86" s="20"/>
+    </row>
+    <row r="87" spans="1:17">
       <c r="A87" s="15" t="s">
         <v>238</v>
       </c>
@@ -11400,8 +11347,8 @@
       <c r="K87" s="15">
         <v>138</v>
       </c>
-      <c r="L87" t="s">
-        <v>332</v>
+      <c r="L87" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M87" s="15">
         <v>1.06</v>
@@ -11409,10 +11356,9 @@
       <c r="N87" s="15">
         <v>0.94</v>
       </c>
-      <c r="O87" s="15"/>
-      <c r="P87" s="15"/>
-    </row>
-    <row r="88" spans="1:16">
+      <c r="Q87" s="20"/>
+    </row>
+    <row r="88" spans="1:17">
       <c r="A88" s="15" t="s">
         <v>239</v>
       </c>
@@ -11444,8 +11390,8 @@
       <c r="K88" s="15">
         <v>161</v>
       </c>
-      <c r="L88" t="s">
-        <v>332</v>
+      <c r="L88" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M88" s="15">
         <v>1.06</v>
@@ -11453,10 +11399,9 @@
       <c r="N88" s="15">
         <v>0.94</v>
       </c>
-      <c r="O88" s="15"/>
-      <c r="P88" s="15"/>
-    </row>
-    <row r="89" spans="1:16">
+      <c r="Q88" s="20"/>
+    </row>
+    <row r="89" spans="1:17">
       <c r="A89" s="15" t="s">
         <v>240</v>
       </c>
@@ -11488,8 +11433,8 @@
       <c r="K89" s="15">
         <v>138</v>
       </c>
-      <c r="L89" t="s">
-        <v>332</v>
+      <c r="L89" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M89" s="15">
         <v>1.06</v>
@@ -11497,10 +11442,9 @@
       <c r="N89" s="15">
         <v>0.94</v>
       </c>
-      <c r="O89" s="15"/>
-      <c r="P89" s="15"/>
-    </row>
-    <row r="90" spans="1:16">
+      <c r="Q89" s="20"/>
+    </row>
+    <row r="90" spans="1:17">
       <c r="A90" s="15" t="s">
         <v>241</v>
       </c>
@@ -11532,8 +11476,8 @@
       <c r="K90" s="15">
         <v>138</v>
       </c>
-      <c r="L90" t="s">
-        <v>332</v>
+      <c r="L90" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M90" s="15">
         <v>1.06</v>
@@ -11541,10 +11485,9 @@
       <c r="N90" s="15">
         <v>0.94</v>
       </c>
-      <c r="O90" s="15"/>
-      <c r="P90" s="15"/>
-    </row>
-    <row r="91" spans="1:16">
+      <c r="Q90" s="20"/>
+    </row>
+    <row r="91" spans="1:17">
       <c r="A91" s="15" t="s">
         <v>242</v>
       </c>
@@ -11576,8 +11519,8 @@
       <c r="K91" s="15">
         <v>138</v>
       </c>
-      <c r="L91" t="s">
-        <v>332</v>
+      <c r="L91" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M91" s="15">
         <v>1.06</v>
@@ -11585,10 +11528,9 @@
       <c r="N91" s="15">
         <v>0.94</v>
       </c>
-      <c r="O91" s="15"/>
-      <c r="P91" s="15"/>
-    </row>
-    <row r="92" spans="1:16">
+      <c r="Q91" s="20"/>
+    </row>
+    <row r="92" spans="1:17">
       <c r="A92" s="15" t="s">
         <v>243</v>
       </c>
@@ -11620,8 +11562,8 @@
       <c r="K92" s="15">
         <v>138</v>
       </c>
-      <c r="L92" t="s">
-        <v>333</v>
+      <c r="L92" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M92" s="15">
         <v>1.06</v>
@@ -11629,10 +11571,9 @@
       <c r="N92" s="15">
         <v>0.94</v>
       </c>
-      <c r="O92" s="15"/>
-      <c r="P92" s="15"/>
-    </row>
-    <row r="93" spans="1:16">
+      <c r="Q92" s="20"/>
+    </row>
+    <row r="93" spans="1:17">
       <c r="A93" s="15" t="s">
         <v>244</v>
       </c>
@@ -11664,8 +11605,8 @@
       <c r="K93" s="15">
         <v>138</v>
       </c>
-      <c r="L93" t="s">
-        <v>333</v>
+      <c r="L93" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M93" s="15">
         <v>1.06</v>
@@ -11673,10 +11614,9 @@
       <c r="N93" s="15">
         <v>0.94</v>
       </c>
-      <c r="O93" s="15"/>
-      <c r="P93" s="15"/>
-    </row>
-    <row r="94" spans="1:16">
+      <c r="Q93" s="20"/>
+    </row>
+    <row r="94" spans="1:17">
       <c r="A94" s="15" t="s">
         <v>245</v>
       </c>
@@ -11708,8 +11648,8 @@
       <c r="K94" s="15">
         <v>138</v>
       </c>
-      <c r="L94" t="s">
-        <v>334</v>
+      <c r="L94" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M94" s="15">
         <v>1.06</v>
@@ -11717,10 +11657,9 @@
       <c r="N94" s="15">
         <v>0.94</v>
       </c>
-      <c r="O94" s="15"/>
-      <c r="P94" s="15"/>
-    </row>
-    <row r="95" spans="1:16">
+      <c r="Q94" s="20"/>
+    </row>
+    <row r="95" spans="1:17">
       <c r="A95" s="15" t="s">
         <v>246</v>
       </c>
@@ -11752,8 +11691,8 @@
       <c r="K95" s="15">
         <v>138</v>
       </c>
-      <c r="L95" t="s">
-        <v>334</v>
+      <c r="L95" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M95" s="15">
         <v>1.06</v>
@@ -11761,10 +11700,9 @@
       <c r="N95" s="15">
         <v>0.94</v>
       </c>
-      <c r="O95" s="15"/>
-      <c r="P95" s="15"/>
-    </row>
-    <row r="96" spans="1:16">
+      <c r="Q95" s="20"/>
+    </row>
+    <row r="96" spans="1:17">
       <c r="A96" s="15" t="s">
         <v>247</v>
       </c>
@@ -11796,8 +11734,8 @@
       <c r="K96" s="15">
         <v>138</v>
       </c>
-      <c r="L96" t="s">
-        <v>334</v>
+      <c r="L96" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M96" s="15">
         <v>1.06</v>
@@ -11805,10 +11743,9 @@
       <c r="N96" s="15">
         <v>0.94</v>
       </c>
-      <c r="O96" s="15"/>
-      <c r="P96" s="15"/>
-    </row>
-    <row r="97" spans="1:16">
+      <c r="Q96" s="20"/>
+    </row>
+    <row r="97" spans="1:17">
       <c r="A97" s="15" t="s">
         <v>248</v>
       </c>
@@ -11840,8 +11777,8 @@
       <c r="K97" s="15">
         <v>138</v>
       </c>
-      <c r="L97" t="s">
-        <v>334</v>
+      <c r="L97" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M97" s="15">
         <v>1.06</v>
@@ -11849,10 +11786,9 @@
       <c r="N97" s="15">
         <v>0.94</v>
       </c>
-      <c r="O97" s="15"/>
-      <c r="P97" s="15"/>
-    </row>
-    <row r="98" spans="1:16">
+      <c r="Q97" s="20"/>
+    </row>
+    <row r="98" spans="1:17">
       <c r="A98" s="15" t="s">
         <v>249</v>
       </c>
@@ -11884,8 +11820,8 @@
       <c r="K98" s="15">
         <v>138</v>
       </c>
-      <c r="L98" t="s">
-        <v>334</v>
+      <c r="L98" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M98" s="15">
         <v>1.06</v>
@@ -11893,10 +11829,9 @@
       <c r="N98" s="15">
         <v>0.94</v>
       </c>
-      <c r="O98" s="15"/>
-      <c r="P98" s="15"/>
-    </row>
-    <row r="99" spans="1:16">
+      <c r="Q98" s="20"/>
+    </row>
+    <row r="99" spans="1:17">
       <c r="A99" s="15" t="s">
         <v>250</v>
       </c>
@@ -11928,8 +11863,8 @@
       <c r="K99" s="15">
         <v>138</v>
       </c>
-      <c r="L99" t="s">
-        <v>334</v>
+      <c r="L99" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M99" s="15">
         <v>1.06</v>
@@ -11937,10 +11872,9 @@
       <c r="N99" s="15">
         <v>0.94</v>
       </c>
-      <c r="O99" s="15"/>
-      <c r="P99" s="15"/>
-    </row>
-    <row r="100" spans="1:16">
+      <c r="Q99" s="20"/>
+    </row>
+    <row r="100" spans="1:17">
       <c r="A100" s="15" t="s">
         <v>251</v>
       </c>
@@ -11972,8 +11906,8 @@
       <c r="K100" s="15">
         <v>138</v>
       </c>
-      <c r="L100" t="s">
-        <v>334</v>
+      <c r="L100" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M100" s="15">
         <v>1.06</v>
@@ -11981,10 +11915,9 @@
       <c r="N100" s="15">
         <v>0.94</v>
       </c>
-      <c r="O100" s="15"/>
-      <c r="P100" s="15"/>
-    </row>
-    <row r="101" spans="1:16">
+      <c r="Q100" s="20"/>
+    </row>
+    <row r="101" spans="1:17">
       <c r="A101" s="15" t="s">
         <v>252</v>
       </c>
@@ -12016,8 +11949,8 @@
       <c r="K101" s="15">
         <v>138</v>
       </c>
-      <c r="L101" t="s">
-        <v>334</v>
+      <c r="L101" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M101" s="15">
         <v>1.06</v>
@@ -12025,10 +11958,9 @@
       <c r="N101" s="15">
         <v>0.94</v>
       </c>
-      <c r="O101" s="15"/>
-      <c r="P101" s="15"/>
-    </row>
-    <row r="102" spans="1:16">
+      <c r="Q101" s="20"/>
+    </row>
+    <row r="102" spans="1:17">
       <c r="A102" s="15" t="s">
         <v>253</v>
       </c>
@@ -12060,8 +11992,8 @@
       <c r="K102" s="15">
         <v>138</v>
       </c>
-      <c r="L102" t="s">
-        <v>334</v>
+      <c r="L102" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M102" s="15">
         <v>1.06</v>
@@ -12069,10 +12001,9 @@
       <c r="N102" s="15">
         <v>0.94</v>
       </c>
-      <c r="O102" s="15"/>
-      <c r="P102" s="15"/>
-    </row>
-    <row r="103" spans="1:16">
+      <c r="Q102" s="20"/>
+    </row>
+    <row r="103" spans="1:17">
       <c r="A103" s="15" t="s">
         <v>254</v>
       </c>
@@ -12104,8 +12035,8 @@
       <c r="K103" s="15">
         <v>138</v>
       </c>
-      <c r="L103" t="s">
-        <v>334</v>
+      <c r="L103" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M103" s="15">
         <v>1.06</v>
@@ -12113,10 +12044,9 @@
       <c r="N103" s="15">
         <v>0.94</v>
       </c>
-      <c r="O103" s="15"/>
-      <c r="P103" s="15"/>
-    </row>
-    <row r="104" spans="1:16">
+      <c r="Q103" s="20"/>
+    </row>
+    <row r="104" spans="1:17">
       <c r="A104" s="15" t="s">
         <v>255</v>
       </c>
@@ -12148,8 +12078,8 @@
       <c r="K104" s="15">
         <v>138</v>
       </c>
-      <c r="L104" t="s">
-        <v>334</v>
+      <c r="L104" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M104" s="15">
         <v>1.06</v>
@@ -12157,10 +12087,9 @@
       <c r="N104" s="15">
         <v>0.94</v>
       </c>
-      <c r="O104" s="15"/>
-      <c r="P104" s="15"/>
-    </row>
-    <row r="105" spans="1:16">
+      <c r="Q104" s="20"/>
+    </row>
+    <row r="105" spans="1:17">
       <c r="A105" s="15" t="s">
         <v>256</v>
       </c>
@@ -12192,8 +12121,8 @@
       <c r="K105" s="15">
         <v>138</v>
       </c>
-      <c r="L105" t="s">
-        <v>334</v>
+      <c r="L105" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M105" s="15">
         <v>1.06</v>
@@ -12201,10 +12130,9 @@
       <c r="N105" s="15">
         <v>0.94</v>
       </c>
-      <c r="O105" s="15"/>
-      <c r="P105" s="15"/>
-    </row>
-    <row r="106" spans="1:16">
+      <c r="Q105" s="20"/>
+    </row>
+    <row r="106" spans="1:17">
       <c r="A106" s="15" t="s">
         <v>257</v>
       </c>
@@ -12236,8 +12164,8 @@
       <c r="K106" s="15">
         <v>138</v>
       </c>
-      <c r="L106" t="s">
-        <v>334</v>
+      <c r="L106" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M106" s="15">
         <v>1.06</v>
@@ -12245,10 +12173,9 @@
       <c r="N106" s="15">
         <v>0.94</v>
       </c>
-      <c r="O106" s="15"/>
-      <c r="P106" s="15"/>
-    </row>
-    <row r="107" spans="1:16">
+      <c r="Q106" s="20"/>
+    </row>
+    <row r="107" spans="1:17">
       <c r="A107" s="15" t="s">
         <v>258</v>
       </c>
@@ -12280,8 +12207,8 @@
       <c r="K107" s="15">
         <v>138</v>
       </c>
-      <c r="L107" t="s">
-        <v>334</v>
+      <c r="L107" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M107" s="15">
         <v>1.06</v>
@@ -12289,10 +12216,9 @@
       <c r="N107" s="15">
         <v>0.94</v>
       </c>
-      <c r="O107" s="15"/>
-      <c r="P107" s="15"/>
-    </row>
-    <row r="108" spans="1:16">
+      <c r="Q107" s="20"/>
+    </row>
+    <row r="108" spans="1:17">
       <c r="A108" s="15" t="s">
         <v>259</v>
       </c>
@@ -12324,8 +12250,8 @@
       <c r="K108" s="15">
         <v>138</v>
       </c>
-      <c r="L108" t="s">
-        <v>334</v>
+      <c r="L108" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M108" s="15">
         <v>1.06</v>
@@ -12333,10 +12259,9 @@
       <c r="N108" s="15">
         <v>0.94</v>
       </c>
-      <c r="O108" s="15"/>
-      <c r="P108" s="15"/>
-    </row>
-    <row r="109" spans="1:16">
+      <c r="Q108" s="20"/>
+    </row>
+    <row r="109" spans="1:17">
       <c r="A109" s="15" t="s">
         <v>260</v>
       </c>
@@ -12368,8 +12293,8 @@
       <c r="K109" s="15">
         <v>138</v>
       </c>
-      <c r="L109" t="s">
-        <v>334</v>
+      <c r="L109" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M109" s="15">
         <v>1.06</v>
@@ -12377,10 +12302,9 @@
       <c r="N109" s="15">
         <v>0.94</v>
       </c>
-      <c r="O109" s="15"/>
-      <c r="P109" s="15"/>
-    </row>
-    <row r="110" spans="1:16">
+      <c r="Q109" s="20"/>
+    </row>
+    <row r="110" spans="1:17">
       <c r="A110" s="15" t="s">
         <v>261</v>
       </c>
@@ -12412,8 +12336,8 @@
       <c r="K110" s="15">
         <v>138</v>
       </c>
-      <c r="L110" t="s">
-        <v>334</v>
+      <c r="L110" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M110" s="15">
         <v>1.06</v>
@@ -12421,10 +12345,9 @@
       <c r="N110" s="15">
         <v>0.94</v>
       </c>
-      <c r="O110" s="15"/>
-      <c r="P110" s="15"/>
-    </row>
-    <row r="111" spans="1:16">
+      <c r="Q110" s="20"/>
+    </row>
+    <row r="111" spans="1:17">
       <c r="A111" s="15" t="s">
         <v>262</v>
       </c>
@@ -12456,8 +12379,8 @@
       <c r="K111" s="15">
         <v>138</v>
       </c>
-      <c r="L111" t="s">
-        <v>334</v>
+      <c r="L111" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M111" s="15">
         <v>1.06</v>
@@ -12465,10 +12388,9 @@
       <c r="N111" s="15">
         <v>0.94</v>
       </c>
-      <c r="O111" s="15"/>
-      <c r="P111" s="15"/>
-    </row>
-    <row r="112" spans="1:16">
+      <c r="Q111" s="20"/>
+    </row>
+    <row r="112" spans="1:17">
       <c r="A112" s="15" t="s">
         <v>263</v>
       </c>
@@ -12500,8 +12422,8 @@
       <c r="K112" s="15">
         <v>138</v>
       </c>
-      <c r="L112" t="s">
-        <v>334</v>
+      <c r="L112" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M112" s="15">
         <v>1.06</v>
@@ -12509,10 +12431,9 @@
       <c r="N112" s="15">
         <v>0.94</v>
       </c>
-      <c r="O112" s="15"/>
-      <c r="P112" s="15"/>
-    </row>
-    <row r="113" spans="1:16">
+      <c r="Q112" s="20"/>
+    </row>
+    <row r="113" spans="1:17">
       <c r="A113" s="15" t="s">
         <v>264</v>
       </c>
@@ -12544,8 +12465,8 @@
       <c r="K113" s="15">
         <v>138</v>
       </c>
-      <c r="L113" t="s">
-        <v>334</v>
+      <c r="L113" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M113" s="15">
         <v>1.06</v>
@@ -12553,10 +12474,9 @@
       <c r="N113" s="15">
         <v>0.94</v>
       </c>
-      <c r="O113" s="15"/>
-      <c r="P113" s="15"/>
-    </row>
-    <row r="114" spans="1:16">
+      <c r="Q113" s="20"/>
+    </row>
+    <row r="114" spans="1:17">
       <c r="A114" s="15" t="s">
         <v>266</v>
       </c>
@@ -12588,8 +12508,8 @@
       <c r="K114" s="15">
         <v>138</v>
       </c>
-      <c r="L114" t="s">
-        <v>332</v>
+      <c r="L114" s="15" t="s">
+        <v>333</v>
       </c>
       <c r="M114" s="15">
         <v>1.06</v>
@@ -12597,10 +12517,9 @@
       <c r="N114" s="15">
         <v>0.94</v>
       </c>
-      <c r="O114" s="15"/>
-      <c r="P114" s="15"/>
-    </row>
-    <row r="115" spans="1:16">
+      <c r="Q114" s="20"/>
+    </row>
+    <row r="115" spans="1:17">
       <c r="A115" s="15" t="s">
         <v>268</v>
       </c>
@@ -12632,8 +12551,8 @@
       <c r="K115" s="15">
         <v>138</v>
       </c>
-      <c r="L115" t="s">
-        <v>332</v>
+      <c r="L115" s="15" t="s">
+        <v>333</v>
       </c>
       <c r="M115" s="15">
         <v>1.06</v>
@@ -12641,10 +12560,9 @@
       <c r="N115" s="15">
         <v>0.94</v>
       </c>
-      <c r="O115" s="15"/>
-      <c r="P115" s="15"/>
-    </row>
-    <row r="116" spans="1:16">
+      <c r="Q115" s="20"/>
+    </row>
+    <row r="116" spans="1:17">
       <c r="A116" s="15" t="s">
         <v>270</v>
       </c>
@@ -12676,8 +12594,8 @@
       <c r="K116" s="15">
         <v>138</v>
       </c>
-      <c r="L116" t="s">
-        <v>332</v>
+      <c r="L116" s="15" t="s">
+        <v>333</v>
       </c>
       <c r="M116" s="15">
         <v>1.06</v>
@@ -12685,10 +12603,9 @@
       <c r="N116" s="15">
         <v>0.94</v>
       </c>
-      <c r="O116" s="15"/>
-      <c r="P116" s="15"/>
-    </row>
-    <row r="117" spans="1:16">
+      <c r="Q116" s="20"/>
+    </row>
+    <row r="117" spans="1:17">
       <c r="A117" s="15" t="s">
         <v>271</v>
       </c>
@@ -12720,8 +12637,8 @@
       <c r="K117" s="15">
         <v>138</v>
       </c>
-      <c r="L117" t="s">
-        <v>332</v>
+      <c r="L117" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M117" s="15">
         <v>1.06</v>
@@ -12729,10 +12646,9 @@
       <c r="N117" s="15">
         <v>0.94</v>
       </c>
-      <c r="O117" s="15"/>
-      <c r="P117" s="15"/>
-    </row>
-    <row r="118" spans="1:16">
+      <c r="Q117" s="20"/>
+    </row>
+    <row r="118" spans="1:17">
       <c r="A118" s="15" t="s">
         <v>273</v>
       </c>
@@ -12764,8 +12680,8 @@
       <c r="K118" s="15">
         <v>138</v>
       </c>
-      <c r="L118" t="s">
-        <v>333</v>
+      <c r="L118" s="15" t="s">
+        <v>332</v>
       </c>
       <c r="M118" s="15">
         <v>1.06</v>
@@ -12773,10 +12689,9 @@
       <c r="N118" s="15">
         <v>0.94</v>
       </c>
-      <c r="O118" s="15"/>
-      <c r="P118" s="15"/>
-    </row>
-    <row r="119" spans="1:16">
+      <c r="Q118" s="20"/>
+    </row>
+    <row r="119" spans="1:17">
       <c r="A119" s="15" t="s">
         <v>274</v>
       </c>
@@ -12808,8 +12723,8 @@
       <c r="K119" s="15">
         <v>138</v>
       </c>
-      <c r="L119" t="s">
-        <v>332</v>
+      <c r="L119" s="15" t="s">
+        <v>337</v>
       </c>
       <c r="M119" s="15">
         <v>1.06</v>
@@ -12817,11 +12732,70 @@
       <c r="N119" s="15">
         <v>0.94</v>
       </c>
-      <c r="O119" s="15"/>
-      <c r="P119" s="15"/>
+      <c r="Q119" s="20"/>
+    </row>
+    <row r="130" spans="17:17" ht="23.25">
+      <c r="Q130" s="21"/>
+    </row>
+    <row r="131" spans="17:17">
+      <c r="Q131" s="22"/>
+    </row>
+    <row r="132" spans="17:17">
+      <c r="Q132" s="22"/>
+    </row>
+    <row r="133" spans="17:17">
+      <c r="Q133" s="22"/>
+    </row>
+    <row r="134" spans="17:17">
+      <c r="Q134" s="22"/>
+    </row>
+    <row r="135" spans="17:17">
+      <c r="Q135" s="22"/>
+    </row>
+    <row r="136" spans="17:17">
+      <c r="Q136" s="22"/>
+    </row>
+    <row r="137" spans="17:17">
+      <c r="Q137" s="22"/>
+    </row>
+    <row r="138" spans="17:17">
+      <c r="Q138" s="22"/>
+    </row>
+    <row r="139" spans="17:17">
+      <c r="Q139" s="22"/>
+    </row>
+    <row r="140" spans="17:17">
+      <c r="Q140" s="22"/>
+    </row>
+    <row r="143" spans="17:17">
+      <c r="Q143" s="22"/>
+    </row>
+    <row r="144" spans="17:17">
+      <c r="Q144" s="22"/>
+    </row>
+    <row r="145" spans="17:17">
+      <c r="Q145" s="22"/>
+    </row>
+    <row r="146" spans="17:17">
+      <c r="Q146" s="22"/>
+    </row>
+    <row r="147" spans="17:17">
+      <c r="Q147" s="22"/>
+    </row>
+    <row r="148" spans="17:17">
+      <c r="Q148" s="22"/>
+    </row>
+    <row r="149" spans="17:17">
+      <c r="Q149" s="22"/>
+    </row>
+    <row r="150" spans="17:17">
+      <c r="Q150" s="22"/>
+    </row>
+    <row r="152" spans="17:17">
+      <c r="Q152" s="23"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="6" type="noConversion"/>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>